<commit_message>
Budget: fee covers diving, insurance and hotel only; George shares a room; prompt and tracker updated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="169">
   <si>
     <t xml:space="preserve">Cozumel group budget — inputs (blue cells are editable)</t>
   </si>
@@ -190,63 +190,54 @@
     <t xml:space="preserve">DAN membership + Preferred plan, bought for each person</t>
   </si>
   <si>
-    <t xml:space="preserve">Airport shuttle both ways</t>
+    <t xml:space="preserve">Leader costs carried by the group (George shares a room like everyone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George's flight allowance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">policy; PHL–CZM band 568–800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George's half of a shared room, 6 nights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">formula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Odd-headcount room risk (one person alone at the group's cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">formula: half a room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George's DAN cover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Own spending guidance, not in the fee (no flights)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunches, dinners and drinks per day (breakfast included)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INFERRED for an MBA crowd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days on the island</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tips for boat crew and hotel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INFERRED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airport transfers both ways</t>
   </si>
   <si>
     <t xml:space="preserve">ADVERTISED shared van 15 each way</t>
   </si>
   <si>
-    <t xml:space="preserve">Two group dinners (welcome, certification or farewell)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INFERRED 35 each</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Welcome drinks and briefing room</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INFERRED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leader costs carried by the group (George)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George's flight allowance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">policy; PHL–CZM band 568–800</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George's single room, 6 nights</t>
-  </si>
-  <si>
-    <t xml:space="preserve">formula: full room at the contracted rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Odd-headcount room risk (one single at the group's cost)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">formula: half a room</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George's DAN cover</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Own spending guidance, not in the fee (no flights)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lunches and dinners not covered, per day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INFERRED for an MBA crowd; breakfast included, two dinners included</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Days on the island</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tips for boat crew and hotel</t>
-  </si>
-  <si>
     <t xml:space="preserve">PADI AOW eLearning (add-on for AOW takers)</t>
   </si>
   <si>
@@ -280,10 +271,7 @@
     <t xml:space="preserve">Hotel Plaza, 6 nights with breakfast, 2 sharing</t>
   </si>
   <si>
-    <t xml:space="preserve">Airport shuttle, group dinners, welcome drinks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leader's costs shared (George's flight, room, DAN, odd-room risk)</t>
+    <t xml:space="preserve">Leader's costs shared (George's flight, half-room, DAN, odd-room risk)</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal</t>
@@ -310,9 +298,6 @@
     <t xml:space="preserve">Nitrox: course free with eLearning; 10 fills</t>
   </si>
   <si>
-    <t xml:space="preserve">Single room (whole room to yourself)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Afternoon two-tank dive, each, incl. park fee</t>
   </si>
   <si>
@@ -325,7 +310,7 @@
     <t xml:space="preserve">Trip fee</t>
   </si>
   <si>
-    <t xml:space="preserve">Own spending: lunches, dinners not covered, drinks, tips</t>
+    <t xml:space="preserve">Own spending: meals, drinks, tips, airport transfers</t>
   </si>
   <si>
     <t xml:space="preserve">Guidance budget, own gear</t>
@@ -337,7 +322,7 @@
     <t xml:space="preserve">Guidance budget, certified taking AOW and nitrox</t>
   </si>
   <si>
-    <t xml:space="preserve">The fee covers everything except the flight. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
+    <t xml:space="preserve">The fee covers diving, insurance and the hotel; everything else is the person's own. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
   </si>
   <si>
     <t xml:space="preserve">Group budget at four sizes (half students; George leads and does not pay)</t>
@@ -367,7 +352,7 @@
     <t xml:space="preserve">Paying certified divers</t>
   </si>
   <si>
-    <t xml:space="preserve">Rooms for participants (2 sharing; odd person alone at the group's cost)</t>
+    <t xml:space="preserve">Rooms, everyone 2 sharing including George (odd person alone at the group's cost)</t>
   </si>
   <si>
     <t xml:space="preserve">Revenue</t>
@@ -415,10 +400,7 @@
     <t xml:space="preserve">DAN cover for everyone including George</t>
   </si>
   <si>
-    <t xml:space="preserve">Hotel Plaza block: participant rooms plus George's single</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shuttle, two group dinners, welcome drinks, everyone</t>
+    <t xml:space="preserve">Hotel Plaza block, all rooms</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL COSTS</t>
@@ -460,7 +442,7 @@
     <t xml:space="preserve">Blue Note balance Fri 13 Nov + hotel balance + eLearning + DAN</t>
   </si>
   <si>
-    <t xml:space="preserve">Cash float to carry to the island (park fees, dinners, shuttle)</t>
+    <t xml:space="preserve">Cash float to carry to the island (park fees)</t>
   </si>
   <si>
     <t xml:space="preserve">Notes: revenue is the fixed fee from the Fee sheet, so the surplus grows with headcount (the leader share is over-recovered) and shrinks below the pricing basis; the contingency keeps it positive down to the minimum. Spare comps reduce the invoice for the group; the commission goes to George.</t>
@@ -529,7 +511,7 @@
     <t xml:space="preserve">Sun 13 Dec</t>
   </si>
   <si>
-    <t xml:space="preserve">Arrival; park fees and dinners paid from the club float</t>
+    <t xml:space="preserve">Arrival; park fees paid from the club float; meals, drinks, tips and transfers are each person's own</t>
   </si>
   <si>
     <t xml:space="preserve">after the trip</t>
@@ -547,7 +529,7 @@
     <t xml:space="preserve">Money handling</t>
   </si>
   <si>
-    <t xml:space="preserve">All payments through CampusGroups or Blue Note's own link, never personal Venmo or Zelle. The sign-up page states that the leader's diving is comped by the shop, his flight and room are carried by the group, and the shop's commission goes to him.</t>
+    <t xml:space="preserve">All payments through CampusGroups or Blue Note's own link, never personal Venmo or Zelle. The sign-up page states that the leader's diving is comped by the shop, his flight and half-room are carried by the group, and the shop's commission goes to him.</t>
   </si>
 </sst>
 </file>
@@ -959,7 +941,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72"/>
@@ -1356,173 +1338,145 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>56</v>
-      </c>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B32" s="7" t="n">
-        <v>70</v>
+        <v>700</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B33" s="7" t="n">
-        <v>10</v>
+        <f aca="false">(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)/2</f>
+        <v>246</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="B34" s="7" t="n">
+        <f aca="false">Inputs!$B$33</f>
+        <v>246</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B35" s="7" t="n">
-        <v>700</v>
+        <v>119</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D35" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B36" s="7" t="n">
-        <f aca="false">Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26</f>
-        <v>492</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>65</v>
-      </c>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B37" s="7" t="n">
-        <f aca="false">Inputs!$B$36/2</f>
-        <v>246</v>
+        <v>45</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D38" s="2"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B38" s="7" t="n">
-        <v>119</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="B40" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="B41" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D41" s="2"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B42" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B43" s="7" t="n">
-        <v>220</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1541,7 +1495,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -1550,7 +1504,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1558,15 +1512,15 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">Inputs!$B$9+Inputs!$B$10</f>
@@ -1579,7 +1533,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">Inputs!$B$13*Inputs!$B$15</f>
@@ -1592,19 +1546,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">Inputs!$B$29</f>
         <v>195</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">Inputs!$B$30</f>
@@ -1617,7 +1571,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">((Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)/2)</f>
@@ -1630,238 +1584,217 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <f aca="false">(Inputs!$B$32+Inputs!$B$33+Inputs!$B$34+Inputs!$B$35)/(Inputs!$B$4-1)</f>
+        <v>69</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <f aca="false">(Inputs!$B$32+Inputs!$B$33+Inputs!$B$34+Inputs!$B$35)/(Inputs!$B$4-1)</f>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="9" t="n">
+        <f aca="false">SUM(B3:B8)</f>
+        <v>1314</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <f aca="false">SUM(C3:C8)</f>
+        <v>1109</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <f aca="false">ROUND(B9*Inputs!$B$7,0)</f>
+        <v>79</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <f aca="false">ROUND(C9*Inputs!$B$7,0)</f>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B8" s="8" t="n">
-        <f aca="false">Inputs!$B$31+Inputs!$B$32+Inputs!$B$33</f>
-        <v>110</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <f aca="false">Inputs!$B$31+Inputs!$B$32+Inputs!$B$33</f>
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="B11" s="9" t="n">
+        <f aca="false">CEILING(B9+B10,5)</f>
+        <v>1395</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <f aca="false">CEILING(C9+C10,5)</f>
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B9" s="8" t="n">
-        <f aca="false">(Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38)/(Inputs!$B$4-1)</f>
-        <v>81.9473684210526</v>
-      </c>
-      <c r="C9" s="8" t="n">
-        <f aca="false">(Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38)/(Inputs!$B$4-1)</f>
-        <v>81.9473684210526</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B10" s="9" t="n">
-        <f aca="false">SUM(B3:B9)</f>
-        <v>1436.94736842105</v>
-      </c>
-      <c r="C10" s="9" t="n">
-        <f aca="false">SUM(C3:C9)</f>
-        <v>1231.94736842105</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B11" s="8" t="n">
-        <f aca="false">ROUND(B10*Inputs!$B$7,0)</f>
-        <v>86</v>
-      </c>
-      <c r="C11" s="8" t="n">
-        <f aca="false">ROUND(C10*Inputs!$B$7,0)</f>
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B12" s="9" t="n">
-        <f aca="false">CEILING(B10+B11,5)</f>
-        <v>1525</v>
-      </c>
-      <c r="C12" s="9" t="n">
-        <f aca="false">CEILING(C10+C11,5)</f>
-        <v>1310</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
+        <v>87</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <f aca="false">Inputs!$B$12*5</f>
+        <v>150</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C15" s="8" t="n">
-        <f aca="false">Inputs!$B$12*5</f>
-        <v>150</v>
+        <f aca="false">Inputs!$B$41</f>
+        <v>220</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C16" s="8" t="n">
-        <f aca="false">Inputs!$B$43</f>
-        <v>220</v>
+        <f aca="false">Inputs!$B$21*10</f>
+        <v>120</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>93</v>
+        <v>91</v>
+      </c>
+      <c r="B17" s="8" t="n">
+        <f aca="false">Inputs!$B$19+Inputs!$B$13</f>
+        <v>145</v>
       </c>
       <c r="C17" s="8" t="n">
-        <f aca="false">Inputs!$B$21*10</f>
-        <v>120</v>
+        <f aca="false">Inputs!$B$19+Inputs!$B$13</f>
+        <v>145</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B18" s="8" t="n">
-        <f aca="false">((Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)/2)</f>
-        <v>246</v>
-      </c>
-      <c r="C18" s="8" t="n">
-        <f aca="false">((Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)/2)</f>
-        <v>246</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B19" s="8" t="n">
-        <f aca="false">Inputs!$B$19+Inputs!$B$13</f>
-        <v>145</v>
-      </c>
-      <c r="C19" s="8" t="n">
-        <f aca="false">Inputs!$B$19+Inputs!$B$13</f>
-        <v>145</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B20" s="8" t="n">
         <f aca="false">Inputs!$B$20/10</f>
         <v>80</v>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C18" s="8" t="n">
         <f aca="false">Inputs!$B$20/10</f>
         <v>80</v>
       </c>
     </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+    </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
+      <c r="A21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="8" t="n">
+        <f aca="false">B11</f>
+        <v>1395</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <f aca="false">C11</f>
+        <v>1180</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
+      <c r="A22" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B22" s="8" t="n">
+        <f aca="false">Inputs!$B$37*Inputs!$B$38+Inputs!$B$39+Inputs!$B$40</f>
+        <v>350</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <f aca="false">Inputs!$B$37*Inputs!$B$38+Inputs!$B$39+Inputs!$B$40</f>
+        <v>350</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B23" s="8" t="n">
-        <f aca="false">B12</f>
-        <v>1525</v>
-      </c>
-      <c r="C23" s="8" t="n">
-        <f aca="false">C12</f>
-        <v>1310</v>
+      <c r="A23" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" s="9" t="n">
+        <f aca="false">B21+B22</f>
+        <v>1745</v>
+      </c>
+      <c r="C23" s="9" t="n">
+        <f aca="false">C21+C22</f>
+        <v>1530</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B24" s="8" t="n">
-        <f aca="false">Inputs!$B$40*Inputs!$B$41+Inputs!$B$42</f>
-        <v>290</v>
-      </c>
-      <c r="C24" s="8" t="n">
-        <f aca="false">Inputs!$B$40*Inputs!$B$41+Inputs!$B$42</f>
-        <v>290</v>
+      <c r="A24" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" s="9" t="n">
+        <f aca="false">B23</f>
+        <v>1745</v>
+      </c>
+      <c r="C24" s="9" t="n">
+        <f aca="false">C23+C14</f>
+        <v>1680</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B25" s="9" t="n">
-        <f aca="false">B23+B24</f>
-        <v>1815</v>
+        <v>98</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>89</v>
       </c>
       <c r="C25" s="9" t="n">
-        <f aca="false">C23+C24</f>
-        <v>1600</v>
+        <f aca="false">C23+C15+C16</f>
+        <v>1870</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="B26" s="9" t="n">
-        <f aca="false">B25</f>
-        <v>1815</v>
-      </c>
-      <c r="C26" s="9" t="n">
-        <f aca="false">C25+C15</f>
-        <v>1750</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="C27" s="9" t="n">
-        <f aca="false">C25+C16+C17</f>
-        <v>1940</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+    </row>
+    <row r="27" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1879,7 +1812,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="66"/>
@@ -1888,7 +1821,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1898,21 +1831,21 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>12</v>
@@ -1929,7 +1862,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
@@ -1950,7 +1883,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$6,0)</f>
@@ -1971,7 +1904,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">B4-B5</f>
@@ -1990,30 +1923,30 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B7" s="10" t="n">
-        <f aca="false">ROUNDUP(B4/2,0)</f>
+        <f aca="false">ROUNDUP(B3/2,0)</f>
         <v>6</v>
       </c>
       <c r="C7" s="10" t="n">
-        <f aca="false">ROUNDUP(C4/2,0)</f>
+        <f aca="false">ROUNDUP(C3/2,0)</f>
         <v>10</v>
       </c>
       <c r="D7" s="10" t="n">
-        <f aca="false">ROUNDUP(D4/2,0)</f>
+        <f aca="false">ROUNDUP(D3/2,0)</f>
         <v>15</v>
       </c>
       <c r="E7" s="10" t="n">
-        <f aca="false">ROUNDUP(E4/2,0)</f>
+        <f aca="false">ROUNDUP(E3/2,0)</f>
         <v>20</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2022,28 +1955,28 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B9" s="9" t="n">
-        <f aca="false">B5*Fee!$B$12+B6*Fee!$C$12</f>
-        <v>15700</v>
+        <f aca="false">B5*Fee!$B$11+B6*Fee!$C$11</f>
+        <v>14270</v>
       </c>
       <c r="C9" s="9" t="n">
-        <f aca="false">C5*Fee!$B$12+C6*Fee!$C$12</f>
-        <v>27040</v>
+        <f aca="false">C5*Fee!$B$11+C6*Fee!$C$11</f>
+        <v>24570</v>
       </c>
       <c r="D9" s="9" t="n">
-        <f aca="false">D5*Fee!$B$12+D6*Fee!$C$12</f>
-        <v>41215</v>
+        <f aca="false">D5*Fee!$B$11+D6*Fee!$C$11</f>
+        <v>37445</v>
       </c>
       <c r="E9" s="9" t="n">
-        <f aca="false">E5*Fee!$B$12+E6*Fee!$C$12</f>
-        <v>55390</v>
+        <f aca="false">E5*Fee!$B$11+E6*Fee!$C$11</f>
+        <v>50320</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2052,7 +1985,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$9+Inputs!$B$10)</f>
@@ -2073,7 +2006,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B6*Inputs!$B$11</f>
@@ -2094,7 +2027,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">INT(B6/Inputs!$B$17)</f>
@@ -2115,7 +2048,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">IF(B13&gt;=1,0,Inputs!$B$11)</f>
@@ -2136,7 +2069,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">-MAX(B13-1,0)*Inputs!$B$11</f>
@@ -2157,7 +2090,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B11+B12+B14+B15</f>
@@ -2178,7 +2111,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">-B12*Inputs!$B$16</f>
@@ -2199,7 +2132,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B16+B17</f>
@@ -2220,7 +2153,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-B17</f>
@@ -2241,7 +2174,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B5*Inputs!$B$13*Inputs!$B$15+(B6+1)*Inputs!$B$13*Inputs!$B$14</f>
@@ -2262,7 +2195,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B21" s="8" t="n">
         <f aca="false">B5*Inputs!$B$29</f>
@@ -2283,7 +2216,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B3*Inputs!$B$30</f>
@@ -2304,345 +2237,324 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B23" s="8" t="n">
-        <f aca="false">(B7+1)*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
-        <v>3444</v>
+        <f aca="false">B7*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
+        <v>2952</v>
       </c>
       <c r="C23" s="8" t="n">
-        <f aca="false">(C7+1)*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
-        <v>5412</v>
+        <f aca="false">C7*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
+        <v>4920</v>
       </c>
       <c r="D23" s="8" t="n">
-        <f aca="false">(D7+1)*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
-        <v>7872</v>
+        <f aca="false">D7*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
+        <v>7380</v>
       </c>
       <c r="E23" s="8" t="n">
-        <f aca="false">(E7+1)*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
-        <v>10332</v>
+        <f aca="false">E7*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
+        <v>9840</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>131</v>
+        <v>56</v>
       </c>
       <c r="B24" s="8" t="n">
-        <f aca="false">B3*(Inputs!$B$31+Inputs!$B$32+Inputs!$B$33)</f>
-        <v>1320</v>
+        <f aca="false">Inputs!$B$32</f>
+        <v>700</v>
       </c>
       <c r="C24" s="8" t="n">
-        <f aca="false">C3*(Inputs!$B$31+Inputs!$B$32+Inputs!$B$33)</f>
-        <v>2200</v>
+        <f aca="false">Inputs!$B$32</f>
+        <v>700</v>
       </c>
       <c r="D24" s="8" t="n">
-        <f aca="false">D3*(Inputs!$B$31+Inputs!$B$32+Inputs!$B$33)</f>
-        <v>3300</v>
+        <f aca="false">Inputs!$B$32</f>
+        <v>700</v>
       </c>
       <c r="E24" s="8" t="n">
-        <f aca="false">E3*(Inputs!$B$31+Inputs!$B$32+Inputs!$B$33)</f>
-        <v>4400</v>
+        <f aca="false">Inputs!$B$32</f>
+        <v>700</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B25" s="8" t="n">
-        <f aca="false">Inputs!$B$35</f>
-        <v>700</v>
-      </c>
-      <c r="C25" s="8" t="n">
-        <f aca="false">Inputs!$B$35</f>
-        <v>700</v>
-      </c>
-      <c r="D25" s="8" t="n">
-        <f aca="false">Inputs!$B$35</f>
-        <v>700</v>
-      </c>
-      <c r="E25" s="8" t="n">
-        <f aca="false">Inputs!$B$35</f>
-        <v>700</v>
+      <c r="A25" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B25" s="9" t="n">
+        <f aca="false">B18+B19+B20+B21+B22+B23+B24</f>
+        <v>13810</v>
+      </c>
+      <c r="C25" s="9" t="n">
+        <f aca="false">C18+C19+C20+C21+C22+C23+C24</f>
+        <v>22950</v>
+      </c>
+      <c r="D25" s="9" t="n">
+        <f aca="false">D18+D19+D20+D21+D22+D23+D24</f>
+        <v>33775</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <f aca="false">E18+E19+E20+E21+E22+E23+E24</f>
+        <v>44600</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="B26" s="9" t="n">
-        <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25</f>
-        <v>15622</v>
-      </c>
-      <c r="C26" s="9" t="n">
-        <f aca="false">C18+C19+C20+C21+C22+C23+C24+C25</f>
-        <v>25642</v>
-      </c>
-      <c r="D26" s="9" t="n">
-        <f aca="false">D18+D19+D20+D21+D22+D23+D24+D25</f>
-        <v>37567</v>
-      </c>
-      <c r="E26" s="9" t="n">
-        <f aca="false">E18+E19+E20+E21+E22+E23+E24+E25</f>
-        <v>49492</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
+        <v>128</v>
+      </c>
+      <c r="B27" s="9" t="n">
+        <f aca="false">B9-B25</f>
+        <v>460</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <f aca="false">C9-C25</f>
+        <v>1620</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <f aca="false">D9-D25</f>
+        <v>3670</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <f aca="false">E9-E25</f>
+        <v>5720</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="B28" s="9" t="n">
-        <f aca="false">B9-B26</f>
-        <v>78</v>
-      </c>
-      <c r="C28" s="9" t="n">
-        <f aca="false">C9-C26</f>
-        <v>1398</v>
-      </c>
-      <c r="D28" s="9" t="n">
-        <f aca="false">D9-D26</f>
-        <v>3648</v>
-      </c>
-      <c r="E28" s="9" t="n">
-        <f aca="false">E9-E26</f>
-        <v>5898</v>
+      <c r="A28" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" s="8" t="n">
+        <f aca="false">B27/B4</f>
+        <v>41.8181818181818</v>
+      </c>
+      <c r="C28" s="8" t="n">
+        <f aca="false">C27/C4</f>
+        <v>85.2631578947368</v>
+      </c>
+      <c r="D28" s="8" t="n">
+        <f aca="false">D27/D4</f>
+        <v>126.551724137931</v>
+      </c>
+      <c r="E28" s="8" t="n">
+        <f aca="false">E27/E4</f>
+        <v>146.666666666667</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B29" s="8" t="n">
-        <f aca="false">B28/B4</f>
-        <v>7.09090909090909</v>
-      </c>
-      <c r="C29" s="8" t="n">
-        <f aca="false">C28/C4</f>
-        <v>73.5789473684211</v>
-      </c>
-      <c r="D29" s="8" t="n">
-        <f aca="false">D28/D4</f>
-        <v>125.793103448276</v>
-      </c>
-      <c r="E29" s="8" t="n">
-        <f aca="false">E28/E4</f>
-        <v>151.230769230769</v>
+        <v>130</v>
+      </c>
+      <c r="B29" s="11" t="n">
+        <f aca="false">B27/B9</f>
+        <v>0.0322354590049054</v>
+      </c>
+      <c r="C29" s="11" t="n">
+        <f aca="false">C27/C9</f>
+        <v>0.0659340659340659</v>
+      </c>
+      <c r="D29" s="11" t="n">
+        <f aca="false">D27/D9</f>
+        <v>0.0980104152757378</v>
+      </c>
+      <c r="E29" s="11" t="n">
+        <f aca="false">E27/E9</f>
+        <v>0.113672496025437</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B30" s="11" t="n">
-        <f aca="false">B28/B9</f>
-        <v>0.00496815286624204</v>
-      </c>
-      <c r="C30" s="11" t="n">
-        <f aca="false">C28/C9</f>
-        <v>0.0517011834319527</v>
-      </c>
-      <c r="D30" s="11" t="n">
-        <f aca="false">D28/D9</f>
-        <v>0.0885114642727163</v>
-      </c>
-      <c r="E30" s="11" t="n">
-        <f aca="false">E28/E9</f>
-        <v>0.106481314316664</v>
+      <c r="A30" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B30" s="12" t="str">
+        <f aca="false">IF(B27&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="C30" s="12" t="str">
+        <f aca="false">IF(C27&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="D30" s="12" t="str">
+        <f aca="false">IF(D27&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="E30" s="12" t="str">
+        <f aca="false">IF(E27&gt;=0,"yes","NO")</f>
+        <v>yes</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B31" s="12" t="str">
-        <f aca="false">IF(B28&gt;=0,"yes","NO")</f>
-        <v>yes</v>
-      </c>
-      <c r="C31" s="12" t="str">
-        <f aca="false">IF(C28&gt;=0,"yes","NO")</f>
-        <v>yes</v>
-      </c>
-      <c r="D31" s="12" t="str">
-        <f aca="false">IF(D28&gt;=0,"yes","NO")</f>
-        <v>yes</v>
-      </c>
-      <c r="E31" s="12" t="str">
-        <f aca="false">IF(E28&gt;=0,"yes","NO")</f>
-        <v>yes</v>
+        <v>132</v>
+      </c>
+      <c r="B31" s="9" t="n">
+        <f aca="false">B19</f>
+        <v>300</v>
+      </c>
+      <c r="C31" s="9" t="n">
+        <f aca="false">C19</f>
+        <v>540</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <f aca="false">D19</f>
+        <v>840</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <f aca="false">E19</f>
+        <v>1140</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="B32" s="9" t="n">
-        <f aca="false">B19</f>
-        <v>300</v>
-      </c>
-      <c r="C32" s="9" t="n">
-        <f aca="false">C19</f>
-        <v>540</v>
-      </c>
-      <c r="D32" s="9" t="n">
-        <f aca="false">D19</f>
-        <v>840</v>
-      </c>
-      <c r="E32" s="9" t="n">
-        <f aca="false">E19</f>
-        <v>1140</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
+      <c r="A33" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B33" s="8" t="n">
+        <f aca="false">B4*400</f>
+        <v>4400</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <f aca="false">C4*400</f>
+        <v>7600</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <f aca="false">D4*400</f>
+        <v>11600</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <f aca="false">E4*400</f>
+        <v>15600</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B34" s="8" t="n">
-        <f aca="false">B4*400</f>
-        <v>4400</v>
+        <f aca="false">B16*Inputs!$B$18+B23*Inputs!$B$27</f>
+        <v>2448</v>
       </c>
       <c r="C34" s="8" t="n">
-        <f aca="false">C4*400</f>
-        <v>7600</v>
+        <f aca="false">C16*Inputs!$B$18+C23*Inputs!$B$27</f>
+        <v>4180</v>
       </c>
       <c r="D34" s="8" t="n">
-        <f aca="false">D4*400</f>
-        <v>11600</v>
+        <f aca="false">D16*Inputs!$B$18+D23*Inputs!$B$27</f>
+        <v>6195</v>
       </c>
       <c r="E34" s="8" t="n">
-        <f aca="false">E4*400</f>
-        <v>15600</v>
+        <f aca="false">E16*Inputs!$B$18+E23*Inputs!$B$27</f>
+        <v>8210</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B35" s="8" t="n">
-        <f aca="false">B16*Inputs!$B$18+B23*Inputs!$B$27</f>
-        <v>2571</v>
-      </c>
-      <c r="C35" s="8" t="n">
-        <f aca="false">C16*Inputs!$B$18+C23*Inputs!$B$27</f>
-        <v>4303</v>
-      </c>
-      <c r="D35" s="8" t="n">
-        <f aca="false">D16*Inputs!$B$18+D23*Inputs!$B$27</f>
-        <v>6318</v>
-      </c>
-      <c r="E35" s="8" t="n">
-        <f aca="false">E16*Inputs!$B$18+E23*Inputs!$B$27</f>
-        <v>8333</v>
+      <c r="A35" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B35" s="9" t="n">
+        <f aca="false">B33-B34</f>
+        <v>1952</v>
+      </c>
+      <c r="C35" s="9" t="n">
+        <f aca="false">C33-C34</f>
+        <v>3420</v>
+      </c>
+      <c r="D35" s="9" t="n">
+        <f aca="false">D33-D34</f>
+        <v>5405</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <f aca="false">E33-E34</f>
+        <v>7390</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="B36" s="9" t="n">
-        <f aca="false">B34-B35</f>
-        <v>1829</v>
-      </c>
-      <c r="C36" s="9" t="n">
-        <f aca="false">C34-C35</f>
-        <v>3297</v>
-      </c>
-      <c r="D36" s="9" t="n">
-        <f aca="false">D34-D35</f>
-        <v>5282</v>
-      </c>
-      <c r="E36" s="9" t="n">
-        <f aca="false">E34-E35</f>
-        <v>7267</v>
+      <c r="A36" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B36" s="8" t="n">
+        <f aca="false">B9-B33</f>
+        <v>9870</v>
+      </c>
+      <c r="C36" s="8" t="n">
+        <f aca="false">C9-C33</f>
+        <v>16970</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <f aca="false">D9-D33</f>
+        <v>25845</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <f aca="false">E9-E33</f>
+        <v>34720</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B37" s="8" t="n">
-        <f aca="false">B9-B34</f>
-        <v>11300</v>
+        <f aca="false">B18-B16*Inputs!$B$18+B23*(1-Inputs!$B$27)+B21+B22</f>
+        <v>9642</v>
       </c>
       <c r="C37" s="8" t="n">
-        <f aca="false">C9-C34</f>
-        <v>19440</v>
+        <f aca="false">C18-C16*Inputs!$B$18+C23*(1-Inputs!$B$27)+C21+C22</f>
+        <v>16330</v>
       </c>
       <c r="D37" s="8" t="n">
-        <f aca="false">D9-D34</f>
-        <v>29615</v>
+        <f aca="false">D18-D16*Inputs!$B$18+D23*(1-Inputs!$B$27)+D21+D22</f>
+        <v>24240</v>
       </c>
       <c r="E37" s="8" t="n">
-        <f aca="false">E9-E34</f>
-        <v>39790</v>
+        <f aca="false">E18-E16*Inputs!$B$18+E23*(1-Inputs!$B$27)+E21+E22</f>
+        <v>32150</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B38" s="8" t="n">
-        <f aca="false">B18-B16*Inputs!$B$18+B23*(1-Inputs!$B$27)+B21+B22</f>
-        <v>10011</v>
+        <f aca="false">B20</f>
+        <v>720</v>
       </c>
       <c r="C38" s="8" t="n">
-        <f aca="false">C18-C16*Inputs!$B$18+C23*(1-Inputs!$B$27)+C21+C22</f>
-        <v>16699</v>
+        <f aca="false">C20</f>
+        <v>1200</v>
       </c>
       <c r="D38" s="8" t="n">
-        <f aca="false">D18-D16*Inputs!$B$18+D23*(1-Inputs!$B$27)+D21+D22</f>
-        <v>24609</v>
+        <f aca="false">D20</f>
+        <v>1800</v>
       </c>
       <c r="E38" s="8" t="n">
-        <f aca="false">E18-E16*Inputs!$B$18+E23*(1-Inputs!$B$27)+E21+E22</f>
-        <v>32519</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">E20</f>
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="B39" s="8" t="n">
-        <f aca="false">B20+B24</f>
-        <v>2040</v>
-      </c>
-      <c r="C39" s="8" t="n">
-        <f aca="false">C20+C24</f>
-        <v>3400</v>
-      </c>
-      <c r="D39" s="8" t="n">
-        <f aca="false">D20+D24</f>
-        <v>5100</v>
-      </c>
-      <c r="E39" s="8" t="n">
-        <f aca="false">E20+E24</f>
-        <v>6800</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
+        <v>140</v>
+      </c>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2670,108 +2582,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2781,10 +2693,10 @@
     </row>
     <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>10</v>
@@ -2792,10 +2704,10 @@
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Budget: all gear rental inside the trip fee
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="173">
   <si>
     <t xml:space="preserve">Cozumel group budget — inputs (blue cells are editable)</t>
   </si>
@@ -88,12 +88,27 @@
     <t xml:space="preserve">Certified 5-day two-tank package</t>
   </si>
   <si>
-    <t xml:space="preserve">Equipment rental per day (add-on at cost for those who need it)</t>
+    <t xml:space="preserve">Equipment rental per day, everyone rents (in the fee)</t>
   </si>
   <si>
     <t xml:space="preserve">USD/day</t>
   </si>
   <si>
+    <t xml:space="preserve">Rental days, certified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">programme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rental days, new divers (course includes equipment; the two extra boat days do not)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSUMED; ask Blue Note whether the USD 240 extra days include gear</t>
+  </si>
+  <si>
     <t xml:space="preserve">Marine park fee per boat day</t>
   </si>
   <si>
@@ -103,12 +118,6 @@
     <t xml:space="preserve">Boat days, certified</t>
   </si>
   <si>
-    <t xml:space="preserve">days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">programme</t>
-  </si>
-  <si>
     <t xml:space="preserve">Boat days, new divers (dive 3–4 day + Thu + Fri)</t>
   </si>
   <si>
@@ -214,6 +223,9 @@
     <t xml:space="preserve">George's DAN cover</t>
   </si>
   <si>
+    <t xml:space="preserve">George's gear rental, 5 days</t>
+  </si>
+  <si>
     <t xml:space="preserve">Own spending guidance, not in the fee (no flights)</t>
   </si>
   <si>
@@ -256,6 +268,9 @@
     <t xml:space="preserve">Diving with Blue Note</t>
   </si>
   <si>
+    <t xml:space="preserve">Gear rental, everyone</t>
+  </si>
+  <si>
     <t xml:space="preserve">Marine park fees</t>
   </si>
   <si>
@@ -271,7 +286,7 @@
     <t xml:space="preserve">Hotel Plaza, 6 nights with breakfast, 2 sharing</t>
   </si>
   <si>
-    <t xml:space="preserve">Leader's costs shared (George's flight, half-room, DAN, odd-room risk)</t>
+    <t xml:space="preserve">Leader's costs shared (George's flight, half-room, DAN, rental, odd-room risk)</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal</t>
@@ -283,10 +298,7 @@
     <t xml:space="preserve">TRIP FEE (rounded up to the nearest 5)</t>
   </si>
   <si>
-    <t xml:space="preserve">Add-ons at sign-up, charged at cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gear rental, 5 days (certified who need it)</t>
+    <t xml:space="preserve">Optional add-ons at sign-up, charged at cost</t>
   </si>
   <si>
     <t xml:space="preserve">AOW: course free with eLearning; eLearning</t>
@@ -313,16 +325,13 @@
     <t xml:space="preserve">Own spending: meals, drinks, tips, airport transfers</t>
   </si>
   <si>
-    <t xml:space="preserve">Guidance budget, own gear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guidance budget, renting gear</t>
+    <t xml:space="preserve">Guidance budget</t>
   </si>
   <si>
     <t xml:space="preserve">Guidance budget, certified taking AOW and nitrox</t>
   </si>
   <si>
-    <t xml:space="preserve">The fee covers diving, insurance and the hotel; everything else is the person's own. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
+    <t xml:space="preserve">The fee covers everything diving-related (course or package, gear, park fees, eLearning), DAN insurance and the hotel; everything else is the person's own. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
   </si>
   <si>
     <t xml:space="preserve">Group budget at four sizes (half students; George leads and does not pay)</t>
@@ -391,6 +400,9 @@
     <t xml:space="preserve">Commission passed to George</t>
   </si>
   <si>
+    <t xml:space="preserve">Gear rental for everyone including George</t>
+  </si>
+  <si>
     <t xml:space="preserve">Marine park fees (cash on the island, paid from the float)</t>
   </si>
   <si>
@@ -439,7 +451,7 @@
     <t xml:space="preserve">Balances due from participants by Fri 6 Nov</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue Note balance Fri 13 Nov + hotel balance + eLearning + DAN</t>
+    <t xml:space="preserve">Blue Note balance Fri 13 Nov + rental + hotel balance + eLearning + DAN</t>
   </si>
   <si>
     <t xml:space="preserve">Cash float to carry to the island (park fees)</t>
@@ -941,7 +953,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72"/>
@@ -1103,25 +1115,25 @@
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="7" t="n">
-        <v>15</v>
+      <c r="B13" s="5" t="n">
+        <v>5</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>27</v>
@@ -1131,28 +1143,28 @@
       <c r="A15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="5" t="n">
-        <v>3</v>
+      <c r="B15" s="7" t="n">
+        <v>15</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" s="6" t="n">
-        <v>0.1</v>
+        <v>30</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>5</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1160,55 +1172,55 @@
         <v>31</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="7" t="n">
-        <v>130</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="D19" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>800</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1216,7 +1228,7 @@
         <v>38</v>
       </c>
       <c r="B21" s="7" t="n">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>17</v>
@@ -1226,19 +1238,25 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+      <c r="B22" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B23" s="7" t="n">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>17</v>
@@ -1248,235 +1266,272 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="7" t="n">
-        <v>88</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>4</v>
+        <v>46</v>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>88</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D26" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="B27" s="6" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
+      <c r="B28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="D28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B29" s="7" t="n">
-        <v>195</v>
+      <c r="B29" s="6" t="n">
+        <v>0.25</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="7" t="n">
-        <v>119</v>
-      </c>
-      <c r="C30" s="2" t="s">
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>195</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
+      <c r="D31" s="2" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B32" s="7" t="n">
-        <v>700</v>
+        <v>119</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="7" t="n">
-        <f aca="false">(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)/2</f>
-        <v>246</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>59</v>
-      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B34" s="7" t="n">
-        <f aca="false">Inputs!$B$33</f>
-        <v>246</v>
+        <v>700</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B35" s="7" t="n">
-        <v>119</v>
+        <f aca="false">(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2</f>
+        <v>246</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
+      <c r="B36" s="7" t="n">
+        <f aca="false">Inputs!$B$35</f>
+        <v>246</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B37" s="7" t="n">
-        <v>45</v>
+        <v>119</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="5" t="n">
-        <v>6</v>
+      <c r="B38" s="7" t="n">
+        <f aca="false">Inputs!$B$12*5</f>
+        <v>150</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D38" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
+      <c r="A39" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B39" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>68</v>
-      </c>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="B40" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B41" s="7" t="n">
+      <c r="B42" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B44" s="7" t="n">
         <v>220</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C44" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>72</v>
+      <c r="D44" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1495,7 +1550,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -1504,7 +1559,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1512,15 +1567,15 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">Inputs!$B$9+Inputs!$B$10</f>
@@ -1533,178 +1588,179 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B4" s="8" t="n">
-        <f aca="false">Inputs!$B$13*Inputs!$B$15</f>
-        <v>45</v>
+        <f aca="false">Inputs!$B$12*Inputs!$B$14</f>
+        <v>60</v>
       </c>
       <c r="C4" s="8" t="n">
-        <f aca="false">Inputs!$B$13*Inputs!$B$14</f>
-        <v>75</v>
+        <f aca="false">Inputs!$B$12*Inputs!$B$13</f>
+        <v>150</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B5" s="8" t="n">
-        <f aca="false">Inputs!$B$29</f>
-        <v>195</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>79</v>
+        <f aca="false">Inputs!$B$15*Inputs!$B$17</f>
+        <v>45</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <f aca="false">Inputs!$B$15*Inputs!$B$16</f>
+        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B6" s="8" t="n">
-        <f aca="false">Inputs!$B$30</f>
-        <v>119</v>
-      </c>
-      <c r="C6" s="8" t="n">
-        <f aca="false">Inputs!$B$30</f>
-        <v>119</v>
+        <f aca="false">Inputs!$B$31</f>
+        <v>195</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B7" s="8" t="n">
-        <f aca="false">((Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)/2)</f>
-        <v>246</v>
+        <f aca="false">Inputs!$B$32</f>
+        <v>119</v>
       </c>
       <c r="C7" s="8" t="n">
-        <f aca="false">((Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)/2)</f>
-        <v>246</v>
+        <f aca="false">Inputs!$B$32</f>
+        <v>119</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B8" s="8" t="n">
-        <f aca="false">(Inputs!$B$32+Inputs!$B$33+Inputs!$B$34+Inputs!$B$35)/(Inputs!$B$4-1)</f>
-        <v>69</v>
+        <f aca="false">((Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2)</f>
+        <v>246</v>
       </c>
       <c r="C8" s="8" t="n">
-        <f aca="false">(Inputs!$B$32+Inputs!$B$33+Inputs!$B$34+Inputs!$B$35)/(Inputs!$B$4-1)</f>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+        <f aca="false">((Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2)</f>
+        <v>246</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" s="8" t="n">
+        <f aca="false">(Inputs!$B$34+Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38)/(Inputs!$B$4-1)</f>
+        <v>76.8947368421053</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <f aca="false">(Inputs!$B$34+Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38)/(Inputs!$B$4-1)</f>
+        <v>76.8947368421053</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" s="9" t="n">
+        <f aca="false">SUM(B3:B9)</f>
+        <v>1381.89473684211</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <f aca="false">SUM(C3:C9)</f>
+        <v>1266.89473684211</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <f aca="false">ROUND(B10*Inputs!$B$7,0)</f>
         <v>83</v>
       </c>
-      <c r="B9" s="9" t="n">
-        <f aca="false">SUM(B3:B8)</f>
-        <v>1314</v>
-      </c>
-      <c r="C9" s="9" t="n">
-        <f aca="false">SUM(C3:C8)</f>
-        <v>1109</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B10" s="8" t="n">
-        <f aca="false">ROUND(B9*Inputs!$B$7,0)</f>
-        <v>79</v>
-      </c>
-      <c r="C10" s="8" t="n">
-        <f aca="false">ROUND(C9*Inputs!$B$7,0)</f>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B11" s="9" t="n">
-        <f aca="false">CEILING(B9+B10,5)</f>
-        <v>1395</v>
-      </c>
-      <c r="C11" s="9" t="n">
-        <f aca="false">CEILING(C9+C10,5)</f>
-        <v>1180</v>
+      <c r="C11" s="8" t="n">
+        <f aca="false">ROUND(C10*Inputs!$B$7,0)</f>
+        <v>76</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
+      <c r="A12" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="9" t="n">
+        <f aca="false">CEILING(B10+B11,5)</f>
+        <v>1465</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <f aca="false">CEILING(C10+C11,5)</f>
+        <v>1345</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>86</v>
-      </c>
+      <c r="A13" s="2"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="C14" s="8" t="n">
-        <f aca="false">Inputs!$B$12*5</f>
-        <v>150</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C15" s="8" t="n">
-        <f aca="false">Inputs!$B$41</f>
+        <f aca="false">Inputs!$B$44</f>
         <v>220</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C16" s="8" t="n">
-        <f aca="false">Inputs!$B$21*10</f>
+        <f aca="false">Inputs!$B$23*10</f>
         <v>120</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B17" s="8" t="n">
-        <f aca="false">Inputs!$B$19+Inputs!$B$13</f>
+        <f aca="false">Inputs!$B$21+Inputs!$B$15</f>
         <v>145</v>
       </c>
       <c r="C17" s="8" t="n">
-        <f aca="false">Inputs!$B$19+Inputs!$B$13</f>
+        <f aca="false">Inputs!$B$21+Inputs!$B$15</f>
         <v>145</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B18" s="8" t="n">
-        <f aca="false">Inputs!$B$20/10</f>
+        <f aca="false">Inputs!$B$22/10</f>
         <v>80</v>
       </c>
       <c r="C18" s="8" t="n">
-        <f aca="false">Inputs!$B$20/10</f>
+        <f aca="false">Inputs!$B$22/10</f>
         <v>80</v>
       </c>
     </row>
@@ -1715,86 +1771,73 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B21" s="8" t="n">
-        <f aca="false">B11</f>
-        <v>1395</v>
+        <f aca="false">B12</f>
+        <v>1465</v>
       </c>
       <c r="C21" s="8" t="n">
-        <f aca="false">C11</f>
-        <v>1180</v>
+        <f aca="false">C12</f>
+        <v>1345</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B22" s="8" t="n">
-        <f aca="false">Inputs!$B$37*Inputs!$B$38+Inputs!$B$39+Inputs!$B$40</f>
+        <f aca="false">Inputs!$B$40*Inputs!$B$41+Inputs!$B$42+Inputs!$B$43</f>
         <v>350</v>
       </c>
       <c r="C22" s="8" t="n">
-        <f aca="false">Inputs!$B$37*Inputs!$B$38+Inputs!$B$39+Inputs!$B$40</f>
+        <f aca="false">Inputs!$B$40*Inputs!$B$41+Inputs!$B$42+Inputs!$B$43</f>
         <v>350</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B23" s="9" t="n">
         <f aca="false">B21+B22</f>
-        <v>1745</v>
+        <v>1815</v>
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">C21+C22</f>
-        <v>1530</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B24" s="9" t="n">
-        <f aca="false">B23</f>
-        <v>1745</v>
+        <v>101</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>93</v>
       </c>
       <c r="C24" s="9" t="n">
-        <f aca="false">C23+C14</f>
-        <v>1680</v>
+        <f aca="false">C23+C15+C16</f>
+        <v>2035</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C25" s="9" t="n">
-        <f aca="false">C23+C15+C16</f>
-        <v>1870</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>102</v>
+      </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
-    </row>
-    <row r="27" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1812,7 +1855,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="66"/>
@@ -1821,7 +1864,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1831,21 +1874,21 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>12</v>
@@ -1862,7 +1905,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
@@ -1883,7 +1926,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$6,0)</f>
@@ -1904,7 +1947,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">B4-B5</f>
@@ -1925,7 +1968,7 @@
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">ROUNDUP(B3/2,0)</f>
@@ -1946,7 +1989,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1955,28 +1998,28 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B9" s="9" t="n">
-        <f aca="false">B5*Fee!$B$11+B6*Fee!$C$11</f>
-        <v>14270</v>
+        <f aca="false">B5*Fee!$B$12+B6*Fee!$C$12</f>
+        <v>15515</v>
       </c>
       <c r="C9" s="9" t="n">
-        <f aca="false">C5*Fee!$B$11+C6*Fee!$C$11</f>
-        <v>24570</v>
+        <f aca="false">C5*Fee!$B$12+C6*Fee!$C$12</f>
+        <v>26755</v>
       </c>
       <c r="D9" s="9" t="n">
-        <f aca="false">D5*Fee!$B$11+D6*Fee!$C$11</f>
-        <v>37445</v>
+        <f aca="false">D5*Fee!$B$12+D6*Fee!$C$12</f>
+        <v>40805</v>
       </c>
       <c r="E9" s="9" t="n">
-        <f aca="false">E5*Fee!$B$11+E6*Fee!$C$11</f>
-        <v>50320</v>
+        <f aca="false">E5*Fee!$B$12+E6*Fee!$C$12</f>
+        <v>54855</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1985,7 +2028,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$9+Inputs!$B$10)</f>
@@ -2006,7 +2049,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B6*Inputs!$B$11</f>
@@ -2027,28 +2070,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B13" s="10" t="n">
-        <f aca="false">INT(B6/Inputs!$B$17)</f>
+        <f aca="false">INT(B6/Inputs!$B$19)</f>
         <v>1</v>
       </c>
       <c r="C13" s="10" t="n">
-        <f aca="false">INT(C6/Inputs!$B$17)</f>
+        <f aca="false">INT(C6/Inputs!$B$19)</f>
         <v>1</v>
       </c>
       <c r="D13" s="10" t="n">
-        <f aca="false">INT(D6/Inputs!$B$17)</f>
+        <f aca="false">INT(D6/Inputs!$B$19)</f>
         <v>2</v>
       </c>
       <c r="E13" s="10" t="n">
-        <f aca="false">INT(E6/Inputs!$B$17)</f>
+        <f aca="false">INT(E6/Inputs!$B$19)</f>
         <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">IF(B13&gt;=1,0,Inputs!$B$11)</f>
@@ -2069,7 +2112,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">-MAX(B13-1,0)*Inputs!$B$11</f>
@@ -2090,7 +2133,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B11+B12+B14+B15</f>
@@ -2111,28 +2154,28 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B17" s="8" t="n">
-        <f aca="false">-B12*Inputs!$B$16</f>
+        <f aca="false">-B12*Inputs!$B$18</f>
         <v>-300</v>
       </c>
       <c r="C17" s="8" t="n">
-        <f aca="false">-C12*Inputs!$B$16</f>
+        <f aca="false">-C12*Inputs!$B$18</f>
         <v>-540</v>
       </c>
       <c r="D17" s="8" t="n">
-        <f aca="false">-D12*Inputs!$B$16</f>
+        <f aca="false">-D12*Inputs!$B$18</f>
         <v>-840</v>
       </c>
       <c r="E17" s="8" t="n">
-        <f aca="false">-E12*Inputs!$B$16</f>
+        <f aca="false">-E12*Inputs!$B$18</f>
         <v>-1140</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B16+B17</f>
@@ -2153,7 +2196,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-B17</f>
@@ -2174,387 +2217,408 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B20" s="8" t="n">
-        <f aca="false">B5*Inputs!$B$13*Inputs!$B$15+(B6+1)*Inputs!$B$13*Inputs!$B$14</f>
-        <v>720</v>
+        <f aca="false">B5*Inputs!$B$12*Inputs!$B$14+(B6+1)*Inputs!$B$12*Inputs!$B$13</f>
+        <v>1260</v>
       </c>
       <c r="C20" s="8" t="n">
-        <f aca="false">C5*Inputs!$B$13*Inputs!$B$15+(C6+1)*Inputs!$B$13*Inputs!$B$14</f>
-        <v>1200</v>
+        <f aca="false">C5*Inputs!$B$12*Inputs!$B$14+(C6+1)*Inputs!$B$12*Inputs!$B$13</f>
+        <v>2100</v>
       </c>
       <c r="D20" s="8" t="n">
-        <f aca="false">D5*Inputs!$B$13*Inputs!$B$15+(D6+1)*Inputs!$B$13*Inputs!$B$14</f>
-        <v>1800</v>
+        <f aca="false">D5*Inputs!$B$12*Inputs!$B$14+(D6+1)*Inputs!$B$12*Inputs!$B$13</f>
+        <v>3150</v>
       </c>
       <c r="E20" s="8" t="n">
-        <f aca="false">E5*Inputs!$B$13*Inputs!$B$15+(E6+1)*Inputs!$B$13*Inputs!$B$14</f>
-        <v>2400</v>
+        <f aca="false">E5*Inputs!$B$12*Inputs!$B$14+(E6+1)*Inputs!$B$12*Inputs!$B$13</f>
+        <v>4200</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B21" s="8" t="n">
-        <f aca="false">B5*Inputs!$B$29</f>
-        <v>1170</v>
+        <f aca="false">B5*Inputs!$B$15*Inputs!$B$17+(B6+1)*Inputs!$B$15*Inputs!$B$16</f>
+        <v>720</v>
       </c>
       <c r="C21" s="8" t="n">
-        <f aca="false">C5*Inputs!$B$29</f>
-        <v>1950</v>
+        <f aca="false">C5*Inputs!$B$15*Inputs!$B$17+(C6+1)*Inputs!$B$15*Inputs!$B$16</f>
+        <v>1200</v>
       </c>
       <c r="D21" s="8" t="n">
-        <f aca="false">D5*Inputs!$B$29</f>
-        <v>2925</v>
+        <f aca="false">D5*Inputs!$B$15*Inputs!$B$17+(D6+1)*Inputs!$B$15*Inputs!$B$16</f>
+        <v>1800</v>
       </c>
       <c r="E21" s="8" t="n">
-        <f aca="false">E5*Inputs!$B$29</f>
-        <v>3900</v>
+        <f aca="false">E5*Inputs!$B$15*Inputs!$B$17+(E6+1)*Inputs!$B$15*Inputs!$B$16</f>
+        <v>2400</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B22" s="8" t="n">
-        <f aca="false">B3*Inputs!$B$30</f>
-        <v>1428</v>
+        <f aca="false">B5*Inputs!$B$31</f>
+        <v>1170</v>
       </c>
       <c r="C22" s="8" t="n">
-        <f aca="false">C3*Inputs!$B$30</f>
-        <v>2380</v>
+        <f aca="false">C5*Inputs!$B$31</f>
+        <v>1950</v>
       </c>
       <c r="D22" s="8" t="n">
-        <f aca="false">D3*Inputs!$B$30</f>
-        <v>3570</v>
+        <f aca="false">D5*Inputs!$B$31</f>
+        <v>2925</v>
       </c>
       <c r="E22" s="8" t="n">
-        <f aca="false">E3*Inputs!$B$30</f>
-        <v>4760</v>
+        <f aca="false">E5*Inputs!$B$31</f>
+        <v>3900</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B23" s="8" t="n">
-        <f aca="false">B7*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
-        <v>2952</v>
+        <f aca="false">B3*Inputs!$B$32</f>
+        <v>1428</v>
       </c>
       <c r="C23" s="8" t="n">
-        <f aca="false">C7*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
-        <v>4920</v>
+        <f aca="false">C3*Inputs!$B$32</f>
+        <v>2380</v>
       </c>
       <c r="D23" s="8" t="n">
-        <f aca="false">D7*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
-        <v>7380</v>
+        <f aca="false">D3*Inputs!$B$32</f>
+        <v>3570</v>
       </c>
       <c r="E23" s="8" t="n">
-        <f aca="false">E7*(Inputs!$B$23*Inputs!$B$25+Inputs!$B$24*Inputs!$B$26)</f>
-        <v>9840</v>
+        <f aca="false">E3*Inputs!$B$32</f>
+        <v>4760</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>56</v>
+        <v>129</v>
       </c>
       <c r="B24" s="8" t="n">
-        <f aca="false">Inputs!$B$32</f>
+        <f aca="false">B7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
+        <v>2952</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <f aca="false">C7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
+        <v>4920</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <f aca="false">D7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
+        <v>7380</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <f aca="false">E7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
+        <v>9840</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B25" s="8" t="n">
+        <f aca="false">Inputs!$B$34</f>
         <v>700</v>
       </c>
-      <c r="C24" s="8" t="n">
-        <f aca="false">Inputs!$B$32</f>
+      <c r="C25" s="8" t="n">
+        <f aca="false">Inputs!$B$34</f>
         <v>700</v>
       </c>
-      <c r="D24" s="8" t="n">
-        <f aca="false">Inputs!$B$32</f>
+      <c r="D25" s="8" t="n">
+        <f aca="false">Inputs!$B$34</f>
         <v>700</v>
       </c>
-      <c r="E24" s="8" t="n">
-        <f aca="false">Inputs!$B$32</f>
+      <c r="E25" s="8" t="n">
+        <f aca="false">Inputs!$B$34</f>
         <v>700</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="B25" s="9" t="n">
-        <f aca="false">B18+B19+B20+B21+B22+B23+B24</f>
-        <v>13810</v>
-      </c>
-      <c r="C25" s="9" t="n">
-        <f aca="false">C18+C19+C20+C21+C22+C23+C24</f>
-        <v>22950</v>
-      </c>
-      <c r="D25" s="9" t="n">
-        <f aca="false">D18+D19+D20+D21+D22+D23+D24</f>
-        <v>33775</v>
-      </c>
-      <c r="E25" s="9" t="n">
-        <f aca="false">E18+E19+E20+E21+E22+E23+E24</f>
-        <v>44600</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
+        <v>130</v>
+      </c>
+      <c r="B26" s="9" t="n">
+        <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25</f>
+        <v>15070</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <f aca="false">C18+C19+C20+C21+C22+C23+C24+C25</f>
+        <v>25050</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <f aca="false">D18+D19+D20+D21+D22+D23+D24+D25</f>
+        <v>36925</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <f aca="false">E18+E19+E20+E21+E22+E23+E24+E25</f>
+        <v>48800</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="B27" s="9" t="n">
-        <f aca="false">B9-B25</f>
-        <v>460</v>
-      </c>
-      <c r="C27" s="9" t="n">
-        <f aca="false">C9-C25</f>
-        <v>1620</v>
-      </c>
-      <c r="D27" s="9" t="n">
-        <f aca="false">D9-D25</f>
-        <v>3670</v>
-      </c>
-      <c r="E27" s="9" t="n">
-        <f aca="false">E9-E25</f>
-        <v>5720</v>
-      </c>
+        <v>131</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="B28" s="8" t="n">
-        <f aca="false">B27/B4</f>
-        <v>41.8181818181818</v>
-      </c>
-      <c r="C28" s="8" t="n">
-        <f aca="false">C27/C4</f>
-        <v>85.2631578947368</v>
-      </c>
-      <c r="D28" s="8" t="n">
-        <f aca="false">D27/D4</f>
-        <v>126.551724137931</v>
-      </c>
-      <c r="E28" s="8" t="n">
-        <f aca="false">E27/E4</f>
-        <v>146.666666666667</v>
+      <c r="A28" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B28" s="9" t="n">
+        <f aca="false">B9-B26</f>
+        <v>445</v>
+      </c>
+      <c r="C28" s="9" t="n">
+        <f aca="false">C9-C26</f>
+        <v>1705</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <f aca="false">D9-D26</f>
+        <v>3880</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <f aca="false">E9-E26</f>
+        <v>6055</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B29" s="11" t="n">
-        <f aca="false">B27/B9</f>
-        <v>0.0322354590049054</v>
-      </c>
-      <c r="C29" s="11" t="n">
-        <f aca="false">C27/C9</f>
-        <v>0.0659340659340659</v>
-      </c>
-      <c r="D29" s="11" t="n">
-        <f aca="false">D27/D9</f>
-        <v>0.0980104152757378</v>
-      </c>
-      <c r="E29" s="11" t="n">
-        <f aca="false">E27/E9</f>
-        <v>0.113672496025437</v>
+        <v>133</v>
+      </c>
+      <c r="B29" s="8" t="n">
+        <f aca="false">B28/B4</f>
+        <v>40.4545454545455</v>
+      </c>
+      <c r="C29" s="8" t="n">
+        <f aca="false">C28/C4</f>
+        <v>89.7368421052632</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <f aca="false">D28/D4</f>
+        <v>133.793103448276</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <f aca="false">E28/E4</f>
+        <v>155.25641025641</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B30" s="12" t="str">
-        <f aca="false">IF(B27&gt;=0,"yes","NO")</f>
-        <v>yes</v>
-      </c>
-      <c r="C30" s="12" t="str">
-        <f aca="false">IF(C27&gt;=0,"yes","NO")</f>
-        <v>yes</v>
-      </c>
-      <c r="D30" s="12" t="str">
-        <f aca="false">IF(D27&gt;=0,"yes","NO")</f>
-        <v>yes</v>
-      </c>
-      <c r="E30" s="12" t="str">
-        <f aca="false">IF(E27&gt;=0,"yes","NO")</f>
-        <v>yes</v>
+      <c r="A30" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B30" s="11" t="n">
+        <f aca="false">B28/B9</f>
+        <v>0.0286819207218821</v>
+      </c>
+      <c r="C30" s="11" t="n">
+        <f aca="false">C28/C9</f>
+        <v>0.0637264062792002</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <f aca="false">D28/D9</f>
+        <v>0.095086386472246</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <f aca="false">E28/E9</f>
+        <v>0.110381915960259</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="B31" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="B31" s="12" t="str">
+        <f aca="false">IF(B28&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="C31" s="12" t="str">
+        <f aca="false">IF(C28&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="D31" s="12" t="str">
+        <f aca="false">IF(D28&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="E31" s="12" t="str">
+        <f aca="false">IF(E28&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B32" s="9" t="n">
         <f aca="false">B19</f>
         <v>300</v>
       </c>
-      <c r="C31" s="9" t="n">
+      <c r="C32" s="9" t="n">
         <f aca="false">C19</f>
         <v>540</v>
       </c>
-      <c r="D31" s="9" t="n">
+      <c r="D32" s="9" t="n">
         <f aca="false">D19</f>
         <v>840</v>
       </c>
-      <c r="E31" s="9" t="n">
+      <c r="E32" s="9" t="n">
         <f aca="false">E19</f>
         <v>1140</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-    </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B33" s="8" t="n">
+      <c r="A33" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B34" s="8" t="n">
         <f aca="false">B4*400</f>
         <v>4400</v>
       </c>
-      <c r="C33" s="8" t="n">
+      <c r="C34" s="8" t="n">
         <f aca="false">C4*400</f>
         <v>7600</v>
       </c>
-      <c r="D33" s="8" t="n">
+      <c r="D34" s="8" t="n">
         <f aca="false">D4*400</f>
         <v>11600</v>
       </c>
-      <c r="E33" s="8" t="n">
+      <c r="E34" s="8" t="n">
         <f aca="false">E4*400</f>
         <v>15600</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B34" s="8" t="n">
-        <f aca="false">B16*Inputs!$B$18+B23*Inputs!$B$27</f>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B35" s="8" t="n">
+        <f aca="false">B16*Inputs!$B$20+B24*Inputs!$B$29</f>
         <v>2448</v>
       </c>
-      <c r="C34" s="8" t="n">
-        <f aca="false">C16*Inputs!$B$18+C23*Inputs!$B$27</f>
+      <c r="C35" s="8" t="n">
+        <f aca="false">C16*Inputs!$B$20+C24*Inputs!$B$29</f>
         <v>4180</v>
       </c>
-      <c r="D34" s="8" t="n">
-        <f aca="false">D16*Inputs!$B$18+D23*Inputs!$B$27</f>
+      <c r="D35" s="8" t="n">
+        <f aca="false">D16*Inputs!$B$20+D24*Inputs!$B$29</f>
         <v>6195</v>
       </c>
-      <c r="E34" s="8" t="n">
-        <f aca="false">E16*Inputs!$B$18+E23*Inputs!$B$27</f>
+      <c r="E35" s="8" t="n">
+        <f aca="false">E16*Inputs!$B$20+E24*Inputs!$B$29</f>
         <v>8210</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="B35" s="9" t="n">
-        <f aca="false">B33-B34</f>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B36" s="9" t="n">
+        <f aca="false">B34-B35</f>
         <v>1952</v>
       </c>
-      <c r="C35" s="9" t="n">
-        <f aca="false">C33-C34</f>
+      <c r="C36" s="9" t="n">
+        <f aca="false">C34-C35</f>
         <v>3420</v>
       </c>
-      <c r="D35" s="9" t="n">
-        <f aca="false">D33-D34</f>
+      <c r="D36" s="9" t="n">
+        <f aca="false">D34-D35</f>
         <v>5405</v>
       </c>
-      <c r="E35" s="9" t="n">
-        <f aca="false">E33-E34</f>
+      <c r="E36" s="9" t="n">
+        <f aca="false">E34-E35</f>
         <v>7390</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B36" s="8" t="n">
-        <f aca="false">B9-B33</f>
-        <v>9870</v>
-      </c>
-      <c r="C36" s="8" t="n">
-        <f aca="false">C9-C33</f>
-        <v>16970</v>
-      </c>
-      <c r="D36" s="8" t="n">
-        <f aca="false">D9-D33</f>
-        <v>25845</v>
-      </c>
-      <c r="E36" s="8" t="n">
-        <f aca="false">E9-E33</f>
-        <v>34720</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B37" s="8" t="n">
-        <f aca="false">B18-B16*Inputs!$B$18+B23*(1-Inputs!$B$27)+B21+B22</f>
-        <v>9642</v>
+        <f aca="false">B9-B34</f>
+        <v>11115</v>
       </c>
       <c r="C37" s="8" t="n">
-        <f aca="false">C18-C16*Inputs!$B$18+C23*(1-Inputs!$B$27)+C21+C22</f>
-        <v>16330</v>
+        <f aca="false">C9-C34</f>
+        <v>19155</v>
       </c>
       <c r="D37" s="8" t="n">
-        <f aca="false">D18-D16*Inputs!$B$18+D23*(1-Inputs!$B$27)+D21+D22</f>
-        <v>24240</v>
+        <f aca="false">D9-D34</f>
+        <v>29205</v>
       </c>
       <c r="E37" s="8" t="n">
-        <f aca="false">E18-E16*Inputs!$B$18+E23*(1-Inputs!$B$27)+E21+E22</f>
-        <v>32150</v>
+        <f aca="false">E9-E34</f>
+        <v>39255</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B38" s="8" t="n">
-        <f aca="false">B20</f>
+        <f aca="false">B18-B16*Inputs!$B$20+B20+B24*(1-Inputs!$B$29)+B22+B23</f>
+        <v>10902</v>
+      </c>
+      <c r="C38" s="8" t="n">
+        <f aca="false">C18-C16*Inputs!$B$20+C20+C24*(1-Inputs!$B$29)+C22+C23</f>
+        <v>18430</v>
+      </c>
+      <c r="D38" s="8" t="n">
+        <f aca="false">D18-D16*Inputs!$B$20+D20+D24*(1-Inputs!$B$29)+D22+D23</f>
+        <v>27390</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <f aca="false">E18-E16*Inputs!$B$20+E20+E24*(1-Inputs!$B$29)+E22+E23</f>
+        <v>36350</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B39" s="8" t="n">
+        <f aca="false">B21</f>
         <v>720</v>
       </c>
-      <c r="C38" s="8" t="n">
-        <f aca="false">C20</f>
+      <c r="C39" s="8" t="n">
+        <f aca="false">C21</f>
         <v>1200</v>
       </c>
-      <c r="D38" s="8" t="n">
-        <f aca="false">D20</f>
+      <c r="D39" s="8" t="n">
+        <f aca="false">D21</f>
         <v>1800</v>
       </c>
-      <c r="E38" s="8" t="n">
-        <f aca="false">E20</f>
+      <c r="E39" s="8" t="n">
+        <f aca="false">E21</f>
         <v>2400</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
+    <row r="40" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2582,108 +2646,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2693,10 +2757,10 @@
     </row>
     <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>10</v>
@@ -2704,10 +2768,10 @@
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Budget: USD 200 tax buffer per head; hotel rate per room assumed; payment fees ignored
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="177">
   <si>
     <t xml:space="preserve">Cozumel group budget — inputs (blue cells are editable)</t>
   </si>
@@ -199,6 +199,12 @@
     <t xml:space="preserve">DAN membership + Preferred plan, bought for each person</t>
   </si>
   <si>
+    <t xml:space="preserve">Tax buffer per head (Mexican IVA and lodging tax if the quotes are pre-tax)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">policy (George, 23 Sep): assume USD 200 until Doug confirms</t>
+  </si>
+  <si>
     <t xml:space="preserve">Leader costs carried by the group (George shares a room like everyone)</t>
   </si>
   <si>
@@ -274,6 +280,9 @@
     <t xml:space="preserve">Marine park fees</t>
   </si>
   <si>
+    <t xml:space="preserve">Tax buffer (IVA and lodging tax, if the quotes are pre-tax)</t>
+  </si>
+  <si>
     <t xml:space="preserve">PADI eLearning</t>
   </si>
   <si>
@@ -401,6 +410,9 @@
   </si>
   <si>
     <t xml:space="preserve">Gear rental for everyone including George</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tax buffer held (paid to Blue Note and the hotel if charged; otherwise refunded)</t>
   </si>
   <si>
     <t xml:space="preserve">Marine park fees (cash on the island, paid from the float)</t>
@@ -953,7 +965,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72"/>
@@ -1378,34 +1390,33 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
+      <c r="B33" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B34" s="7" t="n">
-        <v>700</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D34" s="2" t="s">
+      <c r="A34" s="4" t="s">
         <v>60</v>
       </c>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
         <v>61</v>
       </c>
       <c r="B35" s="7" t="n">
-        <f aca="false">(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2</f>
-        <v>246</v>
+        <v>700</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>17</v>
@@ -1419,7 +1430,7 @@
         <v>63</v>
       </c>
       <c r="B36" s="7" t="n">
-        <f aca="false">Inputs!$B$35</f>
+        <f aca="false">(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2</f>
         <v>246</v>
       </c>
       <c r="C36" s="2" t="s">
@@ -1434,84 +1445,85 @@
         <v>65</v>
       </c>
       <c r="B37" s="7" t="n">
-        <v>119</v>
+        <f aca="false">Inputs!$B$36</f>
+        <v>246</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B38" s="7" t="n">
+        <v>119</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B39" s="7" t="n">
         <f aca="false">Inputs!$B$12*5</f>
         <v>150</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C39" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
+      <c r="D39" s="2" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B40" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D40" s="2" t="s">
+      <c r="A40" s="4" t="s">
         <v>69</v>
       </c>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B41" s="5" t="n">
-        <v>6</v>
+      <c r="B41" s="7" t="n">
+        <v>45</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D41" s="2"/>
+        <v>22</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B42" s="7" t="n">
-        <v>50</v>
+        <v>72</v>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>72</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="D42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B43" s="7" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>17</v>
@@ -1525,13 +1537,27 @@
         <v>75</v>
       </c>
       <c r="B44" s="7" t="n">
-        <v>220</v>
+        <v>30</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>76</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B45" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1550,7 +1576,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -1559,7 +1585,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1567,15 +1593,15 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">Inputs!$B$9+Inputs!$B$10</f>
@@ -1588,7 +1614,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">Inputs!$B$12*Inputs!$B$14</f>
@@ -1601,7 +1627,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">Inputs!$B$15*Inputs!$B$17</f>
@@ -1614,230 +1640,243 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B6" s="8" t="n">
+        <f aca="false">Inputs!$B$33</f>
+        <v>200</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <f aca="false">Inputs!$B$33</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="8" t="n">
         <f aca="false">Inputs!$B$31</f>
         <v>195</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B7" s="8" t="n">
+      <c r="C7" s="8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="8" t="n">
         <f aca="false">Inputs!$B$32</f>
         <v>119</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C8" s="8" t="n">
         <f aca="false">Inputs!$B$32</f>
         <v>119</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B8" s="8" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="8" t="n">
         <f aca="false">((Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2)</f>
         <v>246</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C9" s="8" t="n">
         <f aca="false">((Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2)</f>
         <v>246</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B9" s="8" t="n">
-        <f aca="false">(Inputs!$B$34+Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38)/(Inputs!$B$4-1)</f>
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <f aca="false">(Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39)/(Inputs!$B$4-1)</f>
         <v>76.8947368421053</v>
       </c>
-      <c r="C9" s="8" t="n">
-        <f aca="false">(Inputs!$B$34+Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38)/(Inputs!$B$4-1)</f>
+      <c r="C10" s="8" t="n">
+        <f aca="false">(Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39)/(Inputs!$B$4-1)</f>
         <v>76.8947368421053</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="9" t="n">
+        <f aca="false">SUM(B3:B10)</f>
+        <v>1581.89473684211</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <f aca="false">SUM(C3:C10)</f>
+        <v>1466.89473684211</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <f aca="false">ROUND(B11*Inputs!$B$7,0)</f>
+        <v>95</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <f aca="false">ROUND(C11*Inputs!$B$7,0)</f>
         <v>88</v>
       </c>
-      <c r="B10" s="9" t="n">
-        <f aca="false">SUM(B3:B9)</f>
-        <v>1381.89473684211</v>
-      </c>
-      <c r="C10" s="9" t="n">
-        <f aca="false">SUM(C3:C9)</f>
-        <v>1266.89473684211</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B11" s="8" t="n">
-        <f aca="false">ROUND(B10*Inputs!$B$7,0)</f>
-        <v>83</v>
-      </c>
-      <c r="C11" s="8" t="n">
-        <f aca="false">ROUND(C10*Inputs!$B$7,0)</f>
-        <v>76</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B12" s="9" t="n">
-        <f aca="false">CEILING(B10+B11,5)</f>
-        <v>1465</v>
-      </c>
-      <c r="C12" s="9" t="n">
-        <f aca="false">CEILING(C10+C11,5)</f>
-        <v>1345</v>
-      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
+      <c r="A13" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="9" t="n">
+        <f aca="false">CEILING(B11+B12,5)</f>
+        <v>1680</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <f aca="false">CEILING(C11+C12,5)</f>
+        <v>1555</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>91</v>
-      </c>
+      <c r="A14" s="2"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="C15" s="8" t="n">
-        <f aca="false">Inputs!$B$44</f>
-        <v>220</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C16" s="8" t="n">
+        <f aca="false">Inputs!$B$45</f>
+        <v>220</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C17" s="8" t="n">
         <f aca="false">Inputs!$B$23*10</f>
         <v>120</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B17" s="8" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" s="8" t="n">
         <f aca="false">Inputs!$B$21+Inputs!$B$15</f>
         <v>145</v>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C18" s="8" t="n">
         <f aca="false">Inputs!$B$21+Inputs!$B$15</f>
         <v>145</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B18" s="8" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B19" s="8" t="n">
         <f aca="false">Inputs!$B$22/10</f>
         <v>80</v>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C19" s="8" t="n">
         <f aca="false">Inputs!$B$22/10</f>
         <v>80</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-    </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
+      <c r="A20" s="2"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B21" s="8" t="n">
-        <f aca="false">B12</f>
-        <v>1465</v>
-      </c>
-      <c r="C21" s="8" t="n">
-        <f aca="false">C12</f>
-        <v>1345</v>
-      </c>
+      <c r="A21" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B22" s="8" t="n">
-        <f aca="false">Inputs!$B$40*Inputs!$B$41+Inputs!$B$42+Inputs!$B$43</f>
+        <f aca="false">B13</f>
+        <v>1680</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <f aca="false">C13</f>
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B23" s="8" t="n">
+        <f aca="false">Inputs!$B$41*Inputs!$B$42+Inputs!$B$43+Inputs!$B$44</f>
         <v>350</v>
       </c>
-      <c r="C22" s="8" t="n">
-        <f aca="false">Inputs!$B$40*Inputs!$B$41+Inputs!$B$42+Inputs!$B$43</f>
+      <c r="C23" s="8" t="n">
+        <f aca="false">Inputs!$B$41*Inputs!$B$42+Inputs!$B$43+Inputs!$B$44</f>
         <v>350</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B23" s="9" t="n">
-        <f aca="false">B21+B22</f>
-        <v>1815</v>
-      </c>
-      <c r="C23" s="9" t="n">
-        <f aca="false">C21+C22</f>
-        <v>1695</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>93</v>
+        <v>103</v>
+      </c>
+      <c r="B24" s="9" t="n">
+        <f aca="false">B22+B23</f>
+        <v>2030</v>
       </c>
       <c r="C24" s="9" t="n">
-        <f aca="false">C23+C15+C16</f>
-        <v>2035</v>
+        <f aca="false">C22+C23</f>
+        <v>1905</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-    </row>
-    <row r="26" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>102</v>
-      </c>
+      <c r="A25" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25" s="9" t="n">
+        <f aca="false">C24+C16+C17</f>
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
+    </row>
+    <row r="27" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1855,7 +1894,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="66"/>
@@ -1864,7 +1903,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1874,21 +1913,21 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>12</v>
@@ -1905,7 +1944,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
@@ -1926,7 +1965,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$6,0)</f>
@@ -1947,7 +1986,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">B4-B5</f>
@@ -1968,7 +2007,7 @@
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">ROUNDUP(B3/2,0)</f>
@@ -1989,7 +2028,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1998,28 +2037,28 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B9" s="9" t="n">
-        <f aca="false">B5*Fee!$B$12+B6*Fee!$C$12</f>
-        <v>15515</v>
+        <f aca="false">B5*Fee!$B$13+B6*Fee!$C$13</f>
+        <v>17855</v>
       </c>
       <c r="C9" s="9" t="n">
-        <f aca="false">C5*Fee!$B$12+C6*Fee!$C$12</f>
-        <v>26755</v>
+        <f aca="false">C5*Fee!$B$13+C6*Fee!$C$13</f>
+        <v>30795</v>
       </c>
       <c r="D9" s="9" t="n">
-        <f aca="false">D5*Fee!$B$12+D6*Fee!$C$12</f>
-        <v>40805</v>
+        <f aca="false">D5*Fee!$B$13+D6*Fee!$C$13</f>
+        <v>46970</v>
       </c>
       <c r="E9" s="9" t="n">
-        <f aca="false">E5*Fee!$B$12+E6*Fee!$C$12</f>
-        <v>54855</v>
+        <f aca="false">E5*Fee!$B$13+E6*Fee!$C$13</f>
+        <v>63145</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2028,7 +2067,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$9+Inputs!$B$10)</f>
@@ -2049,7 +2088,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B6*Inputs!$B$11</f>
@@ -2070,7 +2109,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">INT(B6/Inputs!$B$19)</f>
@@ -2091,7 +2130,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">IF(B13&gt;=1,0,Inputs!$B$11)</f>
@@ -2112,7 +2151,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">-MAX(B13-1,0)*Inputs!$B$11</f>
@@ -2133,7 +2172,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B11+B12+B14+B15</f>
@@ -2154,7 +2193,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">-B12*Inputs!$B$18</f>
@@ -2175,7 +2214,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B16+B17</f>
@@ -2196,7 +2235,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-B17</f>
@@ -2217,7 +2256,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B5*Inputs!$B$12*Inputs!$B$14+(B6+1)*Inputs!$B$12*Inputs!$B$13</f>
@@ -2236,389 +2275,410 @@
         <v>4200</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B21" s="8" t="n">
+        <f aca="false">B3*Inputs!$B$33</f>
+        <v>2400</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <f aca="false">C3*Inputs!$B$33</f>
+        <v>4000</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <f aca="false">D3*Inputs!$B$33</f>
+        <v>6000</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <f aca="false">E3*Inputs!$B$33</f>
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B22" s="8" t="n">
         <f aca="false">B5*Inputs!$B$15*Inputs!$B$17+(B6+1)*Inputs!$B$15*Inputs!$B$16</f>
         <v>720</v>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C22" s="8" t="n">
         <f aca="false">C5*Inputs!$B$15*Inputs!$B$17+(C6+1)*Inputs!$B$15*Inputs!$B$16</f>
         <v>1200</v>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="D22" s="8" t="n">
         <f aca="false">D5*Inputs!$B$15*Inputs!$B$17+(D6+1)*Inputs!$B$15*Inputs!$B$16</f>
         <v>1800</v>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E22" s="8" t="n">
         <f aca="false">E5*Inputs!$B$15*Inputs!$B$17+(E6+1)*Inputs!$B$15*Inputs!$B$16</f>
         <v>2400</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="B22" s="8" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" s="8" t="n">
         <f aca="false">B5*Inputs!$B$31</f>
         <v>1170</v>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C23" s="8" t="n">
         <f aca="false">C5*Inputs!$B$31</f>
         <v>1950</v>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D23" s="8" t="n">
         <f aca="false">D5*Inputs!$B$31</f>
         <v>2925</v>
       </c>
-      <c r="E22" s="8" t="n">
+      <c r="E23" s="8" t="n">
         <f aca="false">E5*Inputs!$B$31</f>
         <v>3900</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B23" s="8" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B24" s="8" t="n">
         <f aca="false">B3*Inputs!$B$32</f>
         <v>1428</v>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C24" s="8" t="n">
         <f aca="false">C3*Inputs!$B$32</f>
         <v>2380</v>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D24" s="8" t="n">
         <f aca="false">D3*Inputs!$B$32</f>
         <v>3570</v>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="E24" s="8" t="n">
         <f aca="false">E3*Inputs!$B$32</f>
         <v>4760</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="B24" s="8" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B25" s="8" t="n">
         <f aca="false">B7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
         <v>2952</v>
       </c>
-      <c r="C24" s="8" t="n">
+      <c r="C25" s="8" t="n">
         <f aca="false">C7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
         <v>4920</v>
       </c>
-      <c r="D24" s="8" t="n">
+      <c r="D25" s="8" t="n">
         <f aca="false">D7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
         <v>7380</v>
       </c>
-      <c r="E24" s="8" t="n">
+      <c r="E25" s="8" t="n">
         <f aca="false">E7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
         <v>9840</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B25" s="8" t="n">
-        <f aca="false">Inputs!$B$34</f>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" s="8" t="n">
+        <f aca="false">Inputs!$B$35</f>
         <v>700</v>
       </c>
-      <c r="C25" s="8" t="n">
-        <f aca="false">Inputs!$B$34</f>
+      <c r="C26" s="8" t="n">
+        <f aca="false">Inputs!$B$35</f>
         <v>700</v>
       </c>
-      <c r="D25" s="8" t="n">
-        <f aca="false">Inputs!$B$34</f>
+      <c r="D26" s="8" t="n">
+        <f aca="false">Inputs!$B$35</f>
         <v>700</v>
       </c>
-      <c r="E25" s="8" t="n">
-        <f aca="false">Inputs!$B$34</f>
+      <c r="E26" s="8" t="n">
+        <f aca="false">Inputs!$B$35</f>
         <v>700</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="B26" s="9" t="n">
-        <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25</f>
-        <v>15070</v>
-      </c>
-      <c r="C26" s="9" t="n">
-        <f aca="false">C18+C19+C20+C21+C22+C23+C24+C25</f>
-        <v>25050</v>
-      </c>
-      <c r="D26" s="9" t="n">
-        <f aca="false">D18+D19+D20+D21+D22+D23+D24+D25</f>
-        <v>36925</v>
-      </c>
-      <c r="E26" s="9" t="n">
-        <f aca="false">E18+E19+E20+E21+E22+E23+E24+E25</f>
-        <v>48800</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
+        <v>134</v>
+      </c>
+      <c r="B27" s="9" t="n">
+        <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25+B26</f>
+        <v>17470</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <f aca="false">C18+C19+C20+C21+C22+C23+C24+C25+C26</f>
+        <v>29050</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <f aca="false">D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
+        <v>42925</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <f aca="false">E18+E19+E20+E21+E22+E23+E24+E25+E26</f>
+        <v>56800</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="B28" s="9" t="n">
-        <f aca="false">B9-B26</f>
-        <v>445</v>
-      </c>
-      <c r="C28" s="9" t="n">
-        <f aca="false">C9-C26</f>
-        <v>1705</v>
-      </c>
-      <c r="D28" s="9" t="n">
-        <f aca="false">D9-D26</f>
-        <v>3880</v>
-      </c>
-      <c r="E28" s="9" t="n">
-        <f aca="false">E9-E26</f>
-        <v>6055</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="B29" s="8" t="n">
-        <f aca="false">B28/B4</f>
-        <v>40.4545454545455</v>
-      </c>
-      <c r="C29" s="8" t="n">
-        <f aca="false">C28/C4</f>
-        <v>89.7368421052632</v>
-      </c>
-      <c r="D29" s="8" t="n">
-        <f aca="false">D28/D4</f>
-        <v>133.793103448276</v>
-      </c>
-      <c r="E29" s="8" t="n">
-        <f aca="false">E28/E4</f>
-        <v>155.25641025641</v>
+      <c r="A29" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B29" s="9" t="n">
+        <f aca="false">B9-B27</f>
+        <v>385</v>
+      </c>
+      <c r="C29" s="9" t="n">
+        <f aca="false">C9-C27</f>
+        <v>1745</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <f aca="false">D9-D27</f>
+        <v>4045</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <f aca="false">E9-E27</f>
+        <v>6345</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B30" s="11" t="n">
-        <f aca="false">B28/B9</f>
-        <v>0.0286819207218821</v>
-      </c>
-      <c r="C30" s="11" t="n">
-        <f aca="false">C28/C9</f>
-        <v>0.0637264062792002</v>
-      </c>
-      <c r="D30" s="11" t="n">
-        <f aca="false">D28/D9</f>
-        <v>0.095086386472246</v>
-      </c>
-      <c r="E30" s="11" t="n">
-        <f aca="false">E28/E9</f>
-        <v>0.110381915960259</v>
+        <v>137</v>
+      </c>
+      <c r="B30" s="8" t="n">
+        <f aca="false">B29/B4</f>
+        <v>35</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <f aca="false">C29/C4</f>
+        <v>91.8421052631579</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <f aca="false">D29/D4</f>
+        <v>139.48275862069</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <f aca="false">E29/E4</f>
+        <v>162.692307692308</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="B31" s="12" t="str">
-        <f aca="false">IF(B28&gt;=0,"yes","NO")</f>
-        <v>yes</v>
-      </c>
-      <c r="C31" s="12" t="str">
-        <f aca="false">IF(C28&gt;=0,"yes","NO")</f>
-        <v>yes</v>
-      </c>
-      <c r="D31" s="12" t="str">
-        <f aca="false">IF(D28&gt;=0,"yes","NO")</f>
-        <v>yes</v>
-      </c>
-      <c r="E31" s="12" t="str">
-        <f aca="false">IF(E28&gt;=0,"yes","NO")</f>
-        <v>yes</v>
+      <c r="A31" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B31" s="11" t="n">
+        <f aca="false">B29/B9</f>
+        <v>0.0215625875105013</v>
+      </c>
+      <c r="C31" s="11" t="n">
+        <f aca="false">C29/C9</f>
+        <v>0.0566650430264653</v>
+      </c>
+      <c r="D31" s="11" t="n">
+        <f aca="false">D29/D9</f>
+        <v>0.0861187992335533</v>
+      </c>
+      <c r="E31" s="11" t="n">
+        <f aca="false">E29/E9</f>
+        <v>0.100483015282287</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="B32" s="9" t="n">
+        <v>139</v>
+      </c>
+      <c r="B32" s="12" t="str">
+        <f aca="false">IF(B29&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="C32" s="12" t="str">
+        <f aca="false">IF(C29&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="D32" s="12" t="str">
+        <f aca="false">IF(D29&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="E32" s="12" t="str">
+        <f aca="false">IF(E29&gt;=0,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B33" s="9" t="n">
         <f aca="false">B19</f>
         <v>300</v>
       </c>
-      <c r="C32" s="9" t="n">
+      <c r="C33" s="9" t="n">
         <f aca="false">C19</f>
         <v>540</v>
       </c>
-      <c r="D32" s="9" t="n">
+      <c r="D33" s="9" t="n">
         <f aca="false">D19</f>
         <v>840</v>
       </c>
-      <c r="E32" s="9" t="n">
+      <c r="E33" s="9" t="n">
         <f aca="false">E19</f>
         <v>1140</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-    </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B34" s="8" t="n">
+      <c r="A34" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B35" s="8" t="n">
         <f aca="false">B4*400</f>
         <v>4400</v>
       </c>
-      <c r="C34" s="8" t="n">
+      <c r="C35" s="8" t="n">
         <f aca="false">C4*400</f>
         <v>7600</v>
       </c>
-      <c r="D34" s="8" t="n">
+      <c r="D35" s="8" t="n">
         <f aca="false">D4*400</f>
         <v>11600</v>
       </c>
-      <c r="E34" s="8" t="n">
+      <c r="E35" s="8" t="n">
         <f aca="false">E4*400</f>
         <v>15600</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B35" s="8" t="n">
-        <f aca="false">B16*Inputs!$B$20+B24*Inputs!$B$29</f>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B36" s="8" t="n">
+        <f aca="false">B16*Inputs!$B$20+B25*Inputs!$B$29</f>
         <v>2448</v>
       </c>
-      <c r="C35" s="8" t="n">
-        <f aca="false">C16*Inputs!$B$20+C24*Inputs!$B$29</f>
+      <c r="C36" s="8" t="n">
+        <f aca="false">C16*Inputs!$B$20+C25*Inputs!$B$29</f>
         <v>4180</v>
       </c>
-      <c r="D35" s="8" t="n">
-        <f aca="false">D16*Inputs!$B$20+D24*Inputs!$B$29</f>
+      <c r="D36" s="8" t="n">
+        <f aca="false">D16*Inputs!$B$20+D25*Inputs!$B$29</f>
         <v>6195</v>
       </c>
-      <c r="E35" s="8" t="n">
-        <f aca="false">E16*Inputs!$B$20+E24*Inputs!$B$29</f>
+      <c r="E36" s="8" t="n">
+        <f aca="false">E16*Inputs!$B$20+E25*Inputs!$B$29</f>
         <v>8210</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B36" s="9" t="n">
-        <f aca="false">B34-B35</f>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B37" s="9" t="n">
+        <f aca="false">B35-B36</f>
         <v>1952</v>
       </c>
-      <c r="C36" s="9" t="n">
-        <f aca="false">C34-C35</f>
+      <c r="C37" s="9" t="n">
+        <f aca="false">C35-C36</f>
         <v>3420</v>
       </c>
-      <c r="D36" s="9" t="n">
-        <f aca="false">D34-D35</f>
+      <c r="D37" s="9" t="n">
+        <f aca="false">D35-D36</f>
         <v>5405</v>
       </c>
-      <c r="E36" s="9" t="n">
-        <f aca="false">E34-E35</f>
+      <c r="E37" s="9" t="n">
+        <f aca="false">E35-E36</f>
         <v>7390</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B37" s="8" t="n">
-        <f aca="false">B9-B34</f>
-        <v>11115</v>
-      </c>
-      <c r="C37" s="8" t="n">
-        <f aca="false">C9-C34</f>
-        <v>19155</v>
-      </c>
-      <c r="D37" s="8" t="n">
-        <f aca="false">D9-D34</f>
-        <v>29205</v>
-      </c>
-      <c r="E37" s="8" t="n">
-        <f aca="false">E9-E34</f>
-        <v>39255</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B38" s="8" t="n">
-        <f aca="false">B18-B16*Inputs!$B$20+B20+B24*(1-Inputs!$B$29)+B22+B23</f>
-        <v>10902</v>
+        <f aca="false">B9-B35</f>
+        <v>13455</v>
       </c>
       <c r="C38" s="8" t="n">
-        <f aca="false">C18-C16*Inputs!$B$20+C20+C24*(1-Inputs!$B$29)+C22+C23</f>
-        <v>18430</v>
+        <f aca="false">C9-C35</f>
+        <v>23195</v>
       </c>
       <c r="D38" s="8" t="n">
-        <f aca="false">D18-D16*Inputs!$B$20+D20+D24*(1-Inputs!$B$29)+D22+D23</f>
-        <v>27390</v>
+        <f aca="false">D9-D35</f>
+        <v>35370</v>
       </c>
       <c r="E38" s="8" t="n">
-        <f aca="false">E18-E16*Inputs!$B$20+E20+E24*(1-Inputs!$B$29)+E22+E23</f>
-        <v>36350</v>
+        <f aca="false">E9-E35</f>
+        <v>47545</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B39" s="8" t="n">
-        <f aca="false">B21</f>
+        <f aca="false">B18-B16*Inputs!$B$20+B20+B25*(1-Inputs!$B$29)+B23+B24</f>
+        <v>10902</v>
+      </c>
+      <c r="C39" s="8" t="n">
+        <f aca="false">C18-C16*Inputs!$B$20+C20+C25*(1-Inputs!$B$29)+C23+C24</f>
+        <v>18430</v>
+      </c>
+      <c r="D39" s="8" t="n">
+        <f aca="false">D18-D16*Inputs!$B$20+D20+D25*(1-Inputs!$B$29)+D23+D24</f>
+        <v>27390</v>
+      </c>
+      <c r="E39" s="8" t="n">
+        <f aca="false">E18-E16*Inputs!$B$20+E20+E25*(1-Inputs!$B$29)+E23+E24</f>
+        <v>36350</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B40" s="8" t="n">
+        <f aca="false">B22</f>
         <v>720</v>
       </c>
-      <c r="C39" s="8" t="n">
-        <f aca="false">C21</f>
+      <c r="C40" s="8" t="n">
+        <f aca="false">C22</f>
         <v>1200</v>
       </c>
-      <c r="D39" s="8" t="n">
-        <f aca="false">D21</f>
+      <c r="D40" s="8" t="n">
+        <f aca="false">D22</f>
         <v>1800</v>
       </c>
-      <c r="E39" s="8" t="n">
-        <f aca="false">E21</f>
+      <c r="E40" s="8" t="n">
+        <f aca="false">E22</f>
         <v>2400</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
+    <row r="41" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2646,108 +2706,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2757,10 +2817,10 @@
     </row>
     <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>10</v>
@@ -2768,10 +2828,10 @@
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Decisions log and trip template; fee rounds to the posted hundreds
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -304,7 +304,7 @@
     <t xml:space="preserve">Contingency</t>
   </si>
   <si>
-    <t xml:space="preserve">TRIP FEE (rounded up to the nearest 5)</t>
+    <t xml:space="preserve">TRIP FEE (rounded up to the nearest 100, as posted)</t>
   </si>
   <si>
     <t xml:space="preserve">Optional add-ons at sign-up, charged at cost</t>
@@ -1733,12 +1733,12 @@
         <v>93</v>
       </c>
       <c r="B13" s="9" t="n">
-        <f aca="false">CEILING(B11+B12,5)</f>
-        <v>1680</v>
+        <f aca="false">CEILING(B11+B12,100)</f>
+        <v>1700</v>
       </c>
       <c r="C13" s="9" t="n">
-        <f aca="false">CEILING(C11+C12,5)</f>
-        <v>1555</v>
+        <f aca="false">CEILING(C11+C12,100)</f>
+        <v>1600</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1821,11 +1821,11 @@
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B13</f>
-        <v>1680</v>
+        <v>1700</v>
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">C13</f>
-        <v>1555</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1847,11 +1847,11 @@
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">B22+B23</f>
-        <v>2030</v>
+        <v>2050</v>
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">C22+C23</f>
-        <v>1905</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="C25" s="9" t="n">
         <f aca="false">C24+C16+C17</f>
-        <v>2245</v>
+        <v>2290</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2041,19 +2041,19 @@
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">B5*Fee!$B$13+B6*Fee!$C$13</f>
-        <v>17855</v>
+        <v>18200</v>
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">C5*Fee!$B$13+C6*Fee!$C$13</f>
-        <v>30795</v>
+        <v>31400</v>
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">D5*Fee!$B$13+D6*Fee!$C$13</f>
-        <v>46970</v>
+        <v>47900</v>
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">E5*Fee!$B$13+E6*Fee!$C$13</f>
-        <v>63145</v>
+        <v>64400</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2437,19 +2437,19 @@
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">B9-B27</f>
-        <v>385</v>
+        <v>730</v>
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">C9-C27</f>
-        <v>1745</v>
+        <v>2350</v>
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">D9-D27</f>
-        <v>4045</v>
+        <v>4975</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">E9-E27</f>
-        <v>6345</v>
+        <v>7600</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2458,19 +2458,19 @@
       </c>
       <c r="B30" s="8" t="n">
         <f aca="false">B29/B4</f>
-        <v>35</v>
+        <v>66.3636363636364</v>
       </c>
       <c r="C30" s="8" t="n">
         <f aca="false">C29/C4</f>
-        <v>91.8421052631579</v>
+        <v>123.684210526316</v>
       </c>
       <c r="D30" s="8" t="n">
         <f aca="false">D29/D4</f>
-        <v>139.48275862069</v>
+        <v>171.551724137931</v>
       </c>
       <c r="E30" s="8" t="n">
         <f aca="false">E29/E4</f>
-        <v>162.692307692308</v>
+        <v>194.871794871795</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2479,19 +2479,19 @@
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">B29/B9</f>
-        <v>0.0215625875105013</v>
+        <v>0.0401098901098901</v>
       </c>
       <c r="C31" s="11" t="n">
         <f aca="false">C29/C9</f>
-        <v>0.0566650430264653</v>
+        <v>0.0748407643312102</v>
       </c>
       <c r="D31" s="11" t="n">
         <f aca="false">D29/D9</f>
-        <v>0.0861187992335533</v>
+        <v>0.103862212943633</v>
       </c>
       <c r="E31" s="11" t="n">
         <f aca="false">E29/E9</f>
-        <v>0.100483015282287</v>
+        <v>0.118012422360248</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2614,19 +2614,19 @@
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">B9-B35</f>
-        <v>13455</v>
+        <v>13800</v>
       </c>
       <c r="C38" s="8" t="n">
         <f aca="false">C9-C35</f>
-        <v>23195</v>
+        <v>23800</v>
       </c>
       <c r="D38" s="8" t="n">
         <f aca="false">D9-D35</f>
-        <v>35370</v>
+        <v>36300</v>
       </c>
       <c r="E38" s="8" t="n">
         <f aca="false">E9-E35</f>
-        <v>47545</v>
+        <v>48800</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Cozumel: Blue Note answers (4:1, park on site, min 10), two-week date lock accepted with hold to 12 Oct; Aldora and Sand Dollar replies filed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -112,7 +112,7 @@
     <t xml:space="preserve">Marine park fee per boat day</t>
   </si>
   <si>
-    <t xml:space="preserve">ADVERTISED; whether it is inside the package is asked</t>
+    <t xml:space="preserve">ADVERTISED rate; QUOTED 23 Sep: paid on site for boat days only, none on the two training-site days</t>
   </si>
   <si>
     <t xml:space="preserve">Boat days, certified</t>
@@ -1151,7 +1151,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
Cozumel budget: DAN and tax buffer out of the fee, posted fees 1,400 / 1,300; hotel tiers to 40 asked; decisions logged
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="181">
   <si>
     <t xml:space="preserve">Cozumel group budget — inputs (blue cells are editable)</t>
   </si>
@@ -196,13 +196,16 @@
     <t xml:space="preserve">ADVERTISED</t>
   </si>
   <si>
-    <t xml:space="preserve">DAN membership + Preferred plan, bought for each person</t>
+    <t xml:space="preserve">DAN cover inside the fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George 24 Sep: not in the fee; each diver buys their own dive-accident cover (see own spending)</t>
   </si>
   <si>
     <t xml:space="preserve">Tax buffer per head (Mexican IVA and lodging tax if the quotes are pre-tax)</t>
   </si>
   <si>
-    <t xml:space="preserve">policy (George, 23 Sep): assume USD 200 until Doug confirms</t>
+    <t xml:space="preserve">George 24 Sep: cut; the other three shops quoted tax-inclusive; Doug asked to confirm</t>
   </si>
   <si>
     <t xml:space="preserve">Leader costs carried by the group (George shares a room like everyone)</t>
@@ -226,7 +229,10 @@
     <t xml:space="preserve">formula: half a room</t>
   </si>
   <si>
-    <t xml:space="preserve">George's DAN cover</t>
+    <t xml:space="preserve">George's DAN cover carried by the group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George 24 Sep: own cost like everyone</t>
   </si>
   <si>
     <t xml:space="preserve">George's gear rental, 5 days</t>
@@ -256,6 +262,12 @@
     <t xml:space="preserve">ADVERTISED shared van 15 each way</t>
   </si>
   <si>
+    <t xml:space="preserve">DAN or equivalent dive-accident cover, required, bought by each person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED DAN membership + Preferred plan</t>
+  </si>
+  <si>
     <t xml:space="preserve">PADI AOW eLearning (add-on for AOW takers)</t>
   </si>
   <si>
@@ -289,7 +301,7 @@
     <t xml:space="preserve">0</t>
   </si>
   <si>
-    <t xml:space="preserve">DAN dive-accident cover</t>
+    <t xml:space="preserve">DAN dive-accident cover (not in the fee; each person buys their own, see below)</t>
   </si>
   <si>
     <t xml:space="preserve">Hotel Plaza, 6 nights with breakfast, 2 sharing</t>
@@ -331,7 +343,7 @@
     <t xml:space="preserve">Trip fee</t>
   </si>
   <si>
-    <t xml:space="preserve">Own spending: meals, drinks, tips, airport transfers</t>
+    <t xml:space="preserve">Own spending: DAN cover, meals, drinks, tips, airport transfers</t>
   </si>
   <si>
     <t xml:space="preserve">Guidance budget</t>
@@ -340,7 +352,7 @@
     <t xml:space="preserve">Guidance budget, certified taking AOW and nitrox</t>
   </si>
   <si>
-    <t xml:space="preserve">The fee covers everything diving-related (course or package, gear, park fees, eLearning), DAN insurance and the hotel; everything else is the person's own. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
+    <t xml:space="preserve">The fee covers everything diving-related (course or package, gear, park fees, eLearning) and the hotel; everything else is the person's own, including the required DAN or equivalent dive-accident cover. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
   </si>
   <si>
     <t xml:space="preserve">Group budget at four sizes (half students; George leads and does not pay)</t>
@@ -520,7 +532,7 @@
     <t xml:space="preserve">Fri 13 Nov</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue Note final payment (30 days out); hotel balance per its terms; buy eLearning codes and DAN</t>
+    <t xml:space="preserve">Blue Note final payment (30 days out); hotel balance per its terms; buy eLearning codes</t>
   </si>
   <si>
     <t xml:space="preserve">Sun 6 Dec</t>
@@ -965,7 +977,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72"/>
@@ -1375,37 +1387,37 @@
         <v>56</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
         <v>57</v>
       </c>
       <c r="B32" s="7" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B33" s="7" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -1413,7 +1425,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B35" s="7" t="n">
         <v>700</v>
@@ -1422,12 +1434,12 @@
         <v>17</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B36" s="7" t="n">
         <f aca="false">(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2</f>
@@ -1437,12 +1449,12 @@
         <v>17</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B37" s="7" t="n">
         <f aca="false">Inputs!$B$36</f>
@@ -1452,26 +1464,26 @@
         <v>17</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B38" s="7" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B39" s="7" t="n">
         <f aca="false">Inputs!$B$12*5</f>
@@ -1481,12 +1493,12 @@
         <v>17</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -1494,7 +1506,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B41" s="7" t="n">
         <v>45</v>
@@ -1503,12 +1515,12 @@
         <v>22</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B42" s="5" t="n">
         <v>6</v>
@@ -1520,7 +1532,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B43" s="7" t="n">
         <v>50</v>
@@ -1529,12 +1541,12 @@
         <v>17</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B44" s="7" t="n">
         <v>30</v>
@@ -1543,21 +1555,35 @@
         <v>17</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B45" s="7" t="n">
-        <v>220</v>
+        <v>119</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B46" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1585,7 +1611,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1593,15 +1619,15 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">Inputs!$B$9+Inputs!$B$10</f>
@@ -1614,7 +1640,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">Inputs!$B$12*Inputs!$B$14</f>
@@ -1627,7 +1653,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">Inputs!$B$15*Inputs!$B$17</f>
@@ -1640,45 +1666,45 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">Inputs!$B$33</f>
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">Inputs!$B$33</f>
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">Inputs!$B$31</f>
         <v>195</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">Inputs!$B$32</f>
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">Inputs!$B$32</f>
-        <v>119</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">((Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2)</f>
@@ -1691,54 +1717,54 @@
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">(Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39)/(Inputs!$B$4-1)</f>
-        <v>76.8947368421053</v>
+        <v>70.6315789473684</v>
       </c>
       <c r="C10" s="8" t="n">
         <f aca="false">(Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39)/(Inputs!$B$4-1)</f>
-        <v>76.8947368421053</v>
+        <v>70.6315789473684</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">SUM(B3:B10)</f>
-        <v>1581.89473684211</v>
+        <v>1256.63157894737</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">SUM(C3:C10)</f>
-        <v>1466.89473684211</v>
+        <v>1141.63157894737</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">ROUND(B11*Inputs!$B$7,0)</f>
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">ROUND(C11*Inputs!$B$7,0)</f>
-        <v>88</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">CEILING(B11+B12,100)</f>
-        <v>1700</v>
+        <v>1400</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">CEILING(C11+C12,100)</f>
-        <v>1600</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1748,29 +1774,29 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C16" s="8" t="n">
-        <f aca="false">Inputs!$B$45</f>
+        <f aca="false">Inputs!$B$46</f>
         <v>220</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">Inputs!$B$23*10</f>
@@ -1779,7 +1805,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">Inputs!$B$21+Inputs!$B$15</f>
@@ -1792,7 +1818,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">Inputs!$B$22/10</f>
@@ -1810,60 +1836,60 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B13</f>
-        <v>1700</v>
+        <v>1400</v>
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">C13</f>
-        <v>1600</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B23" s="8" t="n">
-        <f aca="false">Inputs!$B$41*Inputs!$B$42+Inputs!$B$43+Inputs!$B$44</f>
-        <v>350</v>
+        <f aca="false">Inputs!$B$45+Inputs!$B$41*Inputs!$B$42+Inputs!$B$43+Inputs!$B$44</f>
+        <v>469</v>
       </c>
       <c r="C23" s="8" t="n">
-        <f aca="false">Inputs!$B$41*Inputs!$B$42+Inputs!$B$43+Inputs!$B$44</f>
-        <v>350</v>
+        <f aca="false">Inputs!$B$45+Inputs!$B$41*Inputs!$B$42+Inputs!$B$43+Inputs!$B$44</f>
+        <v>469</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">B22+B23</f>
-        <v>2050</v>
+        <v>1869</v>
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">C22+C23</f>
-        <v>1950</v>
+        <v>1769</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C25" s="9" t="n">
         <f aca="false">C24+C16+C17</f>
-        <v>2290</v>
+        <v>2109</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1873,7 +1899,7 @@
     </row>
     <row r="27" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1903,7 +1929,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1913,21 +1939,21 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>12</v>
@@ -1944,7 +1970,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
@@ -1965,7 +1991,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$6,0)</f>
@@ -1986,7 +2012,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">B4-B5</f>
@@ -2007,7 +2033,7 @@
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">ROUNDUP(B3/2,0)</f>
@@ -2028,7 +2054,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2037,28 +2063,28 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">B5*Fee!$B$13+B6*Fee!$C$13</f>
-        <v>18200</v>
+        <v>14900</v>
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">C5*Fee!$B$13+C6*Fee!$C$13</f>
-        <v>31400</v>
+        <v>25700</v>
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">D5*Fee!$B$13+D6*Fee!$C$13</f>
-        <v>47900</v>
+        <v>39200</v>
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">E5*Fee!$B$13+E6*Fee!$C$13</f>
-        <v>64400</v>
+        <v>52700</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2067,7 +2093,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$9+Inputs!$B$10)</f>
@@ -2088,7 +2114,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B6*Inputs!$B$11</f>
@@ -2109,7 +2135,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">INT(B6/Inputs!$B$19)</f>
@@ -2130,7 +2156,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">IF(B13&gt;=1,0,Inputs!$B$11)</f>
@@ -2151,7 +2177,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">-MAX(B13-1,0)*Inputs!$B$11</f>
@@ -2172,7 +2198,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B11+B12+B14+B15</f>
@@ -2193,7 +2219,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">-B12*Inputs!$B$18</f>
@@ -2214,7 +2240,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B16+B17</f>
@@ -2235,7 +2261,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-B17</f>
@@ -2256,7 +2282,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B5*Inputs!$B$12*Inputs!$B$14+(B6+1)*Inputs!$B$12*Inputs!$B$13</f>
@@ -2277,28 +2303,28 @@
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B21" s="8" t="n">
         <f aca="false">B3*Inputs!$B$33</f>
-        <v>2400</v>
+        <v>0</v>
       </c>
       <c r="C21" s="8" t="n">
         <f aca="false">C3*Inputs!$B$33</f>
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="D21" s="8" t="n">
         <f aca="false">D3*Inputs!$B$33</f>
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="E21" s="8" t="n">
         <f aca="false">E3*Inputs!$B$33</f>
-        <v>8000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B5*Inputs!$B$15*Inputs!$B$17+(B6+1)*Inputs!$B$15*Inputs!$B$16</f>
@@ -2319,7 +2345,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">B5*Inputs!$B$31</f>
@@ -2340,28 +2366,28 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">B3*Inputs!$B$32</f>
-        <v>1428</v>
+        <v>0</v>
       </c>
       <c r="C24" s="8" t="n">
         <f aca="false">C3*Inputs!$B$32</f>
-        <v>2380</v>
+        <v>0</v>
       </c>
       <c r="D24" s="8" t="n">
         <f aca="false">D3*Inputs!$B$32</f>
-        <v>3570</v>
+        <v>0</v>
       </c>
       <c r="E24" s="8" t="n">
         <f aca="false">E3*Inputs!$B$32</f>
-        <v>4760</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">B7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
@@ -2382,7 +2408,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">Inputs!$B$35</f>
@@ -2403,28 +2429,28 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B27" s="9" t="n">
         <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25+B26</f>
-        <v>17470</v>
+        <v>13642</v>
       </c>
       <c r="C27" s="9" t="n">
         <f aca="false">C18+C19+C20+C21+C22+C23+C24+C25+C26</f>
-        <v>29050</v>
+        <v>22670</v>
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
-        <v>42925</v>
+        <v>33355</v>
       </c>
       <c r="E27" s="9" t="n">
         <f aca="false">E18+E19+E20+E21+E22+E23+E24+E25+E26</f>
-        <v>56800</v>
+        <v>44040</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -2433,70 +2459,70 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">B9-B27</f>
-        <v>730</v>
+        <v>1258</v>
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">C9-C27</f>
-        <v>2350</v>
+        <v>3030</v>
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">D9-D27</f>
-        <v>4975</v>
+        <v>5845</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">E9-E27</f>
-        <v>7600</v>
+        <v>8660</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B30" s="8" t="n">
         <f aca="false">B29/B4</f>
-        <v>66.3636363636364</v>
+        <v>114.363636363636</v>
       </c>
       <c r="C30" s="8" t="n">
         <f aca="false">C29/C4</f>
-        <v>123.684210526316</v>
+        <v>159.473684210526</v>
       </c>
       <c r="D30" s="8" t="n">
         <f aca="false">D29/D4</f>
-        <v>171.551724137931</v>
+        <v>201.551724137931</v>
       </c>
       <c r="E30" s="8" t="n">
         <f aca="false">E29/E4</f>
-        <v>194.871794871795</v>
+        <v>222.051282051282</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">B29/B9</f>
-        <v>0.0401098901098901</v>
+        <v>0.0844295302013423</v>
       </c>
       <c r="C31" s="11" t="n">
         <f aca="false">C29/C9</f>
-        <v>0.0748407643312102</v>
+        <v>0.117898832684825</v>
       </c>
       <c r="D31" s="11" t="n">
         <f aca="false">D29/D9</f>
-        <v>0.103862212943633</v>
+        <v>0.149107142857143</v>
       </c>
       <c r="E31" s="11" t="n">
         <f aca="false">E29/E9</f>
-        <v>0.118012422360248</v>
+        <v>0.164326375711575</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B32" s="12" t="str">
         <f aca="false">IF(B29&gt;=0,"yes","NO")</f>
@@ -2517,7 +2543,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B33" s="9" t="n">
         <f aca="false">B19</f>
@@ -2538,7 +2564,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -2547,7 +2573,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">B4*400</f>
@@ -2568,7 +2594,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B36" s="8" t="n">
         <f aca="false">B16*Inputs!$B$20+B25*Inputs!$B$29</f>
@@ -2589,7 +2615,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B37" s="9" t="n">
         <f aca="false">B35-B36</f>
@@ -2610,49 +2636,49 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">B9-B35</f>
-        <v>13800</v>
+        <v>10500</v>
       </c>
       <c r="C38" s="8" t="n">
         <f aca="false">C9-C35</f>
-        <v>23800</v>
+        <v>18100</v>
       </c>
       <c r="D38" s="8" t="n">
         <f aca="false">D9-D35</f>
-        <v>36300</v>
+        <v>27600</v>
       </c>
       <c r="E38" s="8" t="n">
         <f aca="false">E9-E35</f>
-        <v>48800</v>
+        <v>37100</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B39" s="8" t="n">
         <f aca="false">B18-B16*Inputs!$B$20+B20+B25*(1-Inputs!$B$29)+B23+B24</f>
-        <v>10902</v>
+        <v>9474</v>
       </c>
       <c r="C39" s="8" t="n">
         <f aca="false">C18-C16*Inputs!$B$20+C20+C25*(1-Inputs!$B$29)+C23+C24</f>
-        <v>18430</v>
+        <v>16050</v>
       </c>
       <c r="D39" s="8" t="n">
         <f aca="false">D18-D16*Inputs!$B$20+D20+D25*(1-Inputs!$B$29)+D23+D24</f>
-        <v>27390</v>
+        <v>23820</v>
       </c>
       <c r="E39" s="8" t="n">
         <f aca="false">E18-E16*Inputs!$B$20+E20+E25*(1-Inputs!$B$29)+E23+E24</f>
-        <v>36350</v>
+        <v>31590</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B40" s="8" t="n">
         <f aca="false">B22</f>
@@ -2673,7 +2699,7 @@
     </row>
     <row r="41" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -2706,108 +2732,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2817,10 +2843,10 @@
     </row>
     <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>10</v>
@@ -2828,10 +2854,10 @@
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Cozumel: cost-lever research (dive cover, rental, eLearning, comps, lodging), Doug question queue and batching rule; park and eLearning inputs corrected
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="182">
   <si>
     <t xml:space="preserve">Cozumel group budget — inputs (blue cells are editable)</t>
   </si>
@@ -94,6 +94,9 @@
     <t xml:space="preserve">USD/day</t>
   </si>
   <si>
+    <t xml:space="preserve">QUOTED; group rate of 20–25 asked (competitors advertise 20–25)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Rental days, certified</t>
   </si>
   <si>
@@ -112,7 +115,7 @@
     <t xml:space="preserve">Marine park fee per boat day</t>
   </si>
   <si>
-    <t xml:space="preserve">ADVERTISED rate; QUOTED 23 Sep: paid on site for boat days only, none on the two training-site days</t>
+    <t xml:space="preserve">ADVERTISED: 225 pesos in 2026 (Blue Note site shows USD 12 / 220 pesos); QUOTED 23 Sep: paid on site for boat days only, none on the two training-site days</t>
   </si>
   <si>
     <t xml:space="preserve">Boat days, certified</t>
@@ -193,7 +196,7 @@
     <t xml:space="preserve">PADI Open Water eLearning (club buys the codes)</t>
   </si>
   <si>
-    <t xml:space="preserve">ADVERTISED</t>
+    <t xml:space="preserve">ADVERTISED store.padi.com about USD 230; Blue Note asked for its code price</t>
   </si>
   <si>
     <t xml:space="preserve">DAN cover inside the fee</t>
@@ -262,10 +265,10 @@
     <t xml:space="preserve">ADVERTISED shared van 15 each way</t>
   </si>
   <si>
-    <t xml:space="preserve">DAN or equivalent dive-accident cover, required, bought by each person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED DAN membership + Preferred plan</t>
+    <t xml:space="preserve">Dive-accident cover, required, bought by each person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED: DAN membership 40 + Master 44; DAN short-term 6–10 day plan USD 50 if Blue Note sells it (asked)</t>
   </si>
   <si>
     <t xml:space="preserve">PADI AOW eLearning (add-on for AOW takers)</t>
@@ -1132,82 +1135,82 @@
         <v>22</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>5</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>2</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B15" s="7" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>5</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B18" s="6" t="n">
         <v>0.1</v>
@@ -1216,18 +1219,18 @@
         <v>12</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>5</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>18</v>
@@ -1235,7 +1238,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B20" s="6" t="n">
         <v>0.25</v>
@@ -1244,12 +1247,12 @@
         <v>12</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B21" s="7" t="n">
         <v>130</v>
@@ -1258,12 +1261,12 @@
         <v>17</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B22" s="7" t="n">
         <v>800</v>
@@ -1272,12 +1275,12 @@
         <v>17</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>12</v>
@@ -1286,12 +1289,12 @@
         <v>17</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -1299,7 +1302,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B25" s="7" t="n">
         <v>70</v>
@@ -1308,12 +1311,12 @@
         <v>17</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B26" s="7" t="n">
         <v>88</v>
@@ -1322,38 +1325,38 @@
         <v>17</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B27" s="5" t="n">
         <v>2</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B28" s="5" t="n">
         <v>4</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B29" s="6" t="n">
         <v>0.25</v>
@@ -1362,34 +1365,34 @@
         <v>12</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B31" s="7" t="n">
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B32" s="7" t="n">
         <v>0</v>
@@ -1398,12 +1401,12 @@
         <v>17</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B33" s="7" t="n">
         <v>0</v>
@@ -1412,12 +1415,12 @@
         <v>17</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -1425,7 +1428,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B35" s="7" t="n">
         <v>700</v>
@@ -1434,12 +1437,12 @@
         <v>17</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B36" s="7" t="n">
         <f aca="false">(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2</f>
@@ -1449,12 +1452,12 @@
         <v>17</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B37" s="7" t="n">
         <f aca="false">Inputs!$B$36</f>
@@ -1464,12 +1467,12 @@
         <v>17</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B38" s="7" t="n">
         <v>0</v>
@@ -1478,12 +1481,12 @@
         <v>17</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B39" s="7" t="n">
         <f aca="false">Inputs!$B$12*5</f>
@@ -1493,12 +1496,12 @@
         <v>17</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -1506,7 +1509,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B41" s="7" t="n">
         <v>45</v>
@@ -1515,24 +1518,24 @@
         <v>22</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B42" s="5" t="n">
         <v>6</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B43" s="7" t="n">
         <v>50</v>
@@ -1541,12 +1544,12 @@
         <v>17</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B44" s="7" t="n">
         <v>30</v>
@@ -1555,26 +1558,26 @@
         <v>17</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B45" s="7" t="n">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B46" s="7" t="n">
         <v>220</v>
@@ -1583,7 +1586,7 @@
         <v>17</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1611,7 +1614,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1619,15 +1622,15 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">Inputs!$B$9+Inputs!$B$10</f>
@@ -1640,7 +1643,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">Inputs!$B$12*Inputs!$B$14</f>
@@ -1653,20 +1656,20 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">Inputs!$B$15*Inputs!$B$17</f>
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C5" s="8" t="n">
         <f aca="false">Inputs!$B$15*Inputs!$B$16</f>
-        <v>75</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">Inputs!$B$33</f>
@@ -1679,19 +1682,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">Inputs!$B$31</f>
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">Inputs!$B$32</f>
@@ -1704,7 +1707,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">((Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2)</f>
@@ -1717,7 +1720,7 @@
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">(Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39)/(Inputs!$B$4-1)</f>
@@ -1730,24 +1733,24 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">SUM(B3:B10)</f>
-        <v>1256.63157894737</v>
+        <v>1285.63157894737</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">SUM(C3:C10)</f>
-        <v>1141.63157894737</v>
+        <v>1131.63157894737</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">ROUND(B11*Inputs!$B$7,0)</f>
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">ROUND(C11*Inputs!$B$7,0)</f>
@@ -1756,7 +1759,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">CEILING(B11+B12,100)</f>
@@ -1764,7 +1767,7 @@
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">CEILING(C11+C12,100)</f>
-        <v>1300</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1774,17 +1777,17 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C16" s="8" t="n">
         <f aca="false">Inputs!$B$46</f>
@@ -1793,10 +1796,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>101</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>100</v>
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">Inputs!$B$23*10</f>
@@ -1805,20 +1808,20 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">Inputs!$B$21+Inputs!$B$15</f>
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C18" s="8" t="n">
         <f aca="false">Inputs!$B$21+Inputs!$B$15</f>
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">Inputs!$B$22/10</f>
@@ -1836,14 +1839,14 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B13</f>
@@ -1851,45 +1854,45 @@
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">C13</f>
-        <v>1300</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">Inputs!$B$45+Inputs!$B$41*Inputs!$B$42+Inputs!$B$43+Inputs!$B$44</f>
-        <v>469</v>
+        <v>434</v>
       </c>
       <c r="C23" s="8" t="n">
         <f aca="false">Inputs!$B$45+Inputs!$B$41*Inputs!$B$42+Inputs!$B$43+Inputs!$B$44</f>
-        <v>469</v>
+        <v>434</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">B22+B23</f>
-        <v>1869</v>
+        <v>1834</v>
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">C22+C23</f>
-        <v>1769</v>
+        <v>1634</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C25" s="9" t="n">
         <f aca="false">C24+C16+C17</f>
-        <v>2109</v>
+        <v>1974</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1899,7 +1902,7 @@
     </row>
     <row r="27" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1929,7 +1932,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1939,21 +1942,21 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>12</v>
@@ -1970,7 +1973,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
@@ -1991,7 +1994,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$6,0)</f>
@@ -2012,7 +2015,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">B4-B5</f>
@@ -2033,7 +2036,7 @@
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">ROUNDUP(B3/2,0)</f>
@@ -2054,7 +2057,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2063,28 +2066,28 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">B5*Fee!$B$13+B6*Fee!$C$13</f>
-        <v>14900</v>
+        <v>14400</v>
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">C5*Fee!$B$13+C6*Fee!$C$13</f>
-        <v>25700</v>
+        <v>24800</v>
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">D5*Fee!$B$13+D6*Fee!$C$13</f>
-        <v>39200</v>
+        <v>37800</v>
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">E5*Fee!$B$13+E6*Fee!$C$13</f>
-        <v>52700</v>
+        <v>50800</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2093,7 +2096,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$9+Inputs!$B$10)</f>
@@ -2114,7 +2117,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B6*Inputs!$B$11</f>
@@ -2135,7 +2138,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">INT(B6/Inputs!$B$19)</f>
@@ -2156,7 +2159,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">IF(B13&gt;=1,0,Inputs!$B$11)</f>
@@ -2177,7 +2180,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">-MAX(B13-1,0)*Inputs!$B$11</f>
@@ -2198,7 +2201,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B11+B12+B14+B15</f>
@@ -2219,7 +2222,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">-B12*Inputs!$B$18</f>
@@ -2240,7 +2243,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B16+B17</f>
@@ -2261,7 +2264,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-B17</f>
@@ -2282,7 +2285,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B5*Inputs!$B$12*Inputs!$B$14+(B6+1)*Inputs!$B$12*Inputs!$B$13</f>
@@ -2303,7 +2306,7 @@
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B21" s="8" t="n">
         <f aca="false">B3*Inputs!$B$33</f>
@@ -2324,49 +2327,49 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B5*Inputs!$B$15*Inputs!$B$17+(B6+1)*Inputs!$B$15*Inputs!$B$16</f>
-        <v>720</v>
+        <v>624</v>
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">C5*Inputs!$B$15*Inputs!$B$17+(C6+1)*Inputs!$B$15*Inputs!$B$16</f>
-        <v>1200</v>
+        <v>1040</v>
       </c>
       <c r="D22" s="8" t="n">
         <f aca="false">D5*Inputs!$B$15*Inputs!$B$17+(D6+1)*Inputs!$B$15*Inputs!$B$16</f>
-        <v>1800</v>
+        <v>1560</v>
       </c>
       <c r="E22" s="8" t="n">
         <f aca="false">E5*Inputs!$B$15*Inputs!$B$17+(E6+1)*Inputs!$B$15*Inputs!$B$16</f>
-        <v>2400</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">B5*Inputs!$B$31</f>
-        <v>1170</v>
+        <v>1380</v>
       </c>
       <c r="C23" s="8" t="n">
         <f aca="false">C5*Inputs!$B$31</f>
-        <v>1950</v>
+        <v>2300</v>
       </c>
       <c r="D23" s="8" t="n">
         <f aca="false">D5*Inputs!$B$31</f>
-        <v>2925</v>
+        <v>3450</v>
       </c>
       <c r="E23" s="8" t="n">
         <f aca="false">E5*Inputs!$B$31</f>
-        <v>3900</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">B3*Inputs!$B$32</f>
@@ -2387,7 +2390,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">B7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
@@ -2408,7 +2411,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">Inputs!$B$35</f>
@@ -2429,28 +2432,28 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B27" s="9" t="n">
         <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25+B26</f>
-        <v>13642</v>
+        <v>13756</v>
       </c>
       <c r="C27" s="9" t="n">
         <f aca="false">C18+C19+C20+C21+C22+C23+C24+C25+C26</f>
-        <v>22670</v>
+        <v>22860</v>
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
-        <v>33355</v>
+        <v>33640</v>
       </c>
       <c r="E27" s="9" t="n">
         <f aca="false">E18+E19+E20+E21+E22+E23+E24+E25+E26</f>
-        <v>44040</v>
+        <v>44420</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -2459,70 +2462,70 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">B9-B27</f>
-        <v>1258</v>
+        <v>644</v>
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">C9-C27</f>
-        <v>3030</v>
+        <v>1940</v>
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">D9-D27</f>
-        <v>5845</v>
+        <v>4160</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">E9-E27</f>
-        <v>8660</v>
+        <v>6380</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B30" s="8" t="n">
         <f aca="false">B29/B4</f>
-        <v>114.363636363636</v>
+        <v>58.5454545454546</v>
       </c>
       <c r="C30" s="8" t="n">
         <f aca="false">C29/C4</f>
-        <v>159.473684210526</v>
+        <v>102.105263157895</v>
       </c>
       <c r="D30" s="8" t="n">
         <f aca="false">D29/D4</f>
-        <v>201.551724137931</v>
+        <v>143.448275862069</v>
       </c>
       <c r="E30" s="8" t="n">
         <f aca="false">E29/E4</f>
-        <v>222.051282051282</v>
+        <v>163.589743589744</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">B29/B9</f>
-        <v>0.0844295302013423</v>
+        <v>0.0447222222222222</v>
       </c>
       <c r="C31" s="11" t="n">
         <f aca="false">C29/C9</f>
-        <v>0.117898832684825</v>
+        <v>0.0782258064516129</v>
       </c>
       <c r="D31" s="11" t="n">
         <f aca="false">D29/D9</f>
-        <v>0.149107142857143</v>
+        <v>0.11005291005291</v>
       </c>
       <c r="E31" s="11" t="n">
         <f aca="false">E29/E9</f>
-        <v>0.164326375711575</v>
+        <v>0.125590551181102</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B32" s="12" t="str">
         <f aca="false">IF(B29&gt;=0,"yes","NO")</f>
@@ -2543,7 +2546,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B33" s="9" t="n">
         <f aca="false">B19</f>
@@ -2564,7 +2567,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -2573,7 +2576,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">B4*400</f>
@@ -2594,7 +2597,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B36" s="8" t="n">
         <f aca="false">B16*Inputs!$B$20+B25*Inputs!$B$29</f>
@@ -2615,7 +2618,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B37" s="9" t="n">
         <f aca="false">B35-B36</f>
@@ -2636,70 +2639,70 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">B9-B35</f>
-        <v>10500</v>
+        <v>10000</v>
       </c>
       <c r="C38" s="8" t="n">
         <f aca="false">C9-C35</f>
-        <v>18100</v>
+        <v>17200</v>
       </c>
       <c r="D38" s="8" t="n">
         <f aca="false">D9-D35</f>
-        <v>27600</v>
+        <v>26200</v>
       </c>
       <c r="E38" s="8" t="n">
         <f aca="false">E9-E35</f>
-        <v>37100</v>
+        <v>35200</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B39" s="8" t="n">
         <f aca="false">B18-B16*Inputs!$B$20+B20+B25*(1-Inputs!$B$29)+B23+B24</f>
-        <v>9474</v>
+        <v>9684</v>
       </c>
       <c r="C39" s="8" t="n">
         <f aca="false">C18-C16*Inputs!$B$20+C20+C25*(1-Inputs!$B$29)+C23+C24</f>
-        <v>16050</v>
+        <v>16400</v>
       </c>
       <c r="D39" s="8" t="n">
         <f aca="false">D18-D16*Inputs!$B$20+D20+D25*(1-Inputs!$B$29)+D23+D24</f>
-        <v>23820</v>
+        <v>24345</v>
       </c>
       <c r="E39" s="8" t="n">
         <f aca="false">E18-E16*Inputs!$B$20+E20+E25*(1-Inputs!$B$29)+E23+E24</f>
-        <v>31590</v>
+        <v>32290</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B40" s="8" t="n">
         <f aca="false">B22</f>
-        <v>720</v>
+        <v>624</v>
       </c>
       <c r="C40" s="8" t="n">
         <f aca="false">C22</f>
-        <v>1200</v>
+        <v>1040</v>
       </c>
       <c r="D40" s="8" t="n">
         <f aca="false">D22</f>
-        <v>1800</v>
+        <v>1560</v>
       </c>
       <c r="E40" s="8" t="n">
         <f aca="false">E22</f>
-        <v>2400</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -2732,108 +2735,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2843,10 +2846,10 @@
     </row>
     <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>10</v>
@@ -2854,10 +2857,10 @@
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Blue Note answers (taxes in, full rental, boat blocked, deposit 12 Oct); Dive Paradise and Aldora closed; Paradise Scuba itinerary agreed; Cozumel fees 1,450 / 1,350 with cover and computers in the fee
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="184">
   <si>
     <t xml:space="preserve">Cozumel group budget — inputs (blue cells are editable)</t>
   </si>
@@ -94,7 +94,13 @@
     <t xml:space="preserve">USD/day</t>
   </si>
   <si>
-    <t xml:space="preserve">QUOTED; group rate of 20–25 asked (competitors advertise 20–25)</t>
+    <t xml:space="preserve">QUOTED 24 Sep: full set BCD, regulator, mask, fins, wetsuit; bulk-rate ask saved for October</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dive computer rental per day (included on courses; extra on regular rentals)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 24 Sep; in the fee for every boat day under the everyone-rents rule</t>
   </si>
   <si>
     <t xml:space="preserve">Rental days, certified</t>
@@ -199,16 +205,16 @@
     <t xml:space="preserve">ADVERTISED store.padi.com about USD 230; Blue Note asked for its code price</t>
   </si>
   <si>
-    <t xml:space="preserve">DAN cover inside the fee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George 24 Sep: not in the fee; each diver buys their own dive-accident cover (see own spending)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tax buffer per head (Mexican IVA and lodging tax if the quotes are pre-tax)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George 24 Sep: cut; the other three shops quoted tax-inclusive; Doug asked to confirm</t>
+    <t xml:space="preserve">Dive-accident cover inside the fee (DAN short-term 6–10 day plan via the shop, one roster)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED plan price; ASSUMED Blue Note sells it (asked 24 Sep). If not: 0 here and each person buys DAN Master (84)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tax buffer per head</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 24 Sep: Blue Note prices include taxes</t>
   </si>
   <si>
     <t xml:space="preserve">Leader costs carried by the group (George shares a room like everyone)</t>
@@ -232,13 +238,13 @@
     <t xml:space="preserve">formula: half a room</t>
   </si>
   <si>
-    <t xml:space="preserve">George's DAN cover carried by the group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George 24 Sep: own cost like everyone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George's gear rental, 5 days</t>
+    <t xml:space="preserve">George's dive cover carried by the group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same plan as everyone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George's gear and computer rental, 5 days</t>
   </si>
   <si>
     <t xml:space="preserve">Own spending guidance, not in the fee (no flights)</t>
@@ -265,10 +271,10 @@
     <t xml:space="preserve">ADVERTISED shared van 15 each way</t>
   </si>
   <si>
-    <t xml:space="preserve">Dive-accident cover, required, bought by each person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED: DAN membership 40 + Master 44; DAN short-term 6–10 day plan USD 50 if Blue Note sells it (asked)</t>
+    <t xml:space="preserve">Dive cover bought by each person (only if the shop cannot sell the short-term plan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 while cover is inside the fee; 84 (DAN membership + Master) if it moves out</t>
   </si>
   <si>
     <t xml:space="preserve">PADI AOW eLearning (add-on for AOW takers)</t>
@@ -289,13 +295,13 @@
     <t xml:space="preserve">Diving with Blue Note</t>
   </si>
   <si>
-    <t xml:space="preserve">Gear rental, everyone</t>
+    <t xml:space="preserve">Gear rental incl. computer, everyone</t>
   </si>
   <si>
     <t xml:space="preserve">Marine park fees</t>
   </si>
   <si>
-    <t xml:space="preserve">Tax buffer (IVA and lodging tax, if the quotes are pre-tax)</t>
+    <t xml:space="preserve">Tax buffer (zero: Blue Note prices include taxes)</t>
   </si>
   <si>
     <t xml:space="preserve">PADI eLearning</t>
@@ -304,7 +310,7 @@
     <t xml:space="preserve">0</t>
   </si>
   <si>
-    <t xml:space="preserve">DAN dive-accident cover (not in the fee; each person buys their own, see below)</t>
+    <t xml:space="preserve">Dive-accident cover (DAN short-term plan via the shop, assumed)</t>
   </si>
   <si>
     <t xml:space="preserve">Hotel Plaza, 6 nights with breakfast, 2 sharing</t>
@@ -319,7 +325,7 @@
     <t xml:space="preserve">Contingency</t>
   </si>
   <si>
-    <t xml:space="preserve">TRIP FEE (rounded up to the nearest 100, as posted)</t>
+    <t xml:space="preserve">TRIP FEE (rounded up to the nearest 50, as posted)</t>
   </si>
   <si>
     <t xml:space="preserve">Optional add-ons at sign-up, charged at cost</t>
@@ -346,7 +352,7 @@
     <t xml:space="preserve">Trip fee</t>
   </si>
   <si>
-    <t xml:space="preserve">Own spending: DAN cover, meals, drinks, tips, airport transfers</t>
+    <t xml:space="preserve">Own spending: meals, drinks, tips, airport transfers (own dive cover only if it leaves the fee)</t>
   </si>
   <si>
     <t xml:space="preserve">Guidance budget</t>
@@ -355,7 +361,7 @@
     <t xml:space="preserve">Guidance budget, certified taking AOW and nitrox</t>
   </si>
   <si>
-    <t xml:space="preserve">The fee covers everything diving-related (course or package, gear, park fees, eLearning) and the hotel; everything else is the person's own, including the required DAN or equivalent dive-accident cover. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
+    <t xml:space="preserve">The fee covers everything diving-related (course or package, gear and computer, park fees, eLearning), dive-accident cover bought through the shop, and the hotel; flights, meals, drinks, tips and transfers are the person's own. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
   </si>
   <si>
     <t xml:space="preserve">Group budget at four sizes (half students; George leads and does not pay)</t>
@@ -424,7 +430,7 @@
     <t xml:space="preserve">Commission passed to George</t>
   </si>
   <si>
-    <t xml:space="preserve">Gear rental for everyone including George</t>
+    <t xml:space="preserve">Gear and computer rental for everyone including George</t>
   </si>
   <si>
     <t xml:space="preserve">Tax buffer held (paid to Blue Note and the hotel if charged; otherwise refunded)</t>
@@ -436,7 +442,7 @@
     <t xml:space="preserve">PADI Open Water eLearning codes</t>
   </si>
   <si>
-    <t xml:space="preserve">DAN cover for everyone including George</t>
+    <t xml:space="preserve">Dive cover for everyone including George (short-term plan via the shop)</t>
   </si>
   <si>
     <t xml:space="preserve">Hotel Plaza block, all rooms</t>
@@ -980,7 +986,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72"/>
@@ -1124,7 +1130,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
@@ -1138,127 +1144,127 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="5" t="n">
-        <v>5</v>
+      <c r="B13" s="7" t="n">
+        <v>10</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="7" t="n">
-        <v>13</v>
+      <c r="B15" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="5" t="n">
-        <v>5</v>
+      <c r="B16" s="7" t="n">
+        <v>13</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B18" s="6" t="n">
-        <v>0.1</v>
+        <v>34</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="5" t="n">
-        <v>5</v>
+      <c r="B19" s="6" t="n">
+        <v>0.1</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="6" t="n">
-        <v>0.25</v>
+      <c r="B20" s="5" t="n">
+        <v>5</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="7" t="n">
-        <v>130</v>
+      <c r="B21" s="6" t="n">
+        <v>0.25</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>40</v>
@@ -1269,57 +1275,57 @@
         <v>41</v>
       </c>
       <c r="B22" s="7" t="n">
-        <v>800</v>
+        <v>130</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B23" s="7" t="n">
-        <v>12</v>
+        <v>800</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
+      <c r="B24" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="A25" s="4" t="s">
         <v>46</v>
       </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B26" s="7" t="n">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>17</v>
@@ -1332,70 +1338,70 @@
       <c r="A27" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B27" s="5" t="n">
-        <v>2</v>
+      <c r="B27" s="7" t="n">
+        <v>88</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D28" s="2"/>
+      <c r="D28" s="2" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B29" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="6" t="n">
         <v>0.25</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-    </row>
-    <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="7" t="n">
-        <v>230</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D31" s="2" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
         <v>57</v>
       </c>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B32" s="7" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>17</v>
@@ -1409,7 +1415,7 @@
         <v>60</v>
       </c>
       <c r="B33" s="7" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>17</v>
@@ -1419,34 +1425,33 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
+      <c r="B34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B35" s="7" t="n">
-        <v>700</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D35" s="2" t="s">
+      <c r="A35" s="4" t="s">
         <v>64</v>
       </c>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B36" s="7" t="n">
-        <f aca="false">(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2</f>
-        <v>246</v>
+        <v>700</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>17</v>
@@ -1460,7 +1465,7 @@
         <v>67</v>
       </c>
       <c r="B37" s="7" t="n">
-        <f aca="false">Inputs!$B$36</f>
+        <f aca="false">(Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)/2</f>
         <v>246</v>
       </c>
       <c r="C37" s="2" t="s">
@@ -1475,7 +1480,8 @@
         <v>69</v>
       </c>
       <c r="B38" s="7" t="n">
-        <v>0</v>
+        <f aca="false">Inputs!$B$37</f>
+        <v>246</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>17</v>
@@ -1489,70 +1495,70 @@
         <v>71</v>
       </c>
       <c r="B39" s="7" t="n">
-        <f aca="false">Inputs!$B$12*5</f>
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
+      <c r="A40" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B40" s="7" t="n">
+        <f aca="false">(Inputs!$B$12+Inputs!$B$13)*5</f>
+        <v>200</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B41" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D41" s="2" t="s">
+      <c r="A41" s="4" t="s">
         <v>74</v>
       </c>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B42" s="5" t="n">
-        <v>6</v>
+      <c r="B42" s="7" t="n">
+        <v>45</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D42" s="2"/>
+        <v>22</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B43" s="7" t="n">
-        <v>50</v>
+        <v>77</v>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>77</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="D43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B44" s="7" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>17</v>
@@ -1561,12 +1567,12 @@
         <v>79</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
         <v>80</v>
       </c>
       <c r="B45" s="7" t="n">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>17</v>
@@ -1575,18 +1581,32 @@
         <v>81</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
         <v>82</v>
       </c>
       <c r="B46" s="7" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>83</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1614,7 +1634,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1622,15 +1642,15 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">Inputs!$B$9+Inputs!$B$10</f>
@@ -1643,131 +1663,131 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B4" s="8" t="n">
-        <f aca="false">Inputs!$B$12*Inputs!$B$14</f>
-        <v>60</v>
+        <f aca="false">(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15</f>
+        <v>80</v>
       </c>
       <c r="C4" s="8" t="n">
-        <f aca="false">Inputs!$B$12*Inputs!$B$13</f>
-        <v>150</v>
+        <f aca="false">(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$14</f>
+        <v>200</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B5" s="8" t="n">
-        <f aca="false">Inputs!$B$15*Inputs!$B$17</f>
+        <f aca="false">Inputs!$B$16*Inputs!$B$18</f>
         <v>39</v>
       </c>
       <c r="C5" s="8" t="n">
-        <f aca="false">Inputs!$B$15*Inputs!$B$16</f>
+        <f aca="false">Inputs!$B$16*Inputs!$B$17</f>
         <v>65</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B6" s="8" t="n">
-        <f aca="false">Inputs!$B$33</f>
+        <f aca="false">Inputs!$B$34</f>
         <v>0</v>
       </c>
       <c r="C6" s="8" t="n">
-        <f aca="false">Inputs!$B$33</f>
+        <f aca="false">Inputs!$B$34</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B7" s="8" t="n">
-        <f aca="false">Inputs!$B$31</f>
+        <f aca="false">Inputs!$B$32</f>
         <v>230</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B8" s="8" t="n">
-        <f aca="false">Inputs!$B$32</f>
-        <v>0</v>
+        <f aca="false">Inputs!$B$33</f>
+        <v>50</v>
       </c>
       <c r="C8" s="8" t="n">
-        <f aca="false">Inputs!$B$32</f>
-        <v>0</v>
+        <f aca="false">Inputs!$B$33</f>
+        <v>50</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B9" s="8" t="n">
-        <f aca="false">((Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2)</f>
+        <f aca="false">((Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)/2)</f>
         <v>246</v>
       </c>
       <c r="C9" s="8" t="n">
-        <f aca="false">((Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)/2)</f>
+        <f aca="false">((Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)/2)</f>
         <v>246</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B10" s="8" t="n">
-        <f aca="false">(Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39)/(Inputs!$B$4-1)</f>
-        <v>70.6315789473684</v>
+        <f aca="false">(Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39+Inputs!$B$40)/(Inputs!$B$4-1)</f>
+        <v>75.8947368421053</v>
       </c>
       <c r="C10" s="8" t="n">
-        <f aca="false">(Inputs!$B$35+Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39)/(Inputs!$B$4-1)</f>
-        <v>70.6315789473684</v>
+        <f aca="false">(Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39+Inputs!$B$40)/(Inputs!$B$4-1)</f>
+        <v>75.8947368421053</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">SUM(B3:B10)</f>
-        <v>1285.63157894737</v>
+        <v>1360.89473684211</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">SUM(C3:C10)</f>
-        <v>1131.63157894737</v>
+        <v>1236.89473684211</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">ROUND(B11*Inputs!$B$7,0)</f>
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">ROUND(C11*Inputs!$B$7,0)</f>
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B13" s="9" t="n">
-        <f aca="false">CEILING(B11+B12,100)</f>
-        <v>1400</v>
+        <f aca="false">CEILING(B11+B12,50)</f>
+        <v>1450</v>
       </c>
       <c r="C13" s="9" t="n">
-        <f aca="false">CEILING(C11+C12,100)</f>
-        <v>1200</v>
+        <f aca="false">CEILING(C11+C12,50)</f>
+        <v>1350</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1777,58 +1797,58 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C16" s="8" t="n">
-        <f aca="false">Inputs!$B$46</f>
+        <f aca="false">Inputs!$B$47</f>
         <v>220</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C17" s="8" t="n">
-        <f aca="false">Inputs!$B$23*10</f>
+        <f aca="false">Inputs!$B$24*10</f>
         <v>120</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B18" s="8" t="n">
-        <f aca="false">Inputs!$B$21+Inputs!$B$15</f>
+        <f aca="false">Inputs!$B$22+Inputs!$B$16</f>
         <v>143</v>
       </c>
       <c r="C18" s="8" t="n">
-        <f aca="false">Inputs!$B$21+Inputs!$B$15</f>
+        <f aca="false">Inputs!$B$22+Inputs!$B$16</f>
         <v>143</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B19" s="8" t="n">
-        <f aca="false">Inputs!$B$22/10</f>
+        <f aca="false">Inputs!$B$23/10</f>
         <v>80</v>
       </c>
       <c r="C19" s="8" t="n">
-        <f aca="false">Inputs!$B$22/10</f>
+        <f aca="false">Inputs!$B$23/10</f>
         <v>80</v>
       </c>
     </row>
@@ -1839,60 +1859,60 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B13</f>
-        <v>1400</v>
+        <v>1450</v>
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">C13</f>
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B23" s="8" t="n">
-        <f aca="false">Inputs!$B$45+Inputs!$B$41*Inputs!$B$42+Inputs!$B$43+Inputs!$B$44</f>
-        <v>434</v>
+        <f aca="false">Inputs!$B$46+Inputs!$B$42*Inputs!$B$43+Inputs!$B$44+Inputs!$B$45</f>
+        <v>350</v>
       </c>
       <c r="C23" s="8" t="n">
-        <f aca="false">Inputs!$B$45+Inputs!$B$41*Inputs!$B$42+Inputs!$B$43+Inputs!$B$44</f>
-        <v>434</v>
+        <f aca="false">Inputs!$B$46+Inputs!$B$42*Inputs!$B$43+Inputs!$B$44+Inputs!$B$45</f>
+        <v>350</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">B22+B23</f>
-        <v>1834</v>
+        <v>1800</v>
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">C22+C23</f>
-        <v>1634</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C25" s="9" t="n">
         <f aca="false">C24+C16+C17</f>
-        <v>1974</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1900,9 +1920,9 @@
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
     </row>
-    <row r="27" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1932,7 +1952,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1942,21 +1962,21 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>12</v>
@@ -1973,7 +1993,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
@@ -1994,7 +2014,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$6,0)</f>
@@ -2015,7 +2035,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">B4-B5</f>
@@ -2036,7 +2056,7 @@
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">ROUNDUP(B3/2,0)</f>
@@ -2057,7 +2077,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2066,28 +2086,28 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">B5*Fee!$B$13+B6*Fee!$C$13</f>
-        <v>14400</v>
+        <v>15450</v>
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">C5*Fee!$B$13+C6*Fee!$C$13</f>
-        <v>24800</v>
+        <v>26650</v>
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">D5*Fee!$B$13+D6*Fee!$C$13</f>
-        <v>37800</v>
+        <v>40650</v>
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">E5*Fee!$B$13+E6*Fee!$C$13</f>
-        <v>50800</v>
+        <v>54650</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2096,7 +2116,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$9+Inputs!$B$10)</f>
@@ -2117,7 +2137,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B6*Inputs!$B$11</f>
@@ -2138,28 +2158,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B13" s="10" t="n">
-        <f aca="false">INT(B6/Inputs!$B$19)</f>
+        <f aca="false">INT(B6/Inputs!$B$20)</f>
         <v>1</v>
       </c>
       <c r="C13" s="10" t="n">
-        <f aca="false">INT(C6/Inputs!$B$19)</f>
+        <f aca="false">INT(C6/Inputs!$B$20)</f>
         <v>1</v>
       </c>
       <c r="D13" s="10" t="n">
-        <f aca="false">INT(D6/Inputs!$B$19)</f>
+        <f aca="false">INT(D6/Inputs!$B$20)</f>
         <v>2</v>
       </c>
       <c r="E13" s="10" t="n">
-        <f aca="false">INT(E6/Inputs!$B$19)</f>
+        <f aca="false">INT(E6/Inputs!$B$20)</f>
         <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">IF(B13&gt;=1,0,Inputs!$B$11)</f>
@@ -2180,7 +2200,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">-MAX(B13-1,0)*Inputs!$B$11</f>
@@ -2201,7 +2221,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B11+B12+B14+B15</f>
@@ -2222,28 +2242,28 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B17" s="8" t="n">
-        <f aca="false">-B12*Inputs!$B$18</f>
+        <f aca="false">-B12*Inputs!$B$19</f>
         <v>-300</v>
       </c>
       <c r="C17" s="8" t="n">
-        <f aca="false">-C12*Inputs!$B$18</f>
+        <f aca="false">-C12*Inputs!$B$19</f>
         <v>-540</v>
       </c>
       <c r="D17" s="8" t="n">
-        <f aca="false">-D12*Inputs!$B$18</f>
+        <f aca="false">-D12*Inputs!$B$19</f>
         <v>-840</v>
       </c>
       <c r="E17" s="8" t="n">
-        <f aca="false">-E12*Inputs!$B$18</f>
+        <f aca="false">-E12*Inputs!$B$19</f>
         <v>-1140</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B16+B17</f>
@@ -2264,7 +2284,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-B17</f>
@@ -2285,175 +2305,175 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B20" s="8" t="n">
-        <f aca="false">B5*Inputs!$B$12*Inputs!$B$14+(B6+1)*Inputs!$B$12*Inputs!$B$13</f>
-        <v>1260</v>
+        <f aca="false">B5*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15+(B6+1)*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$14</f>
+        <v>1680</v>
       </c>
       <c r="C20" s="8" t="n">
-        <f aca="false">C5*Inputs!$B$12*Inputs!$B$14+(C6+1)*Inputs!$B$12*Inputs!$B$13</f>
-        <v>2100</v>
+        <f aca="false">C5*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15+(C6+1)*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$14</f>
+        <v>2800</v>
       </c>
       <c r="D20" s="8" t="n">
-        <f aca="false">D5*Inputs!$B$12*Inputs!$B$14+(D6+1)*Inputs!$B$12*Inputs!$B$13</f>
-        <v>3150</v>
+        <f aca="false">D5*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15+(D6+1)*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$14</f>
+        <v>4200</v>
       </c>
       <c r="E20" s="8" t="n">
-        <f aca="false">E5*Inputs!$B$12*Inputs!$B$14+(E6+1)*Inputs!$B$12*Inputs!$B$13</f>
-        <v>4200</v>
+        <f aca="false">E5*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15+(E6+1)*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$14</f>
+        <v>5600</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B21" s="8" t="n">
-        <f aca="false">B3*Inputs!$B$33</f>
+        <f aca="false">B3*Inputs!$B$34</f>
         <v>0</v>
       </c>
       <c r="C21" s="8" t="n">
-        <f aca="false">C3*Inputs!$B$33</f>
+        <f aca="false">C3*Inputs!$B$34</f>
         <v>0</v>
       </c>
       <c r="D21" s="8" t="n">
-        <f aca="false">D3*Inputs!$B$33</f>
+        <f aca="false">D3*Inputs!$B$34</f>
         <v>0</v>
       </c>
       <c r="E21" s="8" t="n">
-        <f aca="false">E3*Inputs!$B$33</f>
+        <f aca="false">E3*Inputs!$B$34</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B22" s="8" t="n">
-        <f aca="false">B5*Inputs!$B$15*Inputs!$B$17+(B6+1)*Inputs!$B$15*Inputs!$B$16</f>
+        <f aca="false">B5*Inputs!$B$16*Inputs!$B$18+(B6+1)*Inputs!$B$16*Inputs!$B$17</f>
         <v>624</v>
       </c>
       <c r="C22" s="8" t="n">
-        <f aca="false">C5*Inputs!$B$15*Inputs!$B$17+(C6+1)*Inputs!$B$15*Inputs!$B$16</f>
+        <f aca="false">C5*Inputs!$B$16*Inputs!$B$18+(C6+1)*Inputs!$B$16*Inputs!$B$17</f>
         <v>1040</v>
       </c>
       <c r="D22" s="8" t="n">
-        <f aca="false">D5*Inputs!$B$15*Inputs!$B$17+(D6+1)*Inputs!$B$15*Inputs!$B$16</f>
+        <f aca="false">D5*Inputs!$B$16*Inputs!$B$18+(D6+1)*Inputs!$B$16*Inputs!$B$17</f>
         <v>1560</v>
       </c>
       <c r="E22" s="8" t="n">
-        <f aca="false">E5*Inputs!$B$15*Inputs!$B$17+(E6+1)*Inputs!$B$15*Inputs!$B$16</f>
+        <f aca="false">E5*Inputs!$B$16*Inputs!$B$18+(E6+1)*Inputs!$B$16*Inputs!$B$17</f>
         <v>2080</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B23" s="8" t="n">
-        <f aca="false">B5*Inputs!$B$31</f>
+        <f aca="false">B5*Inputs!$B$32</f>
         <v>1380</v>
       </c>
       <c r="C23" s="8" t="n">
-        <f aca="false">C5*Inputs!$B$31</f>
+        <f aca="false">C5*Inputs!$B$32</f>
         <v>2300</v>
       </c>
       <c r="D23" s="8" t="n">
-        <f aca="false">D5*Inputs!$B$31</f>
+        <f aca="false">D5*Inputs!$B$32</f>
         <v>3450</v>
       </c>
       <c r="E23" s="8" t="n">
-        <f aca="false">E5*Inputs!$B$31</f>
+        <f aca="false">E5*Inputs!$B$32</f>
         <v>4600</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B24" s="8" t="n">
-        <f aca="false">B3*Inputs!$B$32</f>
-        <v>0</v>
+        <f aca="false">B3*Inputs!$B$33</f>
+        <v>600</v>
       </c>
       <c r="C24" s="8" t="n">
-        <f aca="false">C3*Inputs!$B$32</f>
-        <v>0</v>
+        <f aca="false">C3*Inputs!$B$33</f>
+        <v>1000</v>
       </c>
       <c r="D24" s="8" t="n">
-        <f aca="false">D3*Inputs!$B$32</f>
-        <v>0</v>
+        <f aca="false">D3*Inputs!$B$33</f>
+        <v>1500</v>
       </c>
       <c r="E24" s="8" t="n">
-        <f aca="false">E3*Inputs!$B$32</f>
-        <v>0</v>
+        <f aca="false">E3*Inputs!$B$33</f>
+        <v>2000</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B25" s="8" t="n">
-        <f aca="false">B7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
+        <f aca="false">B7*(Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)</f>
         <v>2952</v>
       </c>
       <c r="C25" s="8" t="n">
-        <f aca="false">C7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
+        <f aca="false">C7*(Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)</f>
         <v>4920</v>
       </c>
       <c r="D25" s="8" t="n">
-        <f aca="false">D7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
+        <f aca="false">D7*(Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)</f>
         <v>7380</v>
       </c>
       <c r="E25" s="8" t="n">
-        <f aca="false">E7*(Inputs!$B$25*Inputs!$B$27+Inputs!$B$26*Inputs!$B$28)</f>
+        <f aca="false">E7*(Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)</f>
         <v>9840</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B26" s="8" t="n">
-        <f aca="false">Inputs!$B$35</f>
+        <f aca="false">Inputs!$B$36</f>
         <v>700</v>
       </c>
       <c r="C26" s="8" t="n">
-        <f aca="false">Inputs!$B$35</f>
+        <f aca="false">Inputs!$B$36</f>
         <v>700</v>
       </c>
       <c r="D26" s="8" t="n">
-        <f aca="false">Inputs!$B$35</f>
+        <f aca="false">Inputs!$B$36</f>
         <v>700</v>
       </c>
       <c r="E26" s="8" t="n">
-        <f aca="false">Inputs!$B$35</f>
+        <f aca="false">Inputs!$B$36</f>
         <v>700</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B27" s="9" t="n">
         <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25+B26</f>
-        <v>13756</v>
+        <v>14776</v>
       </c>
       <c r="C27" s="9" t="n">
         <f aca="false">C18+C19+C20+C21+C22+C23+C24+C25+C26</f>
-        <v>22860</v>
+        <v>24560</v>
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
-        <v>33640</v>
+        <v>36190</v>
       </c>
       <c r="E27" s="9" t="n">
         <f aca="false">E18+E19+E20+E21+E22+E23+E24+E25+E26</f>
-        <v>44420</v>
+        <v>47820</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -2462,70 +2482,70 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">B9-B27</f>
-        <v>644</v>
+        <v>674</v>
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">C9-C27</f>
-        <v>1940</v>
+        <v>2090</v>
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">D9-D27</f>
-        <v>4160</v>
+        <v>4460</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">E9-E27</f>
-        <v>6380</v>
+        <v>6830</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B30" s="8" t="n">
         <f aca="false">B29/B4</f>
-        <v>58.5454545454546</v>
+        <v>61.2727272727273</v>
       </c>
       <c r="C30" s="8" t="n">
         <f aca="false">C29/C4</f>
-        <v>102.105263157895</v>
+        <v>110</v>
       </c>
       <c r="D30" s="8" t="n">
         <f aca="false">D29/D4</f>
-        <v>143.448275862069</v>
+        <v>153.793103448276</v>
       </c>
       <c r="E30" s="8" t="n">
         <f aca="false">E29/E4</f>
-        <v>163.589743589744</v>
+        <v>175.128205128205</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">B29/B9</f>
-        <v>0.0447222222222222</v>
+        <v>0.0436245954692557</v>
       </c>
       <c r="C31" s="11" t="n">
         <f aca="false">C29/C9</f>
-        <v>0.0782258064516129</v>
+        <v>0.0784240150093809</v>
       </c>
       <c r="D31" s="11" t="n">
         <f aca="false">D29/D9</f>
-        <v>0.11005291005291</v>
+        <v>0.109717097170972</v>
       </c>
       <c r="E31" s="11" t="n">
         <f aca="false">E29/E9</f>
-        <v>0.125590551181102</v>
+        <v>0.124977127172919</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B32" s="12" t="str">
         <f aca="false">IF(B29&gt;=0,"yes","NO")</f>
@@ -2546,7 +2566,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B33" s="9" t="n">
         <f aca="false">B19</f>
@@ -2567,7 +2587,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -2576,7 +2596,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">B4*400</f>
@@ -2597,28 +2617,28 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B36" s="8" t="n">
-        <f aca="false">B16*Inputs!$B$20+B25*Inputs!$B$29</f>
+        <f aca="false">B16*Inputs!$B$21+B25*Inputs!$B$30</f>
         <v>2448</v>
       </c>
       <c r="C36" s="8" t="n">
-        <f aca="false">C16*Inputs!$B$20+C25*Inputs!$B$29</f>
+        <f aca="false">C16*Inputs!$B$21+C25*Inputs!$B$30</f>
         <v>4180</v>
       </c>
       <c r="D36" s="8" t="n">
-        <f aca="false">D16*Inputs!$B$20+D25*Inputs!$B$29</f>
+        <f aca="false">D16*Inputs!$B$21+D25*Inputs!$B$30</f>
         <v>6195</v>
       </c>
       <c r="E36" s="8" t="n">
-        <f aca="false">E16*Inputs!$B$20+E25*Inputs!$B$29</f>
+        <f aca="false">E16*Inputs!$B$21+E25*Inputs!$B$30</f>
         <v>8210</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B37" s="9" t="n">
         <f aca="false">B35-B36</f>
@@ -2639,49 +2659,49 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">B9-B35</f>
-        <v>10000</v>
+        <v>11050</v>
       </c>
       <c r="C38" s="8" t="n">
         <f aca="false">C9-C35</f>
-        <v>17200</v>
+        <v>19050</v>
       </c>
       <c r="D38" s="8" t="n">
         <f aca="false">D9-D35</f>
-        <v>26200</v>
+        <v>29050</v>
       </c>
       <c r="E38" s="8" t="n">
         <f aca="false">E9-E35</f>
-        <v>35200</v>
+        <v>39050</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B39" s="8" t="n">
-        <f aca="false">B18-B16*Inputs!$B$20+B20+B25*(1-Inputs!$B$29)+B23+B24</f>
-        <v>9684</v>
+        <f aca="false">B18-B16*Inputs!$B$21+B20+B25*(1-Inputs!$B$30)+B23+B24</f>
+        <v>10704</v>
       </c>
       <c r="C39" s="8" t="n">
-        <f aca="false">C18-C16*Inputs!$B$20+C20+C25*(1-Inputs!$B$29)+C23+C24</f>
-        <v>16400</v>
+        <f aca="false">C18-C16*Inputs!$B$21+C20+C25*(1-Inputs!$B$30)+C23+C24</f>
+        <v>18100</v>
       </c>
       <c r="D39" s="8" t="n">
-        <f aca="false">D18-D16*Inputs!$B$20+D20+D25*(1-Inputs!$B$29)+D23+D24</f>
-        <v>24345</v>
+        <f aca="false">D18-D16*Inputs!$B$21+D20+D25*(1-Inputs!$B$30)+D23+D24</f>
+        <v>26895</v>
       </c>
       <c r="E39" s="8" t="n">
-        <f aca="false">E18-E16*Inputs!$B$20+E20+E25*(1-Inputs!$B$29)+E23+E24</f>
-        <v>32290</v>
+        <f aca="false">E18-E16*Inputs!$B$21+E20+E25*(1-Inputs!$B$30)+E23+E24</f>
+        <v>35690</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B40" s="8" t="n">
         <f aca="false">B22</f>
@@ -2702,7 +2722,7 @@
     </row>
     <row r="41" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -2735,108 +2755,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2846,10 +2866,10 @@
     </row>
     <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>10</v>
@@ -2857,10 +2877,10 @@
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Blue Note: two boats blocked, alternating boats agreed, shore dive 60, DAN Business Member; Sand Dollar rental 20; late-start reef question sent to Paradise
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="187">
   <si>
     <t xml:space="preserve">Cozumel group budget — inputs (blue cells are editable)</t>
   </si>
@@ -157,6 +157,12 @@
     <t xml:space="preserve">Private night charter, up to 10 divers (optional add-on, shared)</t>
   </si>
   <si>
+    <t xml:space="preserve">Shore dive at Tikila Beach Bar incl. gear (optional add-on on the free mornings)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 24 Sep</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nitrox fill per tank (course free with eLearning)</t>
   </si>
   <si>
@@ -205,10 +211,10 @@
     <t xml:space="preserve">ADVERTISED store.padi.com about USD 230; Blue Note asked for its code price</t>
   </si>
   <si>
-    <t xml:space="preserve">Dive-accident cover inside the fee (DAN short-term 6–10 day plan via the shop, one roster)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED plan price; ASSUMED Blue Note sells it (asked 24 Sep). If not: 0 here and each person buys DAN Master (84)</t>
+    <t xml:space="preserve">Dive-accident cover inside the fee (DAN short-term plan via Blue Note, a DAN Business Member)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED plan price; Blue Note confirmed 24 Sep it is a DAN Business Member and is pricing cover for the certified divers; OW students are covered during the course</t>
   </si>
   <si>
     <t xml:space="preserve">Tax buffer per head</t>
@@ -344,6 +350,9 @@
   </si>
   <si>
     <t xml:space="preserve">Night dive, private charter shared by 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shore dive on a free morning, incl. gear</t>
   </si>
   <si>
     <t xml:space="preserve">GUIDANCE BUDGET WITHOUT FLIGHTS</t>
@@ -986,7 +995,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72"/>
@@ -1303,7 +1312,7 @@
         <v>44</v>
       </c>
       <c r="B24" s="7" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>17</v>
@@ -1313,33 +1322,33 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
+      <c r="B25" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B26" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D26" s="2" t="s">
+      <c r="A26" s="4" t="s">
         <v>48</v>
       </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
         <v>49</v>
       </c>
       <c r="B27" s="7" t="n">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>17</v>
@@ -1352,70 +1361,70 @@
       <c r="A28" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B28" s="5" t="n">
-        <v>2</v>
+      <c r="B28" s="7" t="n">
+        <v>88</v>
       </c>
       <c r="C28" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D29" s="2"/>
+      <c r="D29" s="2" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B30" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="6" t="n">
         <v>0.25</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-    </row>
-    <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+      <c r="D31" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B32" s="7" t="n">
-        <v>230</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D32" s="2" t="s">
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
         <v>59</v>
       </c>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
         <v>60</v>
       </c>
       <c r="B33" s="7" t="n">
-        <v>50</v>
+        <v>230</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>17</v>
@@ -1424,12 +1433,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B34" s="7" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>17</v>
@@ -1439,34 +1448,33 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
+      <c r="B35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B36" s="7" t="n">
-        <v>700</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D36" s="2" t="s">
+      <c r="A36" s="4" t="s">
         <v>66</v>
       </c>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
         <v>67</v>
       </c>
       <c r="B37" s="7" t="n">
-        <f aca="false">(Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)/2</f>
-        <v>246</v>
+        <v>700</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>17</v>
@@ -1480,7 +1488,7 @@
         <v>69</v>
       </c>
       <c r="B38" s="7" t="n">
-        <f aca="false">Inputs!$B$37</f>
+        <f aca="false">(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)/2</f>
         <v>246</v>
       </c>
       <c r="C38" s="2" t="s">
@@ -1495,7 +1503,8 @@
         <v>71</v>
       </c>
       <c r="B39" s="7" t="n">
-        <v>50</v>
+        <f aca="false">Inputs!$B$38</f>
+        <v>246</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>17</v>
@@ -1509,70 +1518,70 @@
         <v>73</v>
       </c>
       <c r="B40" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B41" s="7" t="n">
         <f aca="false">(Inputs!$B$12+Inputs!$B$13)*5</f>
         <v>200</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C41" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
+      <c r="D41" s="2" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B42" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D42" s="2" t="s">
+      <c r="A42" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B43" s="5" t="n">
-        <v>6</v>
+      <c r="B43" s="7" t="n">
+        <v>45</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D43" s="2"/>
+        <v>22</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B44" s="7" t="n">
-        <v>50</v>
+        <v>79</v>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>79</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="D44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
         <v>80</v>
       </c>
       <c r="B45" s="7" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>17</v>
@@ -1581,12 +1590,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
         <v>82</v>
       </c>
       <c r="B46" s="7" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>17</v>
@@ -1595,18 +1604,32 @@
         <v>83</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B47" s="7" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>85</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1634,7 +1657,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1642,15 +1665,15 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">Inputs!$B$9+Inputs!$B$10</f>
@@ -1663,7 +1686,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15</f>
@@ -1676,7 +1699,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">Inputs!$B$16*Inputs!$B$18</f>
@@ -1689,71 +1712,71 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B6" s="8" t="n">
-        <f aca="false">Inputs!$B$34</f>
+        <f aca="false">Inputs!$B$35</f>
         <v>0</v>
       </c>
       <c r="C6" s="8" t="n">
-        <f aca="false">Inputs!$B$34</f>
+        <f aca="false">Inputs!$B$35</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B7" s="8" t="n">
-        <f aca="false">Inputs!$B$32</f>
+        <f aca="false">Inputs!$B$33</f>
         <v>230</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B8" s="8" t="n">
-        <f aca="false">Inputs!$B$33</f>
+        <f aca="false">Inputs!$B$34</f>
         <v>50</v>
       </c>
       <c r="C8" s="8" t="n">
-        <f aca="false">Inputs!$B$33</f>
+        <f aca="false">Inputs!$B$34</f>
         <v>50</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B9" s="8" t="n">
-        <f aca="false">((Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)/2)</f>
+        <f aca="false">((Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)/2)</f>
         <v>246</v>
       </c>
       <c r="C9" s="8" t="n">
-        <f aca="false">((Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)/2)</f>
+        <f aca="false">((Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)/2)</f>
         <v>246</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B10" s="8" t="n">
-        <f aca="false">(Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39+Inputs!$B$40)/(Inputs!$B$4-1)</f>
+        <f aca="false">(Inputs!$B$37+Inputs!$B$38+Inputs!$B$39+Inputs!$B$40+Inputs!$B$41)/(Inputs!$B$4-1)</f>
         <v>75.8947368421053</v>
       </c>
       <c r="C10" s="8" t="n">
-        <f aca="false">(Inputs!$B$36+Inputs!$B$37+Inputs!$B$38+Inputs!$B$39+Inputs!$B$40)/(Inputs!$B$4-1)</f>
+        <f aca="false">(Inputs!$B$37+Inputs!$B$38+Inputs!$B$39+Inputs!$B$40+Inputs!$B$41)/(Inputs!$B$4-1)</f>
         <v>75.8947368421053</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">SUM(B3:B10)</f>
@@ -1766,7 +1789,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">ROUND(B11*Inputs!$B$7,0)</f>
@@ -1779,7 +1802,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">CEILING(B11+B12,50)</f>
@@ -1797,38 +1820,38 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C16" s="8" t="n">
-        <f aca="false">Inputs!$B$47</f>
+        <f aca="false">Inputs!$B$48</f>
         <v>220</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C17" s="8" t="n">
-        <f aca="false">Inputs!$B$24*10</f>
+        <f aca="false">Inputs!$B$25*10</f>
         <v>120</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">Inputs!$B$22+Inputs!$B$16</f>
@@ -1841,7 +1864,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">Inputs!$B$23/10</f>
@@ -1853,76 +1876,84 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
+      <c r="A20" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" s="8" t="n">
+        <f aca="false">Inputs!$B$24</f>
+        <v>60</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <f aca="false">Inputs!$B$24</f>
+        <v>60</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>107</v>
-      </c>
+      <c r="A21" s="4"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B22" s="8" t="n">
+        <v>110</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B23" s="8" t="n">
         <f aca="false">B13</f>
         <v>1450</v>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C23" s="8" t="n">
         <f aca="false">C13</f>
         <v>1350</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B23" s="8" t="n">
-        <f aca="false">Inputs!$B$46+Inputs!$B$42*Inputs!$B$43+Inputs!$B$44+Inputs!$B$45</f>
+    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="9" t="n">
+        <f aca="false">Inputs!$B$47+Inputs!$B$43*Inputs!$B$44+Inputs!$B$45+Inputs!$B$46</f>
         <v>350</v>
       </c>
-      <c r="C23" s="8" t="n">
-        <f aca="false">Inputs!$B$46+Inputs!$B$42*Inputs!$B$43+Inputs!$B$44+Inputs!$B$45</f>
+      <c r="C24" s="9" t="n">
+        <f aca="false">Inputs!$B$47+Inputs!$B$43*Inputs!$B$44+Inputs!$B$45+Inputs!$B$46</f>
         <v>350</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B24" s="9" t="n">
-        <f aca="false">B22+B23</f>
-        <v>1800</v>
-      </c>
-      <c r="C24" s="9" t="n">
-        <f aca="false">C22+C23</f>
-        <v>1700</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>103</v>
+        <v>113</v>
+      </c>
+      <c r="B25" s="9" t="n">
+        <f aca="false">B22+B23</f>
+        <v>1450</v>
       </c>
       <c r="C25" s="9" t="n">
+        <f aca="false">C22+C23</f>
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C26" s="8" t="n">
         <f aca="false">C24+C16+C17</f>
-        <v>2040</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
+        <v>690</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1952,7 +1983,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1962,21 +1993,21 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>12</v>
@@ -1993,7 +2024,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
@@ -2014,7 +2045,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$6,0)</f>
@@ -2035,7 +2066,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">B4-B5</f>
@@ -2056,7 +2087,7 @@
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">ROUNDUP(B3/2,0)</f>
@@ -2077,7 +2108,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2086,7 +2117,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">B5*Fee!$B$13+B6*Fee!$C$13</f>
@@ -2107,7 +2138,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2116,7 +2147,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$9+Inputs!$B$10)</f>
@@ -2137,7 +2168,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B6*Inputs!$B$11</f>
@@ -2158,7 +2189,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">INT(B6/Inputs!$B$20)</f>
@@ -2179,7 +2210,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">IF(B13&gt;=1,0,Inputs!$B$11)</f>
@@ -2200,7 +2231,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">-MAX(B13-1,0)*Inputs!$B$11</f>
@@ -2221,7 +2252,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B11+B12+B14+B15</f>
@@ -2242,7 +2273,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">-B12*Inputs!$B$19</f>
@@ -2263,7 +2294,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B16+B17</f>
@@ -2284,7 +2315,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-B17</f>
@@ -2305,7 +2336,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15+(B6+1)*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$14</f>
@@ -2326,28 +2357,28 @@
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B21" s="8" t="n">
-        <f aca="false">B3*Inputs!$B$34</f>
+        <f aca="false">B3*Inputs!$B$35</f>
         <v>0</v>
       </c>
       <c r="C21" s="8" t="n">
-        <f aca="false">C3*Inputs!$B$34</f>
+        <f aca="false">C3*Inputs!$B$35</f>
         <v>0</v>
       </c>
       <c r="D21" s="8" t="n">
-        <f aca="false">D3*Inputs!$B$34</f>
+        <f aca="false">D3*Inputs!$B$35</f>
         <v>0</v>
       </c>
       <c r="E21" s="8" t="n">
-        <f aca="false">E3*Inputs!$B$34</f>
+        <f aca="false">E3*Inputs!$B$35</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B5*Inputs!$B$16*Inputs!$B$18+(B6+1)*Inputs!$B$16*Inputs!$B$17</f>
@@ -2368,91 +2399,91 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B23" s="8" t="n">
-        <f aca="false">B5*Inputs!$B$32</f>
+        <f aca="false">B5*Inputs!$B$33</f>
         <v>1380</v>
       </c>
       <c r="C23" s="8" t="n">
-        <f aca="false">C5*Inputs!$B$32</f>
+        <f aca="false">C5*Inputs!$B$33</f>
         <v>2300</v>
       </c>
       <c r="D23" s="8" t="n">
-        <f aca="false">D5*Inputs!$B$32</f>
+        <f aca="false">D5*Inputs!$B$33</f>
         <v>3450</v>
       </c>
       <c r="E23" s="8" t="n">
-        <f aca="false">E5*Inputs!$B$32</f>
+        <f aca="false">E5*Inputs!$B$33</f>
         <v>4600</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B24" s="8" t="n">
-        <f aca="false">B3*Inputs!$B$33</f>
+        <f aca="false">B3*Inputs!$B$34</f>
         <v>600</v>
       </c>
       <c r="C24" s="8" t="n">
-        <f aca="false">C3*Inputs!$B$33</f>
+        <f aca="false">C3*Inputs!$B$34</f>
         <v>1000</v>
       </c>
       <c r="D24" s="8" t="n">
-        <f aca="false">D3*Inputs!$B$33</f>
+        <f aca="false">D3*Inputs!$B$34</f>
         <v>1500</v>
       </c>
       <c r="E24" s="8" t="n">
-        <f aca="false">E3*Inputs!$B$33</f>
+        <f aca="false">E3*Inputs!$B$34</f>
         <v>2000</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B25" s="8" t="n">
-        <f aca="false">B7*(Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)</f>
+        <f aca="false">B7*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
         <v>2952</v>
       </c>
       <c r="C25" s="8" t="n">
-        <f aca="false">C7*(Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)</f>
+        <f aca="false">C7*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
         <v>4920</v>
       </c>
       <c r="D25" s="8" t="n">
-        <f aca="false">D7*(Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)</f>
+        <f aca="false">D7*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
         <v>7380</v>
       </c>
       <c r="E25" s="8" t="n">
-        <f aca="false">E7*(Inputs!$B$26*Inputs!$B$28+Inputs!$B$27*Inputs!$B$29)</f>
+        <f aca="false">E7*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
         <v>9840</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B26" s="8" t="n">
-        <f aca="false">Inputs!$B$36</f>
+        <f aca="false">Inputs!$B$37</f>
         <v>700</v>
       </c>
       <c r="C26" s="8" t="n">
-        <f aca="false">Inputs!$B$36</f>
+        <f aca="false">Inputs!$B$37</f>
         <v>700</v>
       </c>
       <c r="D26" s="8" t="n">
-        <f aca="false">Inputs!$B$36</f>
+        <f aca="false">Inputs!$B$37</f>
         <v>700</v>
       </c>
       <c r="E26" s="8" t="n">
-        <f aca="false">Inputs!$B$36</f>
+        <f aca="false">Inputs!$B$37</f>
         <v>700</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B27" s="9" t="n">
         <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25+B26</f>
@@ -2473,7 +2504,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -2482,7 +2513,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">B9-B27</f>
@@ -2503,7 +2534,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B30" s="8" t="n">
         <f aca="false">B29/B4</f>
@@ -2524,7 +2555,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">B29/B9</f>
@@ -2545,7 +2576,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B32" s="12" t="str">
         <f aca="false">IF(B29&gt;=0,"yes","NO")</f>
@@ -2566,7 +2597,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B33" s="9" t="n">
         <f aca="false">B19</f>
@@ -2587,7 +2618,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -2596,7 +2627,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">B4*400</f>
@@ -2617,28 +2648,28 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B36" s="8" t="n">
-        <f aca="false">B16*Inputs!$B$21+B25*Inputs!$B$30</f>
+        <f aca="false">B16*Inputs!$B$21+B25*Inputs!$B$31</f>
         <v>2448</v>
       </c>
       <c r="C36" s="8" t="n">
-        <f aca="false">C16*Inputs!$B$21+C25*Inputs!$B$30</f>
+        <f aca="false">C16*Inputs!$B$21+C25*Inputs!$B$31</f>
         <v>4180</v>
       </c>
       <c r="D36" s="8" t="n">
-        <f aca="false">D16*Inputs!$B$21+D25*Inputs!$B$30</f>
+        <f aca="false">D16*Inputs!$B$21+D25*Inputs!$B$31</f>
         <v>6195</v>
       </c>
       <c r="E36" s="8" t="n">
-        <f aca="false">E16*Inputs!$B$21+E25*Inputs!$B$30</f>
+        <f aca="false">E16*Inputs!$B$21+E25*Inputs!$B$31</f>
         <v>8210</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B37" s="9" t="n">
         <f aca="false">B35-B36</f>
@@ -2659,7 +2690,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">B9-B35</f>
@@ -2680,28 +2711,28 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B39" s="8" t="n">
-        <f aca="false">B18-B16*Inputs!$B$21+B20+B25*(1-Inputs!$B$30)+B23+B24</f>
+        <f aca="false">B18-B16*Inputs!$B$21+B20+B25*(1-Inputs!$B$31)+B23+B24</f>
         <v>10704</v>
       </c>
       <c r="C39" s="8" t="n">
-        <f aca="false">C18-C16*Inputs!$B$21+C20+C25*(1-Inputs!$B$30)+C23+C24</f>
+        <f aca="false">C18-C16*Inputs!$B$21+C20+C25*(1-Inputs!$B$31)+C23+C24</f>
         <v>18100</v>
       </c>
       <c r="D39" s="8" t="n">
-        <f aca="false">D18-D16*Inputs!$B$21+D20+D25*(1-Inputs!$B$30)+D23+D24</f>
+        <f aca="false">D18-D16*Inputs!$B$21+D20+D25*(1-Inputs!$B$31)+D23+D24</f>
         <v>26895</v>
       </c>
       <c r="E39" s="8" t="n">
-        <f aca="false">E18-E16*Inputs!$B$21+E20+E25*(1-Inputs!$B$30)+E23+E24</f>
+        <f aca="false">E18-E16*Inputs!$B$21+E20+E25*(1-Inputs!$B$31)+E23+E24</f>
         <v>35690</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B40" s="8" t="n">
         <f aca="false">B22</f>
@@ -2722,7 +2753,7 @@
     </row>
     <row r="41" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -2755,108 +2786,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2866,10 +2897,10 @@
     </row>
     <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>10</v>
@@ -2877,10 +2908,10 @@
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Cozumel: DAN out of the fee (shop cannot sell it), Hotel Plaza 20 rooms blocked with comp rule, Casa Mexicana re-quote, hotel comparison for George; Casa del Mar chased
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="190">
   <si>
     <t xml:space="preserve">Cozumel group budget — inputs (blue cells are editable)</t>
   </si>
@@ -202,6 +202,15 @@
     <t xml:space="preserve">QUOTE NEEDED; assumption</t>
   </si>
   <si>
+    <t xml:space="preserve">Hotel Plaza: one complimentary room per N paid rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 25 Sep via Blue Note (20 rooms blocked)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Included in the fee for everyone</t>
   </si>
   <si>
@@ -211,10 +220,10 @@
     <t xml:space="preserve">ADVERTISED store.padi.com about USD 230; Blue Note asked for its code price</t>
   </si>
   <si>
-    <t xml:space="preserve">Dive-accident cover inside the fee (DAN short-term plan via Blue Note, a DAN Business Member)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED plan price; Blue Note confirmed 24 Sep it is a DAN Business Member and is pricing cover for the certified divers; OW students are covered during the course</t>
+    <t xml:space="preserve">Dive-accident cover inside the fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 25 Sep: DAN no longer lets shops buy cover for divers; each person buys their own (own spending below); OW students covered by the shop during the course only</t>
   </si>
   <si>
     <t xml:space="preserve">Tax buffer per head</t>
@@ -247,7 +256,7 @@
     <t xml:space="preserve">George's dive cover carried by the group</t>
   </si>
   <si>
-    <t xml:space="preserve">same plan as everyone</t>
+    <t xml:space="preserve">own cost like everyone (25 Sep)</t>
   </si>
   <si>
     <t xml:space="preserve">George's gear and computer rental, 5 days</t>
@@ -277,10 +286,10 @@
     <t xml:space="preserve">ADVERTISED shared van 15 each way</t>
   </si>
   <si>
-    <t xml:space="preserve">Dive cover bought by each person (only if the shop cannot sell the short-term plan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0 while cover is inside the fee; 84 (DAN membership + Master) if it moves out</t>
+    <t xml:space="preserve">Dive cover bought by each person via Blue Note's DAN link (membership 40 + Master 44)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED; required, proof collected at sign-up</t>
   </si>
   <si>
     <t xml:space="preserve">PADI AOW eLearning (add-on for AOW takers)</t>
@@ -316,7 +325,7 @@
     <t xml:space="preserve">0</t>
   </si>
   <si>
-    <t xml:space="preserve">Dive-accident cover (DAN short-term plan via the shop, assumed)</t>
+    <t xml:space="preserve">Dive-accident cover (not in the fee: each person buys their own, see below)</t>
   </si>
   <si>
     <t xml:space="preserve">Hotel Plaza, 6 nights with breakfast, 2 sharing</t>
@@ -361,7 +370,7 @@
     <t xml:space="preserve">Trip fee</t>
   </si>
   <si>
-    <t xml:space="preserve">Own spending: meals, drinks, tips, airport transfers (own dive cover only if it leaves the fee)</t>
+    <t xml:space="preserve">Own spending: DAN cover, meals, drinks, tips, airport transfers</t>
   </si>
   <si>
     <t xml:space="preserve">Guidance budget</t>
@@ -370,7 +379,7 @@
     <t xml:space="preserve">Guidance budget, certified taking AOW and nitrox</t>
   </si>
   <si>
-    <t xml:space="preserve">The fee covers everything diving-related (course or package, gear and computer, park fees, eLearning), dive-accident cover bought through the shop, and the hotel; flights, meals, drinks, tips and transfers are the person's own. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
+    <t xml:space="preserve">The fee covers everything diving-related (course or package, gear and computer, park fees, eLearning) and the hotel; flights, the required DAN cover (bought by each person), meals, drinks, tips and transfers are the person's own. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
   </si>
   <si>
     <t xml:space="preserve">Group budget at four sizes (half students; George leads and does not pay)</t>
@@ -454,7 +463,7 @@
     <t xml:space="preserve">Dive cover for everyone including George (short-term plan via the shop)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hotel Plaza block, all rooms</t>
+    <t xml:space="preserve">Hotel Plaza block, all rooms, less one comp room per 14 paid</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL COSTS</t>
@@ -995,7 +1004,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72"/>
@@ -1412,44 +1421,44 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-    </row>
-    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+      <c r="B32" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B33" s="7" t="n">
+      <c r="D32" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B34" s="7" t="n">
         <v>230</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B34" s="7" t="n">
-        <v>50</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B35" s="7" t="n">
         <v>0</v>
@@ -1458,178 +1467,192 @@
         <v>17</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
+      <c r="A36" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B37" s="7" t="n">
-        <v>700</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>68</v>
-      </c>
+      <c r="A37" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B38" s="7" t="n">
+        <v>700</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B39" s="7" t="n">
         <f aca="false">(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)/2</f>
         <v>246</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B39" s="7" t="n">
-        <f aca="false">Inputs!$B$38</f>
-        <v>246</v>
-      </c>
       <c r="C39" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B40" s="7" t="n">
-        <v>50</v>
+        <f aca="false">Inputs!$B$39</f>
+        <v>246</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" s="7" t="n">
         <f aca="false">(Inputs!$B$12+Inputs!$B$13)*5</f>
         <v>200</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C42" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
+      <c r="D42" s="2" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B43" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="A43" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B44" s="5" t="n">
-        <v>6</v>
+        <v>80</v>
+      </c>
+      <c r="B44" s="7" t="n">
+        <v>45</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D44" s="2"/>
+        <v>22</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B45" s="7" t="n">
-        <v>50</v>
+        <v>82</v>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>81</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="D45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B46" s="7" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B47" s="7" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B48" s="7" t="n">
-        <v>220</v>
+        <v>84</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1648,7 +1671,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -1657,7 +1680,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1665,15 +1688,15 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">Inputs!$B$9+Inputs!$B$10</f>
@@ -1686,7 +1709,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15</f>
@@ -1699,7 +1722,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">Inputs!$B$16*Inputs!$B$18</f>
@@ -1712,45 +1735,45 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B6" s="8" t="n">
+        <f aca="false">Inputs!$B$36</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <f aca="false">Inputs!$B$36</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <f aca="false">Inputs!$B$34</f>
+        <v>230</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="8" t="n">
         <f aca="false">Inputs!$B$35</f>
         <v>0</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C8" s="8" t="n">
         <f aca="false">Inputs!$B$35</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B7" s="8" t="n">
-        <f aca="false">Inputs!$B$33</f>
-        <v>230</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B8" s="8" t="n">
-        <f aca="false">Inputs!$B$34</f>
-        <v>50</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <f aca="false">Inputs!$B$34</f>
-        <v>50</v>
-      </c>
-    </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">((Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)/2)</f>
@@ -1763,54 +1786,54 @@
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B10" s="8" t="n">
-        <f aca="false">(Inputs!$B$37+Inputs!$B$38+Inputs!$B$39+Inputs!$B$40+Inputs!$B$41)/(Inputs!$B$4-1)</f>
-        <v>75.8947368421053</v>
+        <f aca="false">(Inputs!$B$38+Inputs!$B$39+Inputs!$B$40+Inputs!$B$41+Inputs!$B$42)/(Inputs!$B$4-1)</f>
+        <v>73.2631578947368</v>
       </c>
       <c r="C10" s="8" t="n">
-        <f aca="false">(Inputs!$B$37+Inputs!$B$38+Inputs!$B$39+Inputs!$B$40+Inputs!$B$41)/(Inputs!$B$4-1)</f>
-        <v>75.8947368421053</v>
+        <f aca="false">(Inputs!$B$38+Inputs!$B$39+Inputs!$B$40+Inputs!$B$41+Inputs!$B$42)/(Inputs!$B$4-1)</f>
+        <v>73.2631578947368</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">SUM(B3:B10)</f>
-        <v>1360.89473684211</v>
+        <v>1308.26315789474</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">SUM(C3:C10)</f>
-        <v>1236.89473684211</v>
+        <v>1184.26315789474</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">ROUND(B11*Inputs!$B$7,0)</f>
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">ROUND(C11*Inputs!$B$7,0)</f>
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">CEILING(B11+B12,50)</f>
-        <v>1450</v>
+        <v>1400</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">CEILING(C11+C12,50)</f>
-        <v>1350</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1820,29 +1843,29 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C16" s="8" t="n">
-        <f aca="false">Inputs!$B$48</f>
+        <f aca="false">Inputs!$B$49</f>
         <v>220</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">Inputs!$B$25*10</f>
@@ -1851,7 +1874,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">Inputs!$B$22+Inputs!$B$16</f>
@@ -1864,7 +1887,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">Inputs!$B$23/10</f>
@@ -1877,7 +1900,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">Inputs!$B$24</f>
@@ -1889,74 +1912,79 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
+      <c r="A21" s="2"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="B23" s="8" t="n">
+      <c r="A23" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="9" t="n">
         <f aca="false">B13</f>
-        <v>1450</v>
-      </c>
-      <c r="C23" s="8" t="n">
+        <v>1400</v>
+      </c>
+      <c r="C23" s="9" t="n">
         <f aca="false">C13</f>
-        <v>1350</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="B24" s="9" t="n">
-        <f aca="false">Inputs!$B$47+Inputs!$B$43*Inputs!$B$44+Inputs!$B$45+Inputs!$B$46</f>
-        <v>350</v>
-      </c>
-      <c r="C24" s="9" t="n">
-        <f aca="false">Inputs!$B$47+Inputs!$B$43*Inputs!$B$44+Inputs!$B$45+Inputs!$B$46</f>
-        <v>350</v>
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <f aca="false">Inputs!$B$48+Inputs!$B$44*Inputs!$B$45+Inputs!$B$46+Inputs!$B$47</f>
+        <v>434</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <f aca="false">Inputs!$B$48+Inputs!$B$44*Inputs!$B$45+Inputs!$B$46+Inputs!$B$47</f>
+        <v>434</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B25" s="9" t="n">
-        <f aca="false">B22+B23</f>
-        <v>1450</v>
+        <f aca="false">B23+B24</f>
+        <v>1834</v>
       </c>
       <c r="C25" s="9" t="n">
-        <f aca="false">C22+C23</f>
-        <v>1350</v>
+        <f aca="false">C23+C24</f>
+        <v>1734</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="C26" s="8" t="n">
-        <f aca="false">C24+C16+C17</f>
-        <v>690</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>115</v>
-      </c>
+      <c r="A26" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <f aca="false">C25+C16+C17</f>
+        <v>2074</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
+    </row>
+    <row r="28" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1983,7 +2011,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1993,21 +2021,21 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>12</v>
@@ -2024,7 +2052,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
@@ -2045,7 +2073,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$6,0)</f>
@@ -2066,7 +2094,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">B4-B5</f>
@@ -2087,7 +2115,7 @@
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">ROUNDUP(B3/2,0)</f>
@@ -2108,7 +2136,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2117,28 +2145,28 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">B5*Fee!$B$13+B6*Fee!$C$13</f>
-        <v>15450</v>
+        <v>14900</v>
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">C5*Fee!$B$13+C6*Fee!$C$13</f>
-        <v>26650</v>
+        <v>25700</v>
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">D5*Fee!$B$13+D6*Fee!$C$13</f>
-        <v>40650</v>
+        <v>39200</v>
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">E5*Fee!$B$13+E6*Fee!$C$13</f>
-        <v>54650</v>
+        <v>52700</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2147,7 +2175,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$9+Inputs!$B$10)</f>
@@ -2168,7 +2196,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B6*Inputs!$B$11</f>
@@ -2189,7 +2217,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">INT(B6/Inputs!$B$20)</f>
@@ -2210,7 +2238,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">IF(B13&gt;=1,0,Inputs!$B$11)</f>
@@ -2231,7 +2259,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">-MAX(B13-1,0)*Inputs!$B$11</f>
@@ -2252,7 +2280,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B11+B12+B14+B15</f>
@@ -2273,7 +2301,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">-B12*Inputs!$B$19</f>
@@ -2294,7 +2322,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B16+B17</f>
@@ -2315,7 +2343,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-B17</f>
@@ -2336,7 +2364,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15+(B6+1)*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$14</f>
@@ -2357,28 +2385,28 @@
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B21" s="8" t="n">
-        <f aca="false">B3*Inputs!$B$35</f>
+        <f aca="false">B3*Inputs!$B$36</f>
         <v>0</v>
       </c>
       <c r="C21" s="8" t="n">
-        <f aca="false">C3*Inputs!$B$35</f>
+        <f aca="false">C3*Inputs!$B$36</f>
         <v>0</v>
       </c>
       <c r="D21" s="8" t="n">
-        <f aca="false">D3*Inputs!$B$35</f>
+        <f aca="false">D3*Inputs!$B$36</f>
         <v>0</v>
       </c>
       <c r="E21" s="8" t="n">
-        <f aca="false">E3*Inputs!$B$35</f>
+        <f aca="false">E3*Inputs!$B$36</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B5*Inputs!$B$16*Inputs!$B$18+(B6+1)*Inputs!$B$16*Inputs!$B$17</f>
@@ -2399,112 +2427,112 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B23" s="8" t="n">
-        <f aca="false">B5*Inputs!$B$33</f>
+        <f aca="false">B5*Inputs!$B$34</f>
         <v>1380</v>
       </c>
       <c r="C23" s="8" t="n">
-        <f aca="false">C5*Inputs!$B$33</f>
+        <f aca="false">C5*Inputs!$B$34</f>
         <v>2300</v>
       </c>
       <c r="D23" s="8" t="n">
-        <f aca="false">D5*Inputs!$B$33</f>
+        <f aca="false">D5*Inputs!$B$34</f>
         <v>3450</v>
       </c>
       <c r="E23" s="8" t="n">
-        <f aca="false">E5*Inputs!$B$33</f>
+        <f aca="false">E5*Inputs!$B$34</f>
         <v>4600</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B24" s="8" t="n">
-        <f aca="false">B3*Inputs!$B$34</f>
-        <v>600</v>
+        <f aca="false">B3*Inputs!$B$35</f>
+        <v>0</v>
       </c>
       <c r="C24" s="8" t="n">
-        <f aca="false">C3*Inputs!$B$34</f>
-        <v>1000</v>
+        <f aca="false">C3*Inputs!$B$35</f>
+        <v>0</v>
       </c>
       <c r="D24" s="8" t="n">
-        <f aca="false">D3*Inputs!$B$34</f>
-        <v>1500</v>
+        <f aca="false">D3*Inputs!$B$35</f>
+        <v>0</v>
       </c>
       <c r="E24" s="8" t="n">
-        <f aca="false">E3*Inputs!$B$34</f>
-        <v>2000</v>
+        <f aca="false">E3*Inputs!$B$35</f>
+        <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B25" s="8" t="n">
-        <f aca="false">B7*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
+        <f aca="false">(B7-INT(B7/(Inputs!$B$32+1)))*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
         <v>2952</v>
       </c>
       <c r="C25" s="8" t="n">
-        <f aca="false">C7*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
+        <f aca="false">(C7-INT(C7/(Inputs!$B$32+1)))*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
         <v>4920</v>
       </c>
       <c r="D25" s="8" t="n">
-        <f aca="false">D7*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
-        <v>7380</v>
+        <f aca="false">(D7-INT(D7/(Inputs!$B$32+1)))*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
+        <v>6888</v>
       </c>
       <c r="E25" s="8" t="n">
-        <f aca="false">E7*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
-        <v>9840</v>
+        <f aca="false">(E7-INT(E7/(Inputs!$B$32+1)))*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
+        <v>9348</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B26" s="8" t="n">
-        <f aca="false">Inputs!$B$37</f>
+        <f aca="false">Inputs!$B$38</f>
         <v>700</v>
       </c>
       <c r="C26" s="8" t="n">
-        <f aca="false">Inputs!$B$37</f>
+        <f aca="false">Inputs!$B$38</f>
         <v>700</v>
       </c>
       <c r="D26" s="8" t="n">
-        <f aca="false">Inputs!$B$37</f>
+        <f aca="false">Inputs!$B$38</f>
         <v>700</v>
       </c>
       <c r="E26" s="8" t="n">
-        <f aca="false">Inputs!$B$37</f>
+        <f aca="false">Inputs!$B$38</f>
         <v>700</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B27" s="9" t="n">
         <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25+B26</f>
-        <v>14776</v>
+        <v>14176</v>
       </c>
       <c r="C27" s="9" t="n">
         <f aca="false">C18+C19+C20+C21+C22+C23+C24+C25+C26</f>
-        <v>24560</v>
+        <v>23560</v>
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
-        <v>36190</v>
+        <v>34198</v>
       </c>
       <c r="E27" s="9" t="n">
         <f aca="false">E18+E19+E20+E21+E22+E23+E24+E25+E26</f>
-        <v>47820</v>
+        <v>45328</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -2513,70 +2541,70 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">B9-B27</f>
-        <v>674</v>
+        <v>724</v>
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">C9-C27</f>
-        <v>2090</v>
+        <v>2140</v>
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">D9-D27</f>
-        <v>4460</v>
+        <v>5002</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">E9-E27</f>
-        <v>6830</v>
+        <v>7372</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B30" s="8" t="n">
         <f aca="false">B29/B4</f>
-        <v>61.2727272727273</v>
+        <v>65.8181818181818</v>
       </c>
       <c r="C30" s="8" t="n">
         <f aca="false">C29/C4</f>
-        <v>110</v>
+        <v>112.631578947368</v>
       </c>
       <c r="D30" s="8" t="n">
         <f aca="false">D29/D4</f>
-        <v>153.793103448276</v>
+        <v>172.48275862069</v>
       </c>
       <c r="E30" s="8" t="n">
         <f aca="false">E29/E4</f>
-        <v>175.128205128205</v>
+        <v>189.025641025641</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">B29/B9</f>
-        <v>0.0436245954692557</v>
+        <v>0.0485906040268456</v>
       </c>
       <c r="C31" s="11" t="n">
         <f aca="false">C29/C9</f>
-        <v>0.0784240150093809</v>
+        <v>0.0832684824902724</v>
       </c>
       <c r="D31" s="11" t="n">
         <f aca="false">D29/D9</f>
-        <v>0.109717097170972</v>
+        <v>0.127602040816327</v>
       </c>
       <c r="E31" s="11" t="n">
         <f aca="false">E29/E9</f>
-        <v>0.124977127172919</v>
+        <v>0.13988614800759</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B32" s="12" t="str">
         <f aca="false">IF(B29&gt;=0,"yes","NO")</f>
@@ -2597,7 +2625,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B33" s="9" t="n">
         <f aca="false">B19</f>
@@ -2618,7 +2646,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -2627,7 +2655,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">B4*400</f>
@@ -2648,7 +2676,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B36" s="8" t="n">
         <f aca="false">B16*Inputs!$B$21+B25*Inputs!$B$31</f>
@@ -2660,16 +2688,16 @@
       </c>
       <c r="D36" s="8" t="n">
         <f aca="false">D16*Inputs!$B$21+D25*Inputs!$B$31</f>
-        <v>6195</v>
+        <v>6072</v>
       </c>
       <c r="E36" s="8" t="n">
         <f aca="false">E16*Inputs!$B$21+E25*Inputs!$B$31</f>
-        <v>8210</v>
+        <v>8087</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B37" s="9" t="n">
         <f aca="false">B35-B36</f>
@@ -2681,58 +2709,58 @@
       </c>
       <c r="D37" s="9" t="n">
         <f aca="false">D35-D36</f>
-        <v>5405</v>
+        <v>5528</v>
       </c>
       <c r="E37" s="9" t="n">
         <f aca="false">E35-E36</f>
-        <v>7390</v>
+        <v>7513</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">B9-B35</f>
-        <v>11050</v>
+        <v>10500</v>
       </c>
       <c r="C38" s="8" t="n">
         <f aca="false">C9-C35</f>
-        <v>19050</v>
+        <v>18100</v>
       </c>
       <c r="D38" s="8" t="n">
         <f aca="false">D9-D35</f>
-        <v>29050</v>
+        <v>27600</v>
       </c>
       <c r="E38" s="8" t="n">
         <f aca="false">E9-E35</f>
-        <v>39050</v>
+        <v>37100</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B39" s="8" t="n">
         <f aca="false">B18-B16*Inputs!$B$21+B20+B25*(1-Inputs!$B$31)+B23+B24</f>
-        <v>10704</v>
+        <v>10104</v>
       </c>
       <c r="C39" s="8" t="n">
         <f aca="false">C18-C16*Inputs!$B$21+C20+C25*(1-Inputs!$B$31)+C23+C24</f>
-        <v>18100</v>
+        <v>17100</v>
       </c>
       <c r="D39" s="8" t="n">
         <f aca="false">D18-D16*Inputs!$B$21+D20+D25*(1-Inputs!$B$31)+D23+D24</f>
-        <v>26895</v>
+        <v>25026</v>
       </c>
       <c r="E39" s="8" t="n">
         <f aca="false">E18-E16*Inputs!$B$21+E20+E25*(1-Inputs!$B$31)+E23+E24</f>
-        <v>35690</v>
+        <v>33321</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B40" s="8" t="n">
         <f aca="false">B22</f>
@@ -2753,7 +2781,7 @@
     </row>
     <row r="41" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -2786,108 +2814,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>174</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2897,10 +2925,10 @@
     </row>
     <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>10</v>
@@ -2908,10 +2936,10 @@
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Cozumel: fee re-cut to USD 1,350 / 1,200 on Hotel Plaza (pricing basis 30, contingency 3%), flyer prompt and comparison updated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/cozumel_group_budget.xlsx
+++ b/december-plan/pricing/cozumel_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="192">
   <si>
     <t xml:space="preserve">Cozumel group budget — inputs (blue cells are editable)</t>
   </si>
@@ -49,544 +49,550 @@
     <t xml:space="preserve">people</t>
   </si>
   <si>
-    <t xml:space="preserve">policy: conservative</t>
+    <t xml:space="preserve">policy (George, 28 Sep): 30, last year was 40</t>
   </si>
   <si>
     <t xml:space="preserve">Minimum headcount the contingency must cover</t>
   </si>
   <si>
+    <t xml:space="preserve">policy (George, 28 Sep): fee 1,350 / 1,200 is covered from 14 (13 loses the odd-room cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of participants who are Open Water students</t>
+  </si>
+  <si>
+    <t xml:space="preserve">share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingency inside the fee (refunded pro rata if unused)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">policy (George, 28 Sep): 3%, rounding to 50 adds the rest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note Scuba (QUOTED 23 Sep 2026, Doug Atkinson)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open Water course, 3 days, equipment included</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two extra boat days for new divers (Thu–Fri)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Certified 5-day two-tank package</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment rental per day, everyone rents (in the fee)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD/day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 24 Sep: full set BCD, regulator, mask, fins, wetsuit; bulk-rate ask saved for October</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dive computer rental per day (included on courses; extra on regular rentals)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 24 Sep; in the fee for every boat day under the everyone-rents rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rental days, certified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">programme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rental days, new divers (course includes equipment; the two extra boat days do not)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSUMED; ask Blue Note whether the USD 240 extra days include gear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marine park fee per boat day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED: 225 pesos in 2026 (Blue Note site shows USD 12 / 220 pesos); QUOTED 23 Sep: paid on site for boat days only, none on the two training-site days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boat days, certified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boat days, new divers (dive 3–4 day + Thu + Fri)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commission on certified packages, paid to George</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED: deducted from the invoice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One free certified package per N paid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">paid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note deposit at booking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED; balance 30 days out; refund to 7 days out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afternoon two-tank dive (optional add-on)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED price page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Private night charter, up to 10 divers (optional add-on, shared)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shore dive at Tikila Beach Bar incl. gear (optional add-on on the free mornings)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 24 Sep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nitrox fill per tank (course free with eLearning)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INFERRED; QUOTE NEEDED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel Plaza Cozumel (QUOTED via Blue Note's contracted rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Room per night, 2 people with breakfast, low-rate nights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED (Dec 14–15 rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Room per night, 2 people with breakfast, high-rate nights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED (Dec 16–19 rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low-rate nights (Sun 13, Mon 14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assumes the Dec 14–15 rate covers the nights of 13 and 14; CONFIRM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High-rate nights (Tue 15 – Fri 18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel deposit at booking (share of block)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTE NEEDED; assumption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel Plaza: one complimentary room per N paid rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 25 Sep via Blue Note (20 rooms blocked)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Included in the fee for everyone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PADI Open Water eLearning (club buys the codes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED store.padi.com about USD 230; Blue Note asked for its code price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dive-accident cover inside the fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 25 Sep: DAN no longer lets shops buy cover for divers; each person buys their own (own spending below); OW students covered by the shop during the course only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tax buffer per head</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 24 Sep: Blue Note prices include taxes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leader costs carried by the group (George shares a room like everyone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George's flight allowance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">policy; PHL–CZM band 568–800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George's half of a shared room, 6 nights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">formula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Odd-headcount room risk (one person alone at the group's cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">formula: half a room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George's dive cover carried by the group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">own cost like everyone (25 Sep)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George's gear and computer rental, 5 days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Own spending guidance, not in the fee (no flights)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunches, dinners and drinks per day (breakfast included)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INFERRED for an MBA crowd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days on the island</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tips for boat crew and hotel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INFERRED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airport transfers both ways</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED shared van 15 each way</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dive cover bought by each person via Blue Note's DAN link (membership 40 + Master 44)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED; required, proof collected at sign-up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PADI AOW eLearning (add-on for AOW takers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED (about)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trip fee per person, set at the pricing headcount (USD, 2 sharing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open Water student</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Certified diver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diving with Blue Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gear rental incl. computer, everyone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marine park fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tax buffer (zero: Blue Note prices include taxes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PADI eLearning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dive-accident cover (not in the fee: each person buys their own, see below)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel Plaza, 6 nights with breakfast, 2 sharing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leader's costs shared (George's flight, half-room, DAN, rental, odd-room risk)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRIP FEE (rounded up to the nearest 50, as posted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional add-ons at sign-up, charged at cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AOW: course free with eLearning; eLearning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nitrox: course free with eLearning; 10 fills</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afternoon two-tank dive, each, incl. park fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Night dive, private charter shared by 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shore dive on a free morning, incl. gear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GUIDANCE BUDGET WITHOUT FLIGHTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trip fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Own spending: DAN cover, meals, drinks, tips, airport transfers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guidance budget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guidance budget, certified taking AOW and nitrox</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The fee covers everything diving-related (course or package, gear and computer, park fees, eLearning) and the hotel; flights, the required DAN cover (bought by each person), meals, drinks, tips and transfers are the person's own. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group budget at four sizes (half students; George leads and does not pay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 people (minimum)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 people</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 people (pricing basis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40 people</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People including George</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paying participants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open Water students</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paying certified divers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rooms, everyone 2 sharing including George (odd person alone at the group's cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trip fees collected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note: Open Water courses and extra days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note: certified packages, paid divers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comps earned (1 per N paid certified)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George's package (free if at least one comp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spare comps credited against the invoice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note gross invoice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Less 10% commission on paid certified packages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note net payable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commission passed to George</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gear and computer rental for everyone including George</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tax buffer held (paid to Blue Note and the hotel if charged; otherwise refunded)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marine park fees (cash on the island, paid from the float)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PADI Open Water eLearning codes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dive cover for everyone including George (short-term plan via the shop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel Plaza block, all rooms, less one comp room per 14 paid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL COSTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surplus (contingency and over-recovery; refunded pro rata or held)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surplus per paying person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surplus as a share of revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Covered? (surplus must stay positive at the minimum headcount)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George's pot: commission (flight and room already carried above)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deposits and cash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Participant deposits at sign-up (USD 400 each)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note 25% deposit + hotel deposit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deposit cover (positive means deposits fund the outflow)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balances due from participants by Fri 6 Nov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note balance Fri 13 Nov + rental + hotel balance + eLearning + DAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash float to carry to the island (park fees)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes: revenue is the fixed fee from the Fee sheet, so the surplus grows with headcount (the leader share is over-recovered) and shrinks below the pricing basis; the contingency keeps it positive down to the minimum. Spare comps reduce the invoice for the group; the commission goes to George.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payment schedule and refund policy (mirrors Blue Note's terms)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">what</t>
+  </si>
+  <si>
+    <t xml:space="preserve">who</t>
+  </si>
+  <si>
+    <t xml:space="preserve">by Fri 2 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign-ups open on CampusGroups; deposit USD 400 per person holds a place</t>
+  </si>
+  <si>
+    <t xml:space="preserve">participants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sat 10 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign-up deadline for the first block; headcount to Blue Note and Hotel Plaza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George</t>
+  </si>
+  <si>
+    <t xml:space="preserve">by Thu 15 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note deposit 25% of the gross invoice; hotel deposit (terms to confirm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">club account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fri 6 Nov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Participant balances due (fee less deposit, plus any add-ons)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fri 13 Nov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note final payment (30 days out); hotel balance per its terms; buy eLearning codes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun 6 Dec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Note's 7-day refund cut-off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">everyone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun 13 Dec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrival; park fees paid from the club float; meals, drinks, tips and transfers are each person's own</t>
+  </si>
+  <si>
+    <t xml:space="preserve">after the trip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unused contingency and any surplus refunded pro rata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refund ladder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deposit refundable in full until Fri 6 Nov; 7 Nov to 6 Dec refundable only if the place is resold or Blue Note refunds it; from 7 Dec no refund, only Blue Note credit where given. Weather cancellations: Blue Note reschedules or refunds the missed dives.</t>
+  </si>
+  <si>
     <t xml:space="preserve">policy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Share of participants who are Open Water students</t>
-  </si>
-  <si>
-    <t xml:space="preserve">share</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brief</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contingency inside the fee (refunded pro rata if unused)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note Scuba (QUOTED 23 Sep 2026, Doug Atkinson)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open Water course, 3 days, equipment included</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Two extra boat days for new divers (Thu–Fri)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Certified 5-day two-tank package</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipment rental per day, everyone rents (in the fee)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USD/day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED 24 Sep: full set BCD, regulator, mask, fins, wetsuit; bulk-rate ask saved for October</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dive computer rental per day (included on courses; extra on regular rentals)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED 24 Sep; in the fee for every boat day under the everyone-rents rule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rental days, certified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">programme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rental days, new divers (course includes equipment; the two extra boat days do not)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASSUMED; ask Blue Note whether the USD 240 extra days include gear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marine park fee per boat day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED: 225 pesos in 2026 (Blue Note site shows USD 12 / 220 pesos); QUOTED 23 Sep: paid on site for boat days only, none on the two training-site days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boat days, certified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boat days, new divers (dive 3–4 day + Thu + Fri)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commission on certified packages, paid to George</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED: deducted from the invoice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One free certified package per N paid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">paid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note deposit at booking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED; balance 30 days out; refund to 7 days out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Afternoon two-tank dive (optional add-on)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED price page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Private night charter, up to 10 divers (optional add-on, shared)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shore dive at Tikila Beach Bar incl. gear (optional add-on on the free mornings)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED 24 Sep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nitrox fill per tank (course free with eLearning)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INFERRED; QUOTE NEEDED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel Plaza Cozumel (QUOTED via Blue Note's contracted rate)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Room per night, 2 people with breakfast, low-rate nights</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED (Dec 14–15 rate)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Room per night, 2 people with breakfast, high-rate nights</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED (Dec 16–19 rate)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low-rate nights (Sun 13, Mon 14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nights</t>
-  </si>
-  <si>
-    <t xml:space="preserve">assumes the Dec 14–15 rate covers the nights of 13 and 14; CONFIRM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High-rate nights (Tue 15 – Fri 18)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel deposit at booking (share of block)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTE NEEDED; assumption</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel Plaza: one complimentary room per N paid rooms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rooms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED 25 Sep via Blue Note (20 rooms blocked)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Included in the fee for everyone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PADI Open Water eLearning (club buys the codes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED store.padi.com about USD 230; Blue Note asked for its code price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dive-accident cover inside the fee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED 25 Sep: DAN no longer lets shops buy cover for divers; each person buys their own (own spending below); OW students covered by the shop during the course only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tax buffer per head</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED 24 Sep: Blue Note prices include taxes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leader costs carried by the group (George shares a room like everyone)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George's flight allowance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">policy; PHL–CZM band 568–800</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George's half of a shared room, 6 nights</t>
-  </si>
-  <si>
-    <t xml:space="preserve">formula</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Odd-headcount room risk (one person alone at the group's cost)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">formula: half a room</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George's dive cover carried by the group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">own cost like everyone (25 Sep)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George's gear and computer rental, 5 days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Own spending guidance, not in the fee (no flights)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lunches, dinners and drinks per day (breakfast included)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INFERRED for an MBA crowd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Days on the island</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tips for boat crew and hotel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INFERRED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Airport transfers both ways</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED shared van 15 each way</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dive cover bought by each person via Blue Note's DAN link (membership 40 + Master 44)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED; required, proof collected at sign-up</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PADI AOW eLearning (add-on for AOW takers)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED (about)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trip fee per person, set at the pricing headcount (USD, 2 sharing)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open Water student</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Certified diver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diving with Blue Note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gear rental incl. computer, everyone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marine park fees</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tax buffer (zero: Blue Note prices include taxes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PADI eLearning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dive-accident cover (not in the fee: each person buys their own, see below)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel Plaza, 6 nights with breakfast, 2 sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leader's costs shared (George's flight, half-room, DAN, rental, odd-room risk)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contingency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRIP FEE (rounded up to the nearest 50, as posted)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optional add-ons at sign-up, charged at cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AOW: course free with eLearning; eLearning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n/a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nitrox: course free with eLearning; 10 fills</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Afternoon two-tank dive, each, incl. park fee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Night dive, private charter shared by 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shore dive on a free morning, incl. gear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GUIDANCE BUDGET WITHOUT FLIGHTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trip fee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Own spending: DAN cover, meals, drinks, tips, airport transfers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guidance budget</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guidance budget, certified taking AOW and nitrox</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The fee covers everything diving-related (course or package, gear and computer, park fees, eLearning) and the hotel; flights, the required DAN cover (bought by each person), meals, drinks, tips and transfers are the person's own. It is set at the pricing headcount; a bigger group makes a surplus that is refunded pro rata or held as buffer, a smaller group down to the minimum is covered by the contingency (see Group sheet). George's place: diving covered by Blue Note's comp, flight and room carried by the group, commission to George, all disclosed on the sign-up page.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Group budget at four sizes (half students; George leads and does not pay)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 people (minimum)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 people (pricing basis)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 people</t>
-  </si>
-  <si>
-    <t xml:space="preserve">40 people</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People including George</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paying participants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open Water students</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paying certified divers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rooms, everyone 2 sharing including George (odd person alone at the group's cost)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revenue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trip fees collected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note: Open Water courses and extra days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note: certified packages, paid divers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comps earned (1 per N paid certified)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George's package (free if at least one comp)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spare comps credited against the invoice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note gross invoice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Less 10% commission on paid certified packages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note net payable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commission passed to George</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gear and computer rental for everyone including George</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tax buffer held (paid to Blue Note and the hotel if charged; otherwise refunded)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marine park fees (cash on the island, paid from the float)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PADI Open Water eLearning codes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dive cover for everyone including George (short-term plan via the shop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel Plaza block, all rooms, less one comp room per 14 paid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL COSTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Result</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surplus (contingency and over-recovery; refunded pro rata or held)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surplus per paying person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surplus as a share of revenue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covered? (surplus must stay positive at the minimum headcount)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George's pot: commission (flight and room already carried above)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deposits and cash</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Participant deposits at sign-up (USD 400 each)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note 25% deposit + hotel deposit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deposit cover (positive means deposits fund the outflow)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Balances due from participants by Fri 6 Nov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note balance Fri 13 Nov + rental + hotel balance + eLearning + DAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cash float to carry to the island (park fees)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes: revenue is the fixed fee from the Fee sheet, so the surplus grows with headcount (the leader share is over-recovered) and shrinks below the pricing basis; the contingency keeps it positive down to the minimum. Spare comps reduce the invoice for the group; the commission goes to George.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Payment schedule and refund policy (mirrors Blue Note's terms)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">what</t>
-  </si>
-  <si>
-    <t xml:space="preserve">who</t>
-  </si>
-  <si>
-    <t xml:space="preserve">by Fri 2 Oct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sign-ups open on CampusGroups; deposit USD 400 per person holds a place</t>
-  </si>
-  <si>
-    <t xml:space="preserve">participants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sat 10 Oct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sign-up deadline for the first block; headcount to Blue Note and Hotel Plaza</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George</t>
-  </si>
-  <si>
-    <t xml:space="preserve">by Thu 15 Oct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note deposit 25% of the gross invoice; hotel deposit (terms to confirm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">club account</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fri 6 Nov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Participant balances due (fee less deposit, plus any add-ons)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fri 13 Nov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note final payment (30 days out); hotel balance per its terms; buy eLearning codes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sun 6 Dec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Note's 7-day refund cut-off</t>
-  </si>
-  <si>
-    <t xml:space="preserve">everyone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sun 13 Dec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arrival; park fees paid from the club float; meals, drinks, tips and transfers are each person's own</t>
-  </si>
-  <si>
-    <t xml:space="preserve">after the trip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unused contingency and any surplus refunded pro rata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Refund ladder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deposit refundable in full until Fri 6 Nov; 7 Nov to 6 Dec refundable only if the place is resold or Blue Note refunds it; from 7 Dec no refund, only Blue Note credit where given. Weather cancellations: Blue Note reschedules or refunds the missed dives.</t>
   </si>
   <si>
     <t xml:space="preserve">Money handling</t>
@@ -1047,7 +1053,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
@@ -1056,12 +1062,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
@@ -1089,18 +1095,18 @@
         <v>14</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.06</v>
+        <v>0.03</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1108,147 +1114,147 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>400</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>240</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>600</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>30</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>10</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>5</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16" s="7" t="n">
         <v>13</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>5</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B18" s="5" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19" s="6" t="n">
         <v>0.1</v>
@@ -1257,26 +1263,26 @@
         <v>12</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B20" s="5" t="n">
         <v>5</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B21" s="6" t="n">
         <v>0.25</v>
@@ -1285,68 +1291,68 @@
         <v>12</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B22" s="7" t="n">
         <v>130</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>800</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B24" s="7" t="n">
         <v>60</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B25" s="7" t="n">
         <v>12</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1354,61 +1360,61 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B27" s="7" t="n">
         <v>70</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B28" s="7" t="n">
         <v>88</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B29" s="5" t="n">
         <v>2</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B30" s="5" t="n">
         <v>4</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B31" s="6" t="n">
         <v>0.25</v>
@@ -1417,26 +1423,26 @@
         <v>12</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B32" s="5" t="n">
         <v>14</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1444,49 +1450,49 @@
     </row>
     <row r="34" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B34" s="7" t="n">
         <v>230</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B36" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -1494,80 +1500,80 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B38" s="7" t="n">
         <v>700</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B39" s="7" t="n">
         <f aca="false">(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)/2</f>
         <v>246</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B40" s="7" t="n">
         <f aca="false">Inputs!$B$39</f>
         <v>246</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B42" s="7" t="n">
         <f aca="false">(Inputs!$B$12+Inputs!$B$13)*5</f>
         <v>200</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -1575,84 +1581,84 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B44" s="7" t="n">
         <v>45</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B45" s="5" t="n">
         <v>6</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B46" s="7" t="n">
         <v>50</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B47" s="7" t="n">
         <v>30</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B48" s="7" t="n">
         <v>84</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B49" s="7" t="n">
         <v>220</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1680,7 +1686,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1688,15 +1694,15 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">Inputs!$B$9+Inputs!$B$10</f>
@@ -1709,7 +1715,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15</f>
@@ -1722,7 +1728,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">Inputs!$B$16*Inputs!$B$18</f>
@@ -1735,7 +1741,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">Inputs!$B$36</f>
@@ -1748,19 +1754,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">Inputs!$B$34</f>
         <v>230</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">Inputs!$B$35</f>
@@ -1773,7 +1779,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">((Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)/2)</f>
@@ -1786,54 +1792,54 @@
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">(Inputs!$B$38+Inputs!$B$39+Inputs!$B$40+Inputs!$B$41+Inputs!$B$42)/(Inputs!$B$4-1)</f>
-        <v>73.2631578947368</v>
+        <v>48</v>
       </c>
       <c r="C10" s="8" t="n">
         <f aca="false">(Inputs!$B$38+Inputs!$B$39+Inputs!$B$40+Inputs!$B$41+Inputs!$B$42)/(Inputs!$B$4-1)</f>
-        <v>73.2631578947368</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">SUM(B3:B10)</f>
-        <v>1308.26315789474</v>
+        <v>1283</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">SUM(C3:C10)</f>
-        <v>1184.26315789474</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">ROUND(B11*Inputs!$B$7,0)</f>
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">ROUND(C11*Inputs!$B$7,0)</f>
-        <v>71</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">CEILING(B11+B12,50)</f>
-        <v>1400</v>
+        <v>1350</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">CEILING(C11+C12,50)</f>
-        <v>1300</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1843,17 +1849,17 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C16" s="8" t="n">
         <f aca="false">Inputs!$B$49</f>
@@ -1862,10 +1868,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>109</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>108</v>
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">Inputs!$B$25*10</f>
@@ -1874,7 +1880,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">Inputs!$B$22+Inputs!$B$16</f>
@@ -1887,7 +1893,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">Inputs!$B$23/10</f>
@@ -1900,7 +1906,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">Inputs!$B$24</f>
@@ -1918,27 +1924,27 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B23" s="9" t="n">
         <f aca="false">B13</f>
-        <v>1400</v>
+        <v>1350</v>
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">C13</f>
-        <v>1300</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">Inputs!$B$48+Inputs!$B$44*Inputs!$B$45+Inputs!$B$46+Inputs!$B$47</f>
@@ -1951,27 +1957,27 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B25" s="9" t="n">
         <f aca="false">B23+B24</f>
-        <v>1834</v>
+        <v>1784</v>
       </c>
       <c r="C25" s="9" t="n">
         <f aca="false">C23+C24</f>
-        <v>1734</v>
+        <v>1634</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C26" s="9" t="n">
         <f aca="false">C25+C16+C17</f>
-        <v>2074</v>
+        <v>1974</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1981,7 +1987,7 @@
     </row>
     <row r="28" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -2011,7 +2017,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2021,24 +2027,24 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B3" s="10" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C3" s="10" t="n">
         <v>20</v>
@@ -2052,11 +2058,11 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" s="10" t="n">
         <f aca="false">C3-1</f>
@@ -2073,11 +2079,11 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$6,0)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" s="10" t="n">
         <f aca="false">ROUND(C4*Inputs!$B$6,0)</f>
@@ -2094,11 +2100,11 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">B4-B5</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">C4-C5</f>
@@ -2115,11 +2121,11 @@
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">ROUNDUP(B3/2,0)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">ROUNDUP(C3/2,0)</f>
@@ -2136,7 +2142,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2145,28 +2151,28 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">B5*Fee!$B$13+B6*Fee!$C$13</f>
-        <v>14900</v>
+        <v>16650</v>
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">C5*Fee!$B$13+C6*Fee!$C$13</f>
-        <v>25700</v>
+        <v>24300</v>
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">D5*Fee!$B$13+D6*Fee!$C$13</f>
-        <v>39200</v>
+        <v>37050</v>
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">E5*Fee!$B$13+E6*Fee!$C$13</f>
-        <v>52700</v>
+        <v>49800</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2175,11 +2181,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$9+Inputs!$B$10)</f>
-        <v>3840</v>
+        <v>4480</v>
       </c>
       <c r="C11" s="8" t="n">
         <f aca="false">C5*(Inputs!$B$9+Inputs!$B$10)</f>
@@ -2196,11 +2202,11 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B6*Inputs!$B$11</f>
-        <v>3000</v>
+        <v>3600</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">C6*Inputs!$B$11</f>
@@ -2217,7 +2223,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">INT(B6/Inputs!$B$20)</f>
@@ -2238,7 +2244,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">IF(B13&gt;=1,0,Inputs!$B$11)</f>
@@ -2259,7 +2265,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">-MAX(B13-1,0)*Inputs!$B$11</f>
@@ -2280,11 +2286,11 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B11+B12+B14+B15</f>
-        <v>6840</v>
+        <v>8080</v>
       </c>
       <c r="C16" s="8" t="n">
         <f aca="false">C11+C12+C14+C15</f>
@@ -2301,11 +2307,11 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">-B12*Inputs!$B$19</f>
-        <v>-300</v>
+        <v>-360</v>
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">-C12*Inputs!$B$19</f>
@@ -2322,11 +2328,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B16+B17</f>
-        <v>6540</v>
+        <v>7720</v>
       </c>
       <c r="C18" s="9" t="n">
         <f aca="false">C16+C17</f>
@@ -2343,11 +2349,11 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-B17</f>
-        <v>300</v>
+        <v>360</v>
       </c>
       <c r="C19" s="8" t="n">
         <f aca="false">-C17</f>
@@ -2364,11 +2370,11 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15+(B6+1)*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$14</f>
-        <v>1680</v>
+        <v>1960</v>
       </c>
       <c r="C20" s="8" t="n">
         <f aca="false">C5*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$15+(C6+1)*(Inputs!$B$12+Inputs!$B$13)*Inputs!$B$14</f>
@@ -2385,7 +2391,7 @@
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B21" s="8" t="n">
         <f aca="false">B3*Inputs!$B$36</f>
@@ -2406,11 +2412,11 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B5*Inputs!$B$16*Inputs!$B$18+(B6+1)*Inputs!$B$16*Inputs!$B$17</f>
-        <v>624</v>
+        <v>728</v>
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">C5*Inputs!$B$16*Inputs!$B$18+(C6+1)*Inputs!$B$16*Inputs!$B$17</f>
@@ -2427,11 +2433,11 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">B5*Inputs!$B$34</f>
-        <v>1380</v>
+        <v>1610</v>
       </c>
       <c r="C23" s="8" t="n">
         <f aca="false">C5*Inputs!$B$34</f>
@@ -2448,7 +2454,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">B3*Inputs!$B$35</f>
@@ -2469,11 +2475,11 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">(B7-INT(B7/(Inputs!$B$32+1)))*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
-        <v>2952</v>
+        <v>3444</v>
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">(C7-INT(C7/(Inputs!$B$32+1)))*(Inputs!$B$27*Inputs!$B$29+Inputs!$B$28*Inputs!$B$30)</f>
@@ -2490,7 +2496,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">Inputs!$B$38</f>
@@ -2511,11 +2517,11 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B27" s="9" t="n">
         <f aca="false">B18+B19+B20+B21+B22+B23+B24+B25+B26</f>
-        <v>14176</v>
+        <v>16522</v>
       </c>
       <c r="C27" s="9" t="n">
         <f aca="false">C18+C19+C20+C21+C22+C23+C24+C25+C26</f>
@@ -2532,7 +2538,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -2541,70 +2547,70 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">B9-B27</f>
-        <v>724</v>
+        <v>128</v>
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">C9-C27</f>
-        <v>2140</v>
+        <v>740</v>
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">D9-D27</f>
-        <v>5002</v>
+        <v>2852</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">E9-E27</f>
-        <v>7372</v>
+        <v>4472</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B30" s="8" t="n">
         <f aca="false">B29/B4</f>
-        <v>65.8181818181818</v>
+        <v>9.84615384615385</v>
       </c>
       <c r="C30" s="8" t="n">
         <f aca="false">C29/C4</f>
-        <v>112.631578947368</v>
+        <v>38.9473684210526</v>
       </c>
       <c r="D30" s="8" t="n">
         <f aca="false">D29/D4</f>
-        <v>172.48275862069</v>
+        <v>98.3448275862069</v>
       </c>
       <c r="E30" s="8" t="n">
         <f aca="false">E29/E4</f>
-        <v>189.025641025641</v>
+        <v>114.666666666667</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">B29/B9</f>
-        <v>0.0485906040268456</v>
+        <v>0.00768768768768769</v>
       </c>
       <c r="C31" s="11" t="n">
         <f aca="false">C29/C9</f>
-        <v>0.0832684824902724</v>
+        <v>0.0304526748971193</v>
       </c>
       <c r="D31" s="11" t="n">
         <f aca="false">D29/D9</f>
-        <v>0.127602040816327</v>
+        <v>0.0769770580296896</v>
       </c>
       <c r="E31" s="11" t="n">
         <f aca="false">E29/E9</f>
-        <v>0.13988614800759</v>
+        <v>0.0897991967871486</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B32" s="12" t="str">
         <f aca="false">IF(B29&gt;=0,"yes","NO")</f>
@@ -2625,11 +2631,11 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B33" s="9" t="n">
         <f aca="false">B19</f>
-        <v>300</v>
+        <v>360</v>
       </c>
       <c r="C33" s="9" t="n">
         <f aca="false">C19</f>
@@ -2646,7 +2652,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -2655,11 +2661,11 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">B4*400</f>
-        <v>4400</v>
+        <v>5200</v>
       </c>
       <c r="C35" s="8" t="n">
         <f aca="false">C4*400</f>
@@ -2676,11 +2682,11 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B36" s="8" t="n">
         <f aca="false">B16*Inputs!$B$21+B25*Inputs!$B$31</f>
-        <v>2448</v>
+        <v>2881</v>
       </c>
       <c r="C36" s="8" t="n">
         <f aca="false">C16*Inputs!$B$21+C25*Inputs!$B$31</f>
@@ -2697,11 +2703,11 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B37" s="9" t="n">
         <f aca="false">B35-B36</f>
-        <v>1952</v>
+        <v>2319</v>
       </c>
       <c r="C37" s="9" t="n">
         <f aca="false">C35-C36</f>
@@ -2718,32 +2724,32 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">B9-B35</f>
-        <v>10500</v>
+        <v>11450</v>
       </c>
       <c r="C38" s="8" t="n">
         <f aca="false">C9-C35</f>
-        <v>18100</v>
+        <v>16700</v>
       </c>
       <c r="D38" s="8" t="n">
         <f aca="false">D9-D35</f>
-        <v>27600</v>
+        <v>25450</v>
       </c>
       <c r="E38" s="8" t="n">
         <f aca="false">E9-E35</f>
-        <v>37100</v>
+        <v>34200</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B39" s="8" t="n">
         <f aca="false">B18-B16*Inputs!$B$21+B20+B25*(1-Inputs!$B$31)+B23+B24</f>
-        <v>10104</v>
+        <v>11853</v>
       </c>
       <c r="C39" s="8" t="n">
         <f aca="false">C18-C16*Inputs!$B$21+C20+C25*(1-Inputs!$B$31)+C23+C24</f>
@@ -2760,11 +2766,11 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B40" s="8" t="n">
         <f aca="false">B22</f>
-        <v>624</v>
+        <v>728</v>
       </c>
       <c r="C40" s="8" t="n">
         <f aca="false">C22</f>
@@ -2781,7 +2787,7 @@
     </row>
     <row r="41" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -2814,108 +2820,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2925,24 +2931,24 @@
     </row>
     <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>10</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>